<commit_message>
Atualização da base de dados ate 09/03/2026 e adicionei o grafico diario por vendedor
</commit_message>
<xml_diff>
--- a/BASE_KEMPARTS.xlsx
+++ b/BASE_KEMPARTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dash_kp_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{902177DB-F828-4D2A-AAFF-1F8EEF583922}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CCDF60A6-0241-4C84-A5C9-0B6398B4F075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{034ED65E-4C5C-4047-81C4-E67EF536DEAB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{6FEA2588-5565-4B12-8C5E-E6FBB7E9CDF0}"/>
   </bookViews>
   <sheets>
     <sheet name="FSP" sheetId="3" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7147" uniqueCount="1258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7397" uniqueCount="1288">
   <si>
     <t/>
   </si>
@@ -3122,6 +3122,102 @@
     <t>0000406221</t>
   </si>
   <si>
+    <t>000015536</t>
+  </si>
+  <si>
+    <t>173798</t>
+  </si>
+  <si>
+    <t>000015537</t>
+  </si>
+  <si>
+    <t>173800</t>
+  </si>
+  <si>
+    <t>000015538</t>
+  </si>
+  <si>
+    <t>173804</t>
+  </si>
+  <si>
+    <t>000015539</t>
+  </si>
+  <si>
+    <t>C00305</t>
+  </si>
+  <si>
+    <t>RAIOLUX INDUSTRIA E COM DE TINTAS LTDA</t>
+  </si>
+  <si>
+    <t>TRAN.24.004.12.24121017</t>
+  </si>
+  <si>
+    <t>24121017</t>
+  </si>
+  <si>
+    <t>173806</t>
+  </si>
+  <si>
+    <t>000015540</t>
+  </si>
+  <si>
+    <t>C00616</t>
+  </si>
+  <si>
+    <t>AGROPLASTIC COMERCIAL DE PLASTICOS LTDA</t>
+  </si>
+  <si>
+    <t>T00282</t>
+  </si>
+  <si>
+    <t>MEG DE SOUZA COUTINHO TRANSPORTES - EPP</t>
+  </si>
+  <si>
+    <t>173820</t>
+  </si>
+  <si>
+    <t>000015541</t>
+  </si>
+  <si>
+    <t>173824</t>
+  </si>
+  <si>
+    <t>000015542</t>
+  </si>
+  <si>
+    <t>173826</t>
+  </si>
+  <si>
+    <t>000015543</t>
+  </si>
+  <si>
+    <t>173828</t>
+  </si>
+  <si>
+    <t>000015545</t>
+  </si>
+  <si>
+    <t>C00102</t>
+  </si>
+  <si>
+    <t>POLI-COR INDUSTRIA DE TINTAS E VERNIZES</t>
+  </si>
+  <si>
+    <t>HHQ 100 (YL 90)</t>
+  </si>
+  <si>
+    <t>TRAN.25.357.04.250416</t>
+  </si>
+  <si>
+    <t>250416</t>
+  </si>
+  <si>
+    <t>TRAN.25.357.04.</t>
+  </si>
+  <si>
+    <t>153266</t>
+  </si>
+  <si>
     <t>GASTOS GERAIS</t>
   </si>
   <si>
@@ -3227,9 +3323,6 @@
     <t>2025.357.07.251014</t>
   </si>
   <si>
-    <t>HHQ 100 (YL 90)</t>
-  </si>
-  <si>
     <t>000002500</t>
   </si>
   <si>
@@ -3717,9 +3810,6 @@
   </si>
   <si>
     <t>003209</t>
-  </si>
-  <si>
-    <t>24121017</t>
   </si>
   <si>
     <t>2024.004.13.24121017</t>
@@ -4741,8 +4831,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BC32493-C966-4678-BA2F-91D43E76D569}">
-  <dimension ref="A1:AJ219"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{318A57C2-A3D9-48EA-BD6D-8BF7B0CE2ED1}">
+  <dimension ref="A1:AJ229"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
@@ -28872,13 +28962,1113 @@
         <v>13.0503</v>
       </c>
     </row>
+    <row r="220" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A220" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="B220" s="2" t="s">
+        <v>1033</v>
+      </c>
+      <c r="C220" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D220" s="4">
+        <v>46090</v>
+      </c>
+      <c r="E220" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F220" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G220" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="H220" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="I220" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="J220" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="K220" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="L220" s="2" t="s">
+        <v>927</v>
+      </c>
+      <c r="M220" s="2" t="s">
+        <v>928</v>
+      </c>
+      <c r="N220" s="2" t="s">
+        <v>929</v>
+      </c>
+      <c r="O220" s="5">
+        <v>740</v>
+      </c>
+      <c r="P220" s="5">
+        <v>37.32</v>
+      </c>
+      <c r="Q220" s="6">
+        <v>27616.799999999999</v>
+      </c>
+      <c r="R220" s="6">
+        <v>897.55</v>
+      </c>
+      <c r="S220" s="6">
+        <v>28514.35</v>
+      </c>
+      <c r="T220" s="6">
+        <v>27616.799999999999</v>
+      </c>
+      <c r="U220" s="6">
+        <v>4971.0200000000004</v>
+      </c>
+      <c r="V220" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="W220" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="X220" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y220" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="Z220" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA220" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB220" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="AC220" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD220" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE220" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="AF220" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="AG220" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH220" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI220" s="6">
+        <v>18</v>
+      </c>
+      <c r="AJ220" s="5">
+        <v>9825.6164000000008</v>
+      </c>
+    </row>
+    <row r="221" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A221" s="3" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B221" s="3" t="s">
+        <v>1035</v>
+      </c>
+      <c r="C221" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D221" s="7">
+        <v>46090</v>
+      </c>
+      <c r="E221" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F221" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G221" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="H221" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="I221" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="J221" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K221" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="L221" s="3" t="s">
+        <v>893</v>
+      </c>
+      <c r="M221" s="3" t="s">
+        <v>894</v>
+      </c>
+      <c r="N221" s="3" t="s">
+        <v>895</v>
+      </c>
+      <c r="O221" s="8">
+        <v>2220</v>
+      </c>
+      <c r="P221" s="8">
+        <v>24.6</v>
+      </c>
+      <c r="Q221" s="9">
+        <v>54612</v>
+      </c>
+      <c r="R221" s="9">
+        <v>1774.89</v>
+      </c>
+      <c r="S221" s="9">
+        <v>56386.89</v>
+      </c>
+      <c r="T221" s="9">
+        <v>54612</v>
+      </c>
+      <c r="U221" s="9">
+        <v>2184.48</v>
+      </c>
+      <c r="V221" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="W221" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="X221" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y221" s="3" t="s">
+        <v>1036</v>
+      </c>
+      <c r="Z221" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA221" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB221" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="AC221" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="AD221" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE221" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="AF221" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="AG221" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH221" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI221" s="9">
+        <v>4</v>
+      </c>
+      <c r="AJ221" s="8">
+        <v>31058.3328</v>
+      </c>
+    </row>
+    <row r="222" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A222" s="2" t="s">
+        <v>1037</v>
+      </c>
+      <c r="B222" s="2" t="s">
+        <v>1037</v>
+      </c>
+      <c r="C222" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D222" s="4">
+        <v>46090</v>
+      </c>
+      <c r="E222" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F222" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G222" s="2" t="s">
+        <v>655</v>
+      </c>
+      <c r="H222" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="I222" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="J222" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="K222" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="L222" s="2" t="s">
+        <v>657</v>
+      </c>
+      <c r="M222" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="N222" s="2" t="s">
+        <v>659</v>
+      </c>
+      <c r="O222" s="5">
+        <v>2000</v>
+      </c>
+      <c r="P222" s="5">
+        <v>11.98</v>
+      </c>
+      <c r="Q222" s="6">
+        <v>23960</v>
+      </c>
+      <c r="R222" s="6">
+        <v>778.7</v>
+      </c>
+      <c r="S222" s="6">
+        <v>24738.7</v>
+      </c>
+      <c r="T222" s="6">
+        <v>23960</v>
+      </c>
+      <c r="U222" s="6">
+        <v>4312.8</v>
+      </c>
+      <c r="V222" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="W222" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="X222" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y222" s="2" t="s">
+        <v>1038</v>
+      </c>
+      <c r="Z222" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA222" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB222" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="AC222" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD222" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="AE222" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="AF222" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AG222" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH222" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI222" s="6">
+        <v>18</v>
+      </c>
+      <c r="AJ222" s="5">
+        <v>17704.900000000001</v>
+      </c>
+    </row>
+    <row r="223" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A223" s="3" t="s">
+        <v>1039</v>
+      </c>
+      <c r="B223" s="3" t="s">
+        <v>1039</v>
+      </c>
+      <c r="C223" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D223" s="7">
+        <v>46090</v>
+      </c>
+      <c r="E223" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F223" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G223" s="3" t="s">
+        <v>1040</v>
+      </c>
+      <c r="H223" s="3" t="s">
+        <v>1041</v>
+      </c>
+      <c r="I223" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="J223" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="K223" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="L223" s="3" t="s">
+        <v>1042</v>
+      </c>
+      <c r="M223" s="3" t="s">
+        <v>1043</v>
+      </c>
+      <c r="N223" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="O223" s="8">
+        <v>1000</v>
+      </c>
+      <c r="P223" s="8">
+        <v>17.46</v>
+      </c>
+      <c r="Q223" s="9">
+        <v>17460</v>
+      </c>
+      <c r="R223" s="9">
+        <v>567.45000000000005</v>
+      </c>
+      <c r="S223" s="9">
+        <v>18027.45</v>
+      </c>
+      <c r="T223" s="9">
+        <v>17460</v>
+      </c>
+      <c r="U223" s="9">
+        <v>3142.8</v>
+      </c>
+      <c r="V223" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="W223" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="X223" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y223" s="3" t="s">
+        <v>1044</v>
+      </c>
+      <c r="Z223" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA223" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB223" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="AC223" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD223" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="AE223" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="AF223" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="AG223" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH223" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI223" s="9">
+        <v>18</v>
+      </c>
+      <c r="AJ223" s="8">
+        <v>9897.6</v>
+      </c>
+    </row>
+    <row r="224" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A224" s="2" t="s">
+        <v>1045</v>
+      </c>
+      <c r="B224" s="2" t="s">
+        <v>1045</v>
+      </c>
+      <c r="C224" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D224" s="4">
+        <v>46090</v>
+      </c>
+      <c r="E224" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F224" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G224" s="2" t="s">
+        <v>1046</v>
+      </c>
+      <c r="H224" s="2" t="s">
+        <v>1047</v>
+      </c>
+      <c r="I224" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="J224" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="K224" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="L224" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="M224" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="N224" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="O224" s="5">
+        <v>185</v>
+      </c>
+      <c r="P224" s="5">
+        <v>24.78</v>
+      </c>
+      <c r="Q224" s="6">
+        <v>4584.3</v>
+      </c>
+      <c r="R224" s="6">
+        <v>148.99</v>
+      </c>
+      <c r="S224" s="6">
+        <v>4733.29</v>
+      </c>
+      <c r="T224" s="6">
+        <v>4584.3</v>
+      </c>
+      <c r="U224" s="6">
+        <v>183.37</v>
+      </c>
+      <c r="V224" s="2" t="s">
+        <v>1048</v>
+      </c>
+      <c r="W224" s="2" t="s">
+        <v>1049</v>
+      </c>
+      <c r="X224" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y224" s="2" t="s">
+        <v>1050</v>
+      </c>
+      <c r="Z224" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA224" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB224" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="AC224" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="AD224" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE224" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="AF224" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="AG224" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH224" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI224" s="6">
+        <v>4</v>
+      </c>
+      <c r="AJ224" s="5">
+        <v>2456.4041000000002</v>
+      </c>
+    </row>
+    <row r="225" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A225" s="3" t="s">
+        <v>1051</v>
+      </c>
+      <c r="B225" s="3" t="s">
+        <v>1051</v>
+      </c>
+      <c r="C225" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D225" s="7">
+        <v>46090</v>
+      </c>
+      <c r="E225" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F225" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G225" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="H225" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="I225" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="J225" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="K225" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="L225" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="M225" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="N225" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="O225" s="8">
+        <v>1870</v>
+      </c>
+      <c r="P225" s="8">
+        <v>24.59273</v>
+      </c>
+      <c r="Q225" s="9">
+        <v>45988.41</v>
+      </c>
+      <c r="R225" s="9">
+        <v>1494.62</v>
+      </c>
+      <c r="S225" s="9">
+        <v>47483.03</v>
+      </c>
+      <c r="T225" s="9">
+        <v>45988.41</v>
+      </c>
+      <c r="U225" s="9">
+        <v>8277.91</v>
+      </c>
+      <c r="V225" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="W225" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="X225" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y225" s="3" t="s">
+        <v>1052</v>
+      </c>
+      <c r="Z225" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA225" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB225" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="AC225" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD225" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE225" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="AF225" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="AG225" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH225" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI225" s="9">
+        <v>18</v>
+      </c>
+      <c r="AJ225" s="8">
+        <v>21765.603200000001</v>
+      </c>
+    </row>
+    <row r="226" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A226" s="2" t="s">
+        <v>1053</v>
+      </c>
+      <c r="B226" s="2" t="s">
+        <v>1053</v>
+      </c>
+      <c r="C226" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D226" s="4">
+        <v>46090</v>
+      </c>
+      <c r="E226" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F226" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G226" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="H226" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="I226" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="J226" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="K226" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="L226" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="M226" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="N226" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="O226" s="5">
+        <v>370</v>
+      </c>
+      <c r="P226" s="5">
+        <v>21.5</v>
+      </c>
+      <c r="Q226" s="6">
+        <v>7955</v>
+      </c>
+      <c r="R226" s="6">
+        <v>258.54000000000002</v>
+      </c>
+      <c r="S226" s="6">
+        <v>8213.5400000000009</v>
+      </c>
+      <c r="T226" s="6">
+        <v>7955</v>
+      </c>
+      <c r="U226" s="6">
+        <v>318.2</v>
+      </c>
+      <c r="V226" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="W226" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="X226" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y226" s="2" t="s">
+        <v>1054</v>
+      </c>
+      <c r="Z226" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA226" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB226" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="AC226" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="AD226" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE226" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="AF226" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="AG226" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH226" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI226" s="6">
+        <v>4</v>
+      </c>
+      <c r="AJ226" s="5">
+        <v>5176.3887999999997</v>
+      </c>
+    </row>
+    <row r="227" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A227" s="3" t="s">
+        <v>1055</v>
+      </c>
+      <c r="B227" s="3" t="s">
+        <v>1055</v>
+      </c>
+      <c r="C227" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D227" s="7">
+        <v>46090</v>
+      </c>
+      <c r="E227" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F227" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G227" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="H227" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="I227" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="J227" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="K227" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="L227" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="M227" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="N227" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="O227" s="8">
+        <v>170</v>
+      </c>
+      <c r="P227" s="8">
+        <v>26.89</v>
+      </c>
+      <c r="Q227" s="9">
+        <v>4571.3</v>
+      </c>
+      <c r="R227" s="9">
+        <v>148.57</v>
+      </c>
+      <c r="S227" s="9">
+        <v>4719.87</v>
+      </c>
+      <c r="T227" s="9">
+        <v>4571.3</v>
+      </c>
+      <c r="U227" s="9">
+        <v>822.83</v>
+      </c>
+      <c r="V227" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="W227" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="X227" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y227" s="3" t="s">
+        <v>1056</v>
+      </c>
+      <c r="Z227" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA227" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB227" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="AC227" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD227" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE227" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="AF227" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="AG227" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH227" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI227" s="9">
+        <v>18</v>
+      </c>
+      <c r="AJ227" s="8">
+        <v>1978.6912</v>
+      </c>
+    </row>
+    <row r="228" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A228" s="2" t="s">
+        <v>1057</v>
+      </c>
+      <c r="B228" s="2" t="s">
+        <v>1057</v>
+      </c>
+      <c r="C228" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D228" s="4">
+        <v>46090</v>
+      </c>
+      <c r="E228" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="F228" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="G228" s="2" t="s">
+        <v>1058</v>
+      </c>
+      <c r="H228" s="2" t="s">
+        <v>1059</v>
+      </c>
+      <c r="I228" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="J228" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="K228" s="2" t="s">
+        <v>1060</v>
+      </c>
+      <c r="L228" s="2" t="s">
+        <v>1061</v>
+      </c>
+      <c r="M228" s="2" t="s">
+        <v>1062</v>
+      </c>
+      <c r="N228" s="2" t="s">
+        <v>1063</v>
+      </c>
+      <c r="O228" s="5">
+        <v>1</v>
+      </c>
+      <c r="P228" s="5">
+        <v>10</v>
+      </c>
+      <c r="Q228" s="6">
+        <v>10</v>
+      </c>
+      <c r="R228" s="6">
+        <v>0</v>
+      </c>
+      <c r="S228" s="6">
+        <v>10</v>
+      </c>
+      <c r="T228" s="6">
+        <v>0</v>
+      </c>
+      <c r="U228" s="6">
+        <v>0</v>
+      </c>
+      <c r="V228" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="W228" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="X228" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y228" s="2" t="s">
+        <v>1064</v>
+      </c>
+      <c r="Z228" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA228" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB228" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="AC228" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD228" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="AE228" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="AF228" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="AG228" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH228" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI228" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ228" s="5">
+        <v>9.1311099999999996</v>
+      </c>
+    </row>
+    <row r="229" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A229" s="3" t="s">
+        <v>1057</v>
+      </c>
+      <c r="B229" s="3" t="s">
+        <v>1057</v>
+      </c>
+      <c r="C229" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D229" s="7">
+        <v>46090</v>
+      </c>
+      <c r="E229" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="F229" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="G229" s="3" t="s">
+        <v>1058</v>
+      </c>
+      <c r="H229" s="3" t="s">
+        <v>1059</v>
+      </c>
+      <c r="I229" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="J229" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="K229" s="3" t="s">
+        <v>784</v>
+      </c>
+      <c r="L229" s="3" t="s">
+        <v>865</v>
+      </c>
+      <c r="M229" s="3" t="s">
+        <v>866</v>
+      </c>
+      <c r="N229" s="3" t="s">
+        <v>867</v>
+      </c>
+      <c r="O229" s="8">
+        <v>1</v>
+      </c>
+      <c r="P229" s="8">
+        <v>10</v>
+      </c>
+      <c r="Q229" s="9">
+        <v>10</v>
+      </c>
+      <c r="R229" s="9">
+        <v>0</v>
+      </c>
+      <c r="S229" s="9">
+        <v>10</v>
+      </c>
+      <c r="T229" s="9">
+        <v>0</v>
+      </c>
+      <c r="U229" s="9">
+        <v>0</v>
+      </c>
+      <c r="V229" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="W229" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="X229" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y229" s="3" t="s">
+        <v>1064</v>
+      </c>
+      <c r="Z229" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA229" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB229" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="AC229" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD229" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="AE229" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="AF229" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="AG229" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH229" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI229" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ229" s="8">
+        <v>9.8148</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08A0FB20-CDDD-4477-B867-5F1CAAB1D4C5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11535412-83B7-4F7D-A32C-87312564DCEE}">
   <dimension ref="A1:AJ66"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
@@ -29030,13 +30220,13 @@
     </row>
     <row r="2" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>1257</v>
+        <v>1287</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>1257</v>
+        <v>1287</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D2" s="4">
         <v>46024</v>
@@ -29048,10 +30238,10 @@
         <v>40</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>1038</v>
+        <v>1070</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>1037</v>
+        <v>1069</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>43</v>
@@ -29063,13 +30253,13 @@
         <v>440</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>1106</v>
+        <v>1137</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>1105</v>
+        <v>1136</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>1104</v>
+        <v>1135</v>
       </c>
       <c r="O2" s="5">
         <v>50</v>
@@ -29093,16 +30283,16 @@
         <v>39.06</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>1103</v>
+        <v>1134</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>1102</v>
+        <v>1133</v>
       </c>
       <c r="X2" s="2" t="s">
         <v>51</v>
       </c>
       <c r="Y2" s="2" t="s">
-        <v>1256</v>
+        <v>1286</v>
       </c>
       <c r="Z2" s="2" t="s">
         <v>0</v>
@@ -29140,13 +30330,13 @@
     </row>
     <row r="3" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>1255</v>
+        <v>1285</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>1255</v>
+        <v>1285</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D3" s="7">
         <v>46027</v>
@@ -29158,10 +30348,10 @@
         <v>61</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>1121</v>
+        <v>1152</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>1120</v>
+        <v>1151</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>163</v>
@@ -29173,13 +30363,13 @@
         <v>632</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>1119</v>
+        <v>1150</v>
       </c>
       <c r="M3" s="3" t="s">
         <v>648</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>1118</v>
+        <v>1149</v>
       </c>
       <c r="O3" s="8">
         <v>1001</v>
@@ -29212,7 +30402,7 @@
         <v>51</v>
       </c>
       <c r="Y3" s="3" t="s">
-        <v>1254</v>
+        <v>1284</v>
       </c>
       <c r="Z3" s="3" t="s">
         <v>0</v>
@@ -29250,13 +30440,13 @@
     </row>
     <row r="4" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>1253</v>
+        <v>1283</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>1253</v>
+        <v>1283</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D4" s="4">
         <v>46027</v>
@@ -29268,10 +30458,10 @@
         <v>61</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>1252</v>
+        <v>1282</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>1251</v>
+        <v>1281</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>152</v>
@@ -29283,13 +30473,13 @@
         <v>342</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>1250</v>
+        <v>1280</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>1249</v>
+        <v>1279</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>1248</v>
+        <v>1278</v>
       </c>
       <c r="O4" s="5">
         <v>600</v>
@@ -29313,16 +30503,16 @@
         <v>355.68</v>
       </c>
       <c r="V4" s="2" t="s">
-        <v>1247</v>
+        <v>1277</v>
       </c>
       <c r="W4" s="2" t="s">
-        <v>1246</v>
+        <v>1276</v>
       </c>
       <c r="X4" s="2" t="s">
         <v>51</v>
       </c>
       <c r="Y4" s="2" t="s">
-        <v>1245</v>
+        <v>1275</v>
       </c>
       <c r="Z4" s="2" t="s">
         <v>0</v>
@@ -29360,13 +30550,13 @@
     </row>
     <row r="5" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>1244</v>
+        <v>1274</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1244</v>
+        <v>1274</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D5" s="7">
         <v>46029</v>
@@ -29378,10 +30568,10 @@
         <v>212</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>1162</v>
+        <v>1193</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>1161</v>
+        <v>1192</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>139</v>
@@ -29390,7 +30580,7 @@
         <v>140</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>1243</v>
+        <v>1273</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>0</v>
@@ -29432,7 +30622,7 @@
         <v>87</v>
       </c>
       <c r="Y5" s="3" t="s">
-        <v>1242</v>
+        <v>1272</v>
       </c>
       <c r="Z5" s="3" t="s">
         <v>0</v>
@@ -29470,13 +30660,13 @@
     </row>
     <row r="6" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>1244</v>
+        <v>1274</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1244</v>
+        <v>1274</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D6" s="4">
         <v>46029</v>
@@ -29488,10 +30678,10 @@
         <v>212</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>1162</v>
+        <v>1193</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>1161</v>
+        <v>1192</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>139</v>
@@ -29500,7 +30690,7 @@
         <v>140</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>1243</v>
+        <v>1273</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>0</v>
@@ -29542,7 +30732,7 @@
         <v>87</v>
       </c>
       <c r="Y6" s="2" t="s">
-        <v>1242</v>
+        <v>1272</v>
       </c>
       <c r="Z6" s="2" t="s">
         <v>0</v>
@@ -29580,13 +30770,13 @@
     </row>
     <row r="7" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>1241</v>
+        <v>1271</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1241</v>
+        <v>1271</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D7" s="7">
         <v>46029</v>
@@ -29604,22 +30794,22 @@
         <v>386</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>1125</v>
+        <v>1156</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>1124</v>
+        <v>1155</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>1068</v>
+        <v>1060</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>1240</v>
+        <v>1270</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>1239</v>
+        <v>1269</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>1238</v>
+        <v>1268</v>
       </c>
       <c r="O7" s="8">
         <v>1000</v>
@@ -29652,7 +30842,7 @@
         <v>51</v>
       </c>
       <c r="Y7" s="3" t="s">
-        <v>1237</v>
+        <v>1267</v>
       </c>
       <c r="Z7" s="3" t="s">
         <v>0</v>
@@ -29690,13 +30880,13 @@
     </row>
     <row r="8" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>1236</v>
+        <v>1266</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>1236</v>
+        <v>1266</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D8" s="4">
         <v>46036</v>
@@ -29708,10 +30898,10 @@
         <v>61</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>1121</v>
+        <v>1152</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>1120</v>
+        <v>1151</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>163</v>
@@ -29723,13 +30913,13 @@
         <v>632</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>1119</v>
+        <v>1150</v>
       </c>
       <c r="M8" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>1118</v>
+        <v>1149</v>
       </c>
       <c r="O8" s="5">
         <v>1001</v>
@@ -29762,7 +30952,7 @@
         <v>51</v>
       </c>
       <c r="Y8" s="2" t="s">
-        <v>1235</v>
+        <v>1265</v>
       </c>
       <c r="Z8" s="2" t="s">
         <v>0</v>
@@ -29800,13 +30990,13 @@
     </row>
     <row r="9" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
-        <v>1234</v>
+        <v>1264</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1234</v>
+        <v>1264</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D9" s="7">
         <v>46037</v>
@@ -29818,10 +31008,10 @@
         <v>61</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>1134</v>
+        <v>1165</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>1133</v>
+        <v>1164</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>163</v>
@@ -29833,13 +31023,13 @@
         <v>417</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>1233</v>
+        <v>1263</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>1232</v>
+        <v>1043</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>1130</v>
+        <v>1161</v>
       </c>
       <c r="O9" s="8">
         <v>1000</v>
@@ -29872,7 +31062,7 @@
         <v>51</v>
       </c>
       <c r="Y9" s="3" t="s">
-        <v>1231</v>
+        <v>1262</v>
       </c>
       <c r="Z9" s="3" t="s">
         <v>0</v>
@@ -29910,13 +31100,13 @@
     </row>
     <row r="10" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>1230</v>
+        <v>1261</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>1230</v>
+        <v>1261</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D10" s="4">
         <v>46037</v>
@@ -29928,10 +31118,10 @@
         <v>40</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>1082</v>
+        <v>1113</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>1081</v>
+        <v>1112</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>139</v>
@@ -29943,13 +31133,13 @@
         <v>784</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>1080</v>
+        <v>1111</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>1079</v>
+        <v>1110</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>1078</v>
+        <v>1109</v>
       </c>
       <c r="O10" s="5">
         <v>300</v>
@@ -29982,7 +31172,7 @@
         <v>51</v>
       </c>
       <c r="Y10" s="2" t="s">
-        <v>1229</v>
+        <v>1260</v>
       </c>
       <c r="Z10" s="2" t="s">
         <v>0</v>
@@ -30020,13 +31210,13 @@
     </row>
     <row r="11" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>1228</v>
+        <v>1259</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>1228</v>
+        <v>1259</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D11" s="7">
         <v>46037</v>
@@ -30038,10 +31228,10 @@
         <v>40</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>1172</v>
+        <v>1203</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>1171</v>
+        <v>1202</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>43</v>
@@ -30053,13 +31243,13 @@
         <v>300</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>1227</v>
+        <v>1258</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>1226</v>
+        <v>1257</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>1225</v>
+        <v>1256</v>
       </c>
       <c r="O11" s="8">
         <v>25</v>
@@ -30092,7 +31282,7 @@
         <v>51</v>
       </c>
       <c r="Y11" s="3" t="s">
-        <v>1224</v>
+        <v>1255</v>
       </c>
       <c r="Z11" s="3" t="s">
         <v>0</v>
@@ -30130,13 +31320,13 @@
     </row>
     <row r="12" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>1223</v>
+        <v>1254</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>1223</v>
+        <v>1254</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D12" s="4">
         <v>46041</v>
@@ -30148,10 +31338,10 @@
         <v>212</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>1162</v>
+        <v>1193</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>1161</v>
+        <v>1192</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>139</v>
@@ -30160,7 +31350,7 @@
         <v>140</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>1054</v>
+        <v>1086</v>
       </c>
       <c r="L12" s="2" t="s">
         <v>0</v>
@@ -30202,7 +31392,7 @@
         <v>87</v>
       </c>
       <c r="Y12" s="2" t="s">
-        <v>1222</v>
+        <v>1253</v>
       </c>
       <c r="Z12" s="2" t="s">
         <v>0</v>
@@ -30217,10 +31407,10 @@
         <v>55</v>
       </c>
       <c r="AD12" s="2" t="s">
-        <v>1049</v>
+        <v>1081</v>
       </c>
       <c r="AE12" s="2" t="s">
-        <v>1048</v>
+        <v>1080</v>
       </c>
       <c r="AF12" s="2" t="s">
         <v>442</v>
@@ -30240,13 +31430,13 @@
     </row>
     <row r="13" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>1221</v>
+        <v>1252</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>1221</v>
+        <v>1252</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D13" s="7">
         <v>46042</v>
@@ -30264,22 +31454,22 @@
         <v>386</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>1125</v>
+        <v>1156</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>1124</v>
+        <v>1155</v>
       </c>
       <c r="K13" s="3" t="s">
         <v>446</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>1128</v>
+        <v>1159</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>1127</v>
+        <v>1158</v>
       </c>
       <c r="N13" s="3" t="s">
-        <v>1093</v>
+        <v>1124</v>
       </c>
       <c r="O13" s="8">
         <v>2000</v>
@@ -30312,7 +31502,7 @@
         <v>51</v>
       </c>
       <c r="Y13" s="3" t="s">
-        <v>1220</v>
+        <v>1251</v>
       </c>
       <c r="Z13" s="3" t="s">
         <v>0</v>
@@ -30350,13 +31540,13 @@
     </row>
     <row r="14" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>1219</v>
+        <v>1250</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>1219</v>
+        <v>1250</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D14" s="4">
         <v>46042</v>
@@ -30380,16 +31570,16 @@
         <v>294</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>1054</v>
+        <v>1086</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>1187</v>
+        <v>1218</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>1186</v>
+        <v>1217</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>1051</v>
+        <v>1083</v>
       </c>
       <c r="O14" s="5">
         <v>6000</v>
@@ -30413,16 +31603,16 @@
         <v>12873.6</v>
       </c>
       <c r="V14" s="2" t="s">
-        <v>1218</v>
+        <v>1249</v>
       </c>
       <c r="W14" s="2" t="s">
-        <v>1217</v>
+        <v>1248</v>
       </c>
       <c r="X14" s="2" t="s">
         <v>51</v>
       </c>
       <c r="Y14" s="2" t="s">
-        <v>1216</v>
+        <v>1247</v>
       </c>
       <c r="Z14" s="2" t="s">
         <v>0</v>
@@ -30437,10 +31627,10 @@
         <v>298</v>
       </c>
       <c r="AD14" s="2" t="s">
-        <v>1049</v>
+        <v>1081</v>
       </c>
       <c r="AE14" s="2" t="s">
-        <v>1048</v>
+        <v>1080</v>
       </c>
       <c r="AF14" s="2" t="s">
         <v>77</v>
@@ -30460,13 +31650,13 @@
     </row>
     <row r="15" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>1215</v>
+        <v>1246</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>1215</v>
+        <v>1246</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D15" s="7">
         <v>46042</v>
@@ -30478,10 +31668,10 @@
         <v>212</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>1162</v>
+        <v>1193</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>1161</v>
+        <v>1192</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>139</v>
@@ -30532,7 +31722,7 @@
         <v>87</v>
       </c>
       <c r="Y15" s="3" t="s">
-        <v>1214</v>
+        <v>1245</v>
       </c>
       <c r="Z15" s="3" t="s">
         <v>0</v>
@@ -30553,7 +31743,7 @@
         <v>518</v>
       </c>
       <c r="AF15" s="3" t="s">
-        <v>1182</v>
+        <v>1213</v>
       </c>
       <c r="AG15" s="9">
         <v>0</v>
@@ -30570,13 +31760,13 @@
     </row>
     <row r="16" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>1215</v>
+        <v>1246</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>1215</v>
+        <v>1246</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D16" s="4">
         <v>46042</v>
@@ -30588,10 +31778,10 @@
         <v>212</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>1162</v>
+        <v>1193</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>1161</v>
+        <v>1192</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>139</v>
@@ -30642,7 +31832,7 @@
         <v>87</v>
       </c>
       <c r="Y16" s="2" t="s">
-        <v>1214</v>
+        <v>1245</v>
       </c>
       <c r="Z16" s="2" t="s">
         <v>0</v>
@@ -30663,7 +31853,7 @@
         <v>518</v>
       </c>
       <c r="AF16" s="2" t="s">
-        <v>1182</v>
+        <v>1213</v>
       </c>
       <c r="AG16" s="6">
         <v>0</v>
@@ -30680,13 +31870,13 @@
     </row>
     <row r="17" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
-        <v>1213</v>
+        <v>1244</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>1213</v>
+        <v>1244</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D17" s="7">
         <v>46043</v>
@@ -30713,13 +31903,13 @@
         <v>417</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>1132</v>
+        <v>1163</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>1131</v>
+        <v>1162</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>1130</v>
+        <v>1161</v>
       </c>
       <c r="O17" s="8">
         <v>1000</v>
@@ -30752,7 +31942,7 @@
         <v>51</v>
       </c>
       <c r="Y17" s="3" t="s">
-        <v>1212</v>
+        <v>1243</v>
       </c>
       <c r="Z17" s="3" t="s">
         <v>0</v>
@@ -30790,28 +31980,28 @@
     </row>
     <row r="18" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>1200</v>
+        <v>1231</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>1200</v>
+        <v>1231</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D18" s="4">
         <v>46045</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>1199</v>
+        <v>1230</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>1198</v>
+        <v>1229</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>1138</v>
+        <v>1169</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>1137</v>
+        <v>1168</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>139</v>
@@ -30823,13 +32013,13 @@
         <v>628</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>1211</v>
+        <v>1242</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>1210</v>
+        <v>1241</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>1209</v>
+        <v>1240</v>
       </c>
       <c r="O18" s="5">
         <v>2000</v>
@@ -30853,16 +32043,16 @@
         <v>0</v>
       </c>
       <c r="V18" s="2" t="s">
-        <v>1194</v>
+        <v>1225</v>
       </c>
       <c r="W18" s="2" t="s">
-        <v>1161</v>
+        <v>1192</v>
       </c>
       <c r="X18" s="2" t="s">
         <v>87</v>
       </c>
       <c r="Y18" s="2" t="s">
-        <v>1193</v>
+        <v>1224</v>
       </c>
       <c r="Z18" s="2" t="s">
         <v>0</v>
@@ -30900,28 +32090,28 @@
     </row>
     <row r="19" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
-        <v>1200</v>
+        <v>1231</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>1200</v>
+        <v>1231</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D19" s="7">
         <v>46045</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>1199</v>
+        <v>1230</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>1198</v>
+        <v>1229</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>1138</v>
+        <v>1169</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>1137</v>
+        <v>1168</v>
       </c>
       <c r="I19" s="3" t="s">
         <v>139</v>
@@ -30933,13 +32123,13 @@
         <v>631</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>1208</v>
+        <v>1239</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>1207</v>
+        <v>1238</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>1195</v>
+        <v>1226</v>
       </c>
       <c r="O19" s="8">
         <v>11725</v>
@@ -30963,16 +32153,16 @@
         <v>0</v>
       </c>
       <c r="V19" s="3" t="s">
-        <v>1194</v>
+        <v>1225</v>
       </c>
       <c r="W19" s="3" t="s">
-        <v>1161</v>
+        <v>1192</v>
       </c>
       <c r="X19" s="3" t="s">
         <v>87</v>
       </c>
       <c r="Y19" s="3" t="s">
-        <v>1193</v>
+        <v>1224</v>
       </c>
       <c r="Z19" s="3" t="s">
         <v>0</v>
@@ -31010,28 +32200,28 @@
     </row>
     <row r="20" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>1200</v>
+        <v>1231</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>1200</v>
+        <v>1231</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D20" s="4">
         <v>46045</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>1199</v>
+        <v>1230</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>1198</v>
+        <v>1229</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>1138</v>
+        <v>1169</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>1137</v>
+        <v>1168</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>139</v>
@@ -31043,13 +32233,13 @@
         <v>632</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>1119</v>
+        <v>1150</v>
       </c>
       <c r="M20" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>1118</v>
+        <v>1149</v>
       </c>
       <c r="O20" s="5">
         <v>2925</v>
@@ -31073,16 +32263,16 @@
         <v>0</v>
       </c>
       <c r="V20" s="2" t="s">
-        <v>1194</v>
+        <v>1225</v>
       </c>
       <c r="W20" s="2" t="s">
-        <v>1161</v>
+        <v>1192</v>
       </c>
       <c r="X20" s="2" t="s">
         <v>87</v>
       </c>
       <c r="Y20" s="2" t="s">
-        <v>1193</v>
+        <v>1224</v>
       </c>
       <c r="Z20" s="2" t="s">
         <v>0</v>
@@ -31120,28 +32310,28 @@
     </row>
     <row r="21" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
-        <v>1200</v>
+        <v>1231</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>1200</v>
+        <v>1231</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D21" s="7">
         <v>46045</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>1199</v>
+        <v>1230</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>1198</v>
+        <v>1229</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>1138</v>
+        <v>1169</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>1137</v>
+        <v>1168</v>
       </c>
       <c r="I21" s="3" t="s">
         <v>139</v>
@@ -31153,13 +32343,13 @@
         <v>633</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>1062</v>
+        <v>1094</v>
       </c>
       <c r="M21" s="3" t="s">
         <v>652</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>1061</v>
+        <v>1093</v>
       </c>
       <c r="O21" s="8">
         <v>2925</v>
@@ -31183,16 +32373,16 @@
         <v>0</v>
       </c>
       <c r="V21" s="3" t="s">
-        <v>1194</v>
+        <v>1225</v>
       </c>
       <c r="W21" s="3" t="s">
-        <v>1161</v>
+        <v>1192</v>
       </c>
       <c r="X21" s="3" t="s">
         <v>87</v>
       </c>
       <c r="Y21" s="3" t="s">
-        <v>1193</v>
+        <v>1224</v>
       </c>
       <c r="Z21" s="3" t="s">
         <v>0</v>
@@ -31230,28 +32420,28 @@
     </row>
     <row r="22" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>1200</v>
+        <v>1231</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>1200</v>
+        <v>1231</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D22" s="4">
         <v>46045</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>1199</v>
+        <v>1230</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>1198</v>
+        <v>1229</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>1138</v>
+        <v>1169</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>1137</v>
+        <v>1168</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>139</v>
@@ -31263,13 +32453,13 @@
         <v>465</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>1206</v>
+        <v>1237</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>1205</v>
+        <v>1236</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>1204</v>
+        <v>1235</v>
       </c>
       <c r="O22" s="5">
         <v>2400</v>
@@ -31293,16 +32483,16 @@
         <v>0</v>
       </c>
       <c r="V22" s="2" t="s">
-        <v>1194</v>
+        <v>1225</v>
       </c>
       <c r="W22" s="2" t="s">
-        <v>1161</v>
+        <v>1192</v>
       </c>
       <c r="X22" s="2" t="s">
         <v>87</v>
       </c>
       <c r="Y22" s="2" t="s">
-        <v>1193</v>
+        <v>1224</v>
       </c>
       <c r="Z22" s="2" t="s">
         <v>0</v>
@@ -31340,28 +32530,28 @@
     </row>
     <row r="23" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
-        <v>1200</v>
+        <v>1231</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>1200</v>
+        <v>1231</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D23" s="7">
         <v>46045</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>1199</v>
+        <v>1230</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>1198</v>
+        <v>1229</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>1138</v>
+        <v>1169</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>1137</v>
+        <v>1168</v>
       </c>
       <c r="I23" s="3" t="s">
         <v>139</v>
@@ -31373,13 +32563,13 @@
         <v>465</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>1203</v>
+        <v>1234</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>1202</v>
+        <v>1233</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>1201</v>
+        <v>1232</v>
       </c>
       <c r="O23" s="8">
         <v>1800</v>
@@ -31403,16 +32593,16 @@
         <v>0</v>
       </c>
       <c r="V23" s="3" t="s">
-        <v>1194</v>
+        <v>1225</v>
       </c>
       <c r="W23" s="3" t="s">
-        <v>1161</v>
+        <v>1192</v>
       </c>
       <c r="X23" s="3" t="s">
         <v>87</v>
       </c>
       <c r="Y23" s="3" t="s">
-        <v>1193</v>
+        <v>1224</v>
       </c>
       <c r="Z23" s="3" t="s">
         <v>0</v>
@@ -31450,28 +32640,28 @@
     </row>
     <row r="24" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>1200</v>
+        <v>1231</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>1200</v>
+        <v>1231</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D24" s="4">
         <v>46045</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>1199</v>
+        <v>1230</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>1198</v>
+        <v>1229</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>1138</v>
+        <v>1169</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>1137</v>
+        <v>1168</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>139</v>
@@ -31483,13 +32673,13 @@
         <v>634</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>1197</v>
+        <v>1228</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>1196</v>
+        <v>1227</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>1195</v>
+        <v>1226</v>
       </c>
       <c r="O24" s="5">
         <v>1400</v>
@@ -31513,16 +32703,16 @@
         <v>0</v>
       </c>
       <c r="V24" s="2" t="s">
-        <v>1194</v>
+        <v>1225</v>
       </c>
       <c r="W24" s="2" t="s">
-        <v>1161</v>
+        <v>1192</v>
       </c>
       <c r="X24" s="2" t="s">
         <v>87</v>
       </c>
       <c r="Y24" s="2" t="s">
-        <v>1193</v>
+        <v>1224</v>
       </c>
       <c r="Z24" s="2" t="s">
         <v>0</v>
@@ -31560,13 +32750,13 @@
     </row>
     <row r="25" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
-        <v>1192</v>
+        <v>1223</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>1192</v>
+        <v>1223</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D25" s="7">
         <v>46048</v>
@@ -31593,13 +32783,13 @@
         <v>417</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>1144</v>
+        <v>1175</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>1143</v>
+        <v>1174</v>
       </c>
       <c r="N25" s="3" t="s">
-        <v>1142</v>
+        <v>1173</v>
       </c>
       <c r="O25" s="8">
         <v>5000</v>
@@ -31623,16 +32813,16 @@
         <v>2354</v>
       </c>
       <c r="V25" s="3" t="s">
-        <v>1072</v>
+        <v>1103</v>
       </c>
       <c r="W25" s="3" t="s">
-        <v>1071</v>
+        <v>1102</v>
       </c>
       <c r="X25" s="3" t="s">
         <v>51</v>
       </c>
       <c r="Y25" s="3" t="s">
-        <v>1191</v>
+        <v>1222</v>
       </c>
       <c r="Z25" s="3" t="s">
         <v>0</v>
@@ -31670,13 +32860,13 @@
     </row>
     <row r="26" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>1190</v>
+        <v>1221</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>1190</v>
+        <v>1221</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D26" s="4">
         <v>46048</v>
@@ -31688,10 +32878,10 @@
         <v>40</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>1082</v>
+        <v>1113</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>1081</v>
+        <v>1112</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>139</v>
@@ -31703,13 +32893,13 @@
         <v>784</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>1080</v>
+        <v>1111</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>1079</v>
+        <v>1110</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>1078</v>
+        <v>1109</v>
       </c>
       <c r="O26" s="5">
         <v>300</v>
@@ -31742,7 +32932,7 @@
         <v>51</v>
       </c>
       <c r="Y26" s="2" t="s">
-        <v>1189</v>
+        <v>1220</v>
       </c>
       <c r="Z26" s="2" t="s">
         <v>0</v>
@@ -31780,13 +32970,13 @@
     </row>
     <row r="27" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
-        <v>1188</v>
+        <v>1219</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>1188</v>
+        <v>1219</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D27" s="7">
         <v>46048</v>
@@ -31798,10 +32988,10 @@
         <v>61</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>1121</v>
+        <v>1152</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>1120</v>
+        <v>1151</v>
       </c>
       <c r="I27" s="3" t="s">
         <v>163</v>
@@ -31813,13 +33003,13 @@
         <v>632</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>1119</v>
+        <v>1150</v>
       </c>
       <c r="M27" s="3" t="s">
         <v>648</v>
       </c>
       <c r="N27" s="3" t="s">
-        <v>1118</v>
+        <v>1149</v>
       </c>
       <c r="O27" s="8">
         <v>611</v>
@@ -31852,7 +33042,7 @@
         <v>51</v>
       </c>
       <c r="Y27" s="3" t="s">
-        <v>1185</v>
+        <v>1216</v>
       </c>
       <c r="Z27" s="3" t="s">
         <v>0</v>
@@ -31890,13 +33080,13 @@
     </row>
     <row r="28" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>1188</v>
+        <v>1219</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>1188</v>
+        <v>1219</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D28" s="4">
         <v>46048</v>
@@ -31908,10 +33098,10 @@
         <v>61</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>1121</v>
+        <v>1152</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>1120</v>
+        <v>1151</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>163</v>
@@ -31920,16 +33110,16 @@
         <v>164</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>1054</v>
+        <v>1086</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>1187</v>
+        <v>1218</v>
       </c>
       <c r="M28" s="2" t="s">
-        <v>1186</v>
+        <v>1217</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>1051</v>
+        <v>1083</v>
       </c>
       <c r="O28" s="5">
         <v>700</v>
@@ -31962,7 +33152,7 @@
         <v>51</v>
       </c>
       <c r="Y28" s="2" t="s">
-        <v>1185</v>
+        <v>1216</v>
       </c>
       <c r="Z28" s="2" t="s">
         <v>0</v>
@@ -31977,10 +33167,10 @@
         <v>55</v>
       </c>
       <c r="AD28" s="2" t="s">
-        <v>1049</v>
+        <v>1081</v>
       </c>
       <c r="AE28" s="2" t="s">
-        <v>1048</v>
+        <v>1080</v>
       </c>
       <c r="AF28" s="2" t="s">
         <v>77</v>
@@ -32000,13 +33190,13 @@
     </row>
     <row r="29" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
-        <v>1184</v>
+        <v>1215</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>1184</v>
+        <v>1215</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D29" s="7">
         <v>46048</v>
@@ -32018,10 +33208,10 @@
         <v>212</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>1162</v>
+        <v>1193</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>1161</v>
+        <v>1192</v>
       </c>
       <c r="I29" s="3" t="s">
         <v>139</v>
@@ -32072,7 +33262,7 @@
         <v>87</v>
       </c>
       <c r="Y29" s="3" t="s">
-        <v>1183</v>
+        <v>1214</v>
       </c>
       <c r="Z29" s="3" t="s">
         <v>0</v>
@@ -32093,7 +33283,7 @@
         <v>57</v>
       </c>
       <c r="AF29" s="3" t="s">
-        <v>1182</v>
+        <v>1213</v>
       </c>
       <c r="AG29" s="9">
         <v>0</v>
@@ -32110,13 +33300,13 @@
     </row>
     <row r="30" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>1181</v>
+        <v>1212</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>1181</v>
+        <v>1212</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D30" s="4">
         <v>46049</v>
@@ -32128,10 +33318,10 @@
         <v>212</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>1162</v>
+        <v>1193</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>1161</v>
+        <v>1192</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>139</v>
@@ -32182,7 +33372,7 @@
         <v>87</v>
       </c>
       <c r="Y30" s="2" t="s">
-        <v>1180</v>
+        <v>1211</v>
       </c>
       <c r="Z30" s="2" t="s">
         <v>0</v>
@@ -32220,13 +33410,13 @@
     </row>
     <row r="31" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
-        <v>1181</v>
+        <v>1212</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>1181</v>
+        <v>1212</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D31" s="7">
         <v>46049</v>
@@ -32238,10 +33428,10 @@
         <v>212</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>1162</v>
+        <v>1193</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>1161</v>
+        <v>1192</v>
       </c>
       <c r="I31" s="3" t="s">
         <v>139</v>
@@ -32292,7 +33482,7 @@
         <v>87</v>
       </c>
       <c r="Y31" s="3" t="s">
-        <v>1180</v>
+        <v>1211</v>
       </c>
       <c r="Z31" s="3" t="s">
         <v>0</v>
@@ -32330,13 +33520,13 @@
     </row>
     <row r="32" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>1177</v>
+        <v>1208</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>1177</v>
+        <v>1208</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D32" s="4">
         <v>46050</v>
@@ -32354,22 +33544,22 @@
         <v>386</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>1125</v>
+        <v>1156</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>1124</v>
+        <v>1155</v>
       </c>
       <c r="K32" s="2" t="s">
         <v>446</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>1179</v>
+        <v>1210</v>
       </c>
       <c r="M32" s="2" t="s">
         <v>448</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>1178</v>
+        <v>1209</v>
       </c>
       <c r="O32" s="5">
         <v>1000</v>
@@ -32402,7 +33592,7 @@
         <v>51</v>
       </c>
       <c r="Y32" s="2" t="s">
-        <v>1176</v>
+        <v>1207</v>
       </c>
       <c r="Z32" s="2" t="s">
         <v>0</v>
@@ -32440,13 +33630,13 @@
     </row>
     <row r="33" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
-        <v>1177</v>
+        <v>1208</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>1177</v>
+        <v>1208</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D33" s="7">
         <v>46050</v>
@@ -32464,22 +33654,22 @@
         <v>386</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>1125</v>
+        <v>1156</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>1124</v>
+        <v>1155</v>
       </c>
       <c r="K33" s="3" t="s">
         <v>446</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>1128</v>
+        <v>1159</v>
       </c>
       <c r="M33" s="3" t="s">
-        <v>1127</v>
+        <v>1158</v>
       </c>
       <c r="N33" s="3" t="s">
-        <v>1093</v>
+        <v>1124</v>
       </c>
       <c r="O33" s="8">
         <v>1000</v>
@@ -32512,7 +33702,7 @@
         <v>51</v>
       </c>
       <c r="Y33" s="3" t="s">
-        <v>1176</v>
+        <v>1207</v>
       </c>
       <c r="Z33" s="3" t="s">
         <v>0</v>
@@ -32550,13 +33740,13 @@
     </row>
     <row r="34" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>1175</v>
+        <v>1206</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>1175</v>
+        <v>1206</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D34" s="4">
         <v>46050</v>
@@ -32568,10 +33758,10 @@
         <v>212</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>1162</v>
+        <v>1193</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>1161</v>
+        <v>1192</v>
       </c>
       <c r="I34" s="2" t="s">
         <v>139</v>
@@ -32622,7 +33812,7 @@
         <v>87</v>
       </c>
       <c r="Y34" s="2" t="s">
-        <v>1174</v>
+        <v>1205</v>
       </c>
       <c r="Z34" s="2" t="s">
         <v>0</v>
@@ -32660,13 +33850,13 @@
     </row>
     <row r="35" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
-        <v>1173</v>
+        <v>1204</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>1173</v>
+        <v>1204</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D35" s="7">
         <v>46051</v>
@@ -32678,10 +33868,10 @@
         <v>40</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>1172</v>
+        <v>1203</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>1171</v>
+        <v>1202</v>
       </c>
       <c r="I35" s="3" t="s">
         <v>43</v>
@@ -32693,13 +33883,13 @@
         <v>632</v>
       </c>
       <c r="L35" s="3" t="s">
-        <v>1119</v>
+        <v>1150</v>
       </c>
       <c r="M35" s="3" t="s">
         <v>648</v>
       </c>
       <c r="N35" s="3" t="s">
-        <v>1118</v>
+        <v>1149</v>
       </c>
       <c r="O35" s="8">
         <v>26</v>
@@ -32732,7 +33922,7 @@
         <v>51</v>
       </c>
       <c r="Y35" s="3" t="s">
-        <v>1170</v>
+        <v>1201</v>
       </c>
       <c r="Z35" s="3" t="s">
         <v>0</v>
@@ -32770,13 +33960,13 @@
     </row>
     <row r="36" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>1169</v>
+        <v>1200</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>1169</v>
+        <v>1200</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D36" s="4">
         <v>46052</v>
@@ -32788,10 +33978,10 @@
         <v>61</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>1121</v>
+        <v>1152</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>1120</v>
+        <v>1151</v>
       </c>
       <c r="I36" s="2" t="s">
         <v>163</v>
@@ -32803,13 +33993,13 @@
         <v>632</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>1119</v>
+        <v>1150</v>
       </c>
       <c r="M36" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>1118</v>
+        <v>1149</v>
       </c>
       <c r="O36" s="5">
         <v>507</v>
@@ -32842,7 +34032,7 @@
         <v>51</v>
       </c>
       <c r="Y36" s="2" t="s">
-        <v>1168</v>
+        <v>1199</v>
       </c>
       <c r="Z36" s="2" t="s">
         <v>0</v>
@@ -32880,13 +34070,13 @@
     </row>
     <row r="37" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
-        <v>1167</v>
+        <v>1198</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>1167</v>
+        <v>1198</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D37" s="7">
         <v>46052</v>
@@ -32910,16 +34100,16 @@
         <v>164</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>1059</v>
+        <v>1091</v>
       </c>
       <c r="L37" s="3" t="s">
-        <v>1087</v>
+        <v>1118</v>
       </c>
       <c r="M37" s="3" t="s">
-        <v>1086</v>
+        <v>1117</v>
       </c>
       <c r="N37" s="3" t="s">
-        <v>1056</v>
+        <v>1088</v>
       </c>
       <c r="O37" s="8">
         <v>500</v>
@@ -32952,7 +34142,7 @@
         <v>51</v>
       </c>
       <c r="Y37" s="3" t="s">
-        <v>1166</v>
+        <v>1197</v>
       </c>
       <c r="Z37" s="3" t="s">
         <v>0</v>
@@ -32990,13 +34180,13 @@
     </row>
     <row r="38" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>1165</v>
+        <v>1196</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>1165</v>
+        <v>1196</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D38" s="4">
         <v>46052</v>
@@ -33008,10 +34198,10 @@
         <v>40</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>1082</v>
+        <v>1113</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>1081</v>
+        <v>1112</v>
       </c>
       <c r="I38" s="2" t="s">
         <v>139</v>
@@ -33023,13 +34213,13 @@
         <v>784</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>1080</v>
+        <v>1111</v>
       </c>
       <c r="M38" s="2" t="s">
-        <v>1079</v>
+        <v>1110</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>1078</v>
+        <v>1109</v>
       </c>
       <c r="O38" s="5">
         <v>300</v>
@@ -33062,7 +34252,7 @@
         <v>51</v>
       </c>
       <c r="Y38" s="2" t="s">
-        <v>1164</v>
+        <v>1195</v>
       </c>
       <c r="Z38" s="2" t="s">
         <v>0</v>
@@ -33100,13 +34290,13 @@
     </row>
     <row r="39" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
-        <v>1163</v>
+        <v>1194</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>1163</v>
+        <v>1194</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D39" s="7">
         <v>46055</v>
@@ -33118,10 +34308,10 @@
         <v>212</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>1162</v>
+        <v>1193</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>1161</v>
+        <v>1192</v>
       </c>
       <c r="I39" s="3" t="s">
         <v>139</v>
@@ -33130,7 +34320,7 @@
         <v>140</v>
       </c>
       <c r="K39" s="3" t="s">
-        <v>1160</v>
+        <v>1191</v>
       </c>
       <c r="L39" s="3" t="s">
         <v>0</v>
@@ -33172,7 +34362,7 @@
         <v>87</v>
       </c>
       <c r="Y39" s="3" t="s">
-        <v>1159</v>
+        <v>1190</v>
       </c>
       <c r="Z39" s="3" t="s">
         <v>0</v>
@@ -33210,13 +34400,13 @@
     </row>
     <row r="40" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>1158</v>
+        <v>1189</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>1158</v>
+        <v>1189</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D40" s="4">
         <v>46057</v>
@@ -33228,10 +34418,10 @@
         <v>61</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>1121</v>
+        <v>1152</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>1120</v>
+        <v>1151</v>
       </c>
       <c r="I40" s="2" t="s">
         <v>163</v>
@@ -33243,13 +34433,13 @@
         <v>632</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>1119</v>
+        <v>1150</v>
       </c>
       <c r="M40" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>1118</v>
+        <v>1149</v>
       </c>
       <c r="O40" s="5">
         <v>507</v>
@@ -33282,7 +34472,7 @@
         <v>51</v>
       </c>
       <c r="Y40" s="2" t="s">
-        <v>1157</v>
+        <v>1188</v>
       </c>
       <c r="Z40" s="2" t="s">
         <v>0</v>
@@ -33320,13 +34510,13 @@
     </row>
     <row r="41" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
-        <v>1156</v>
+        <v>1187</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>1156</v>
+        <v>1187</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D41" s="7">
         <v>46057</v>
@@ -33344,22 +34534,22 @@
         <v>386</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>1125</v>
+        <v>1156</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>1124</v>
+        <v>1155</v>
       </c>
       <c r="K41" s="3" t="s">
         <v>446</v>
       </c>
       <c r="L41" s="3" t="s">
-        <v>1128</v>
+        <v>1159</v>
       </c>
       <c r="M41" s="3" t="s">
-        <v>1127</v>
+        <v>1158</v>
       </c>
       <c r="N41" s="3" t="s">
-        <v>1093</v>
+        <v>1124</v>
       </c>
       <c r="O41" s="8">
         <v>2000</v>
@@ -33392,7 +34582,7 @@
         <v>51</v>
       </c>
       <c r="Y41" s="3" t="s">
-        <v>1123</v>
+        <v>1154</v>
       </c>
       <c r="Z41" s="3" t="s">
         <v>0</v>
@@ -33430,13 +34620,13 @@
     </row>
     <row r="42" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>1155</v>
+        <v>1186</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>1155</v>
+        <v>1186</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D42" s="4">
         <v>46058</v>
@@ -33448,10 +34638,10 @@
         <v>61</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>1121</v>
+        <v>1152</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>1120</v>
+        <v>1151</v>
       </c>
       <c r="I42" s="2" t="s">
         <v>163</v>
@@ -33463,13 +34653,13 @@
         <v>632</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>1119</v>
+        <v>1150</v>
       </c>
       <c r="M42" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>1118</v>
+        <v>1149</v>
       </c>
       <c r="O42" s="5">
         <v>507</v>
@@ -33502,7 +34692,7 @@
         <v>51</v>
       </c>
       <c r="Y42" s="2" t="s">
-        <v>1154</v>
+        <v>1185</v>
       </c>
       <c r="Z42" s="2" t="s">
         <v>0</v>
@@ -33540,13 +34730,13 @@
     </row>
     <row r="43" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
-        <v>1153</v>
+        <v>1184</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>1153</v>
+        <v>1184</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D43" s="7">
         <v>46058</v>
@@ -33558,10 +34748,10 @@
         <v>61</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>1090</v>
+        <v>1121</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>1089</v>
+        <v>1120</v>
       </c>
       <c r="I43" s="3" t="s">
         <v>163</v>
@@ -33573,13 +34763,13 @@
         <v>417</v>
       </c>
       <c r="L43" s="3" t="s">
-        <v>1144</v>
+        <v>1175</v>
       </c>
       <c r="M43" s="3" t="s">
-        <v>1143</v>
+        <v>1174</v>
       </c>
       <c r="N43" s="3" t="s">
-        <v>1142</v>
+        <v>1173</v>
       </c>
       <c r="O43" s="8">
         <v>1800</v>
@@ -33612,7 +34802,7 @@
         <v>51</v>
       </c>
       <c r="Y43" s="3" t="s">
-        <v>1152</v>
+        <v>1183</v>
       </c>
       <c r="Z43" s="3" t="s">
         <v>0</v>
@@ -33650,13 +34840,13 @@
     </row>
     <row r="44" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>1151</v>
+        <v>1182</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>1151</v>
+        <v>1182</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D44" s="4">
         <v>46059</v>
@@ -33668,10 +34858,10 @@
         <v>40</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>1150</v>
+        <v>1181</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>1149</v>
+        <v>1180</v>
       </c>
       <c r="I44" s="2" t="s">
         <v>43</v>
@@ -33683,13 +34873,13 @@
         <v>784</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>1080</v>
+        <v>1111</v>
       </c>
       <c r="M44" s="2" t="s">
-        <v>1079</v>
+        <v>1110</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>1078</v>
+        <v>1109</v>
       </c>
       <c r="O44" s="5">
         <v>500</v>
@@ -33722,7 +34912,7 @@
         <v>51</v>
       </c>
       <c r="Y44" s="2" t="s">
-        <v>1148</v>
+        <v>1179</v>
       </c>
       <c r="Z44" s="2" t="s">
         <v>0</v>
@@ -33760,13 +34950,13 @@
     </row>
     <row r="45" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="3" t="s">
-        <v>1147</v>
+        <v>1178</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>1147</v>
+        <v>1178</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D45" s="7">
         <v>46059</v>
@@ -33778,10 +34968,10 @@
         <v>40</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>1146</v>
+        <v>1177</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>1145</v>
+        <v>1176</v>
       </c>
       <c r="I45" s="3" t="s">
         <v>43</v>
@@ -33793,13 +34983,13 @@
         <v>417</v>
       </c>
       <c r="L45" s="3" t="s">
-        <v>1144</v>
+        <v>1175</v>
       </c>
       <c r="M45" s="3" t="s">
-        <v>1143</v>
+        <v>1174</v>
       </c>
       <c r="N45" s="3" t="s">
-        <v>1142</v>
+        <v>1173</v>
       </c>
       <c r="O45" s="8">
         <v>200</v>
@@ -33832,7 +35022,7 @@
         <v>51</v>
       </c>
       <c r="Y45" s="3" t="s">
-        <v>1141</v>
+        <v>1172</v>
       </c>
       <c r="Z45" s="3" t="s">
         <v>0</v>
@@ -33870,28 +35060,28 @@
     </row>
     <row r="46" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
-        <v>1140</v>
+        <v>1171</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>1140</v>
+        <v>1171</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D46" s="4">
         <v>46063</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>1139</v>
+        <v>1170</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>267</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>1138</v>
+        <v>1169</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>1137</v>
+        <v>1168</v>
       </c>
       <c r="I46" s="2" t="s">
         <v>139</v>
@@ -33900,7 +35090,7 @@
         <v>140</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>1036</v>
+        <v>1068</v>
       </c>
       <c r="L46" s="2" t="s">
         <v>0</v>
@@ -33942,7 +35132,7 @@
         <v>0</v>
       </c>
       <c r="Y46" s="2" t="s">
-        <v>1136</v>
+        <v>1167</v>
       </c>
       <c r="Z46" s="2" t="s">
         <v>0</v>
@@ -33957,10 +35147,10 @@
         <v>74</v>
       </c>
       <c r="AD46" s="2" t="s">
-        <v>1034</v>
+        <v>1066</v>
       </c>
       <c r="AE46" s="2" t="s">
-        <v>1033</v>
+        <v>1065</v>
       </c>
       <c r="AF46" s="2" t="s">
         <v>0</v>
@@ -33980,13 +35170,13 @@
     </row>
     <row r="47" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
-        <v>1135</v>
+        <v>1166</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>1135</v>
+        <v>1166</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D47" s="7">
         <v>46064</v>
@@ -33998,10 +35188,10 @@
         <v>61</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>1134</v>
+        <v>1165</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>1133</v>
+        <v>1164</v>
       </c>
       <c r="I47" s="3" t="s">
         <v>139</v>
@@ -34013,13 +35203,13 @@
         <v>417</v>
       </c>
       <c r="L47" s="3" t="s">
-        <v>1132</v>
+        <v>1163</v>
       </c>
       <c r="M47" s="3" t="s">
-        <v>1131</v>
+        <v>1162</v>
       </c>
       <c r="N47" s="3" t="s">
-        <v>1130</v>
+        <v>1161</v>
       </c>
       <c r="O47" s="8">
         <v>1000</v>
@@ -34052,7 +35242,7 @@
         <v>51</v>
       </c>
       <c r="Y47" s="3" t="s">
-        <v>1129</v>
+        <v>1160</v>
       </c>
       <c r="Z47" s="3" t="s">
         <v>0</v>
@@ -34090,13 +35280,13 @@
     </row>
     <row r="48" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
-        <v>1126</v>
+        <v>1157</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>1126</v>
+        <v>1157</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D48" s="4">
         <v>46064</v>
@@ -34114,22 +35304,22 @@
         <v>386</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>1125</v>
+        <v>1156</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>1124</v>
+        <v>1155</v>
       </c>
       <c r="K48" s="2" t="s">
         <v>446</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>1128</v>
+        <v>1159</v>
       </c>
       <c r="M48" s="2" t="s">
-        <v>1127</v>
+        <v>1158</v>
       </c>
       <c r="N48" s="2" t="s">
-        <v>1093</v>
+        <v>1124</v>
       </c>
       <c r="O48" s="5">
         <v>1000</v>
@@ -34162,7 +35352,7 @@
         <v>51</v>
       </c>
       <c r="Y48" s="2" t="s">
-        <v>1123</v>
+        <v>1154</v>
       </c>
       <c r="Z48" s="2" t="s">
         <v>0</v>
@@ -34200,13 +35390,13 @@
     </row>
     <row r="49" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
-        <v>1126</v>
+        <v>1157</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>1126</v>
+        <v>1157</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D49" s="7">
         <v>46064</v>
@@ -34224,22 +35414,22 @@
         <v>386</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>1125</v>
+        <v>1156</v>
       </c>
       <c r="J49" s="3" t="s">
-        <v>1124</v>
+        <v>1155</v>
       </c>
       <c r="K49" s="3" t="s">
         <v>446</v>
       </c>
       <c r="L49" s="3" t="s">
-        <v>1095</v>
+        <v>1126</v>
       </c>
       <c r="M49" s="3" t="s">
-        <v>1094</v>
+        <v>1125</v>
       </c>
       <c r="N49" s="3" t="s">
-        <v>1093</v>
+        <v>1124</v>
       </c>
       <c r="O49" s="8">
         <v>1000</v>
@@ -34272,7 +35462,7 @@
         <v>51</v>
       </c>
       <c r="Y49" s="3" t="s">
-        <v>1123</v>
+        <v>1154</v>
       </c>
       <c r="Z49" s="3" t="s">
         <v>0</v>
@@ -34310,13 +35500,13 @@
     </row>
     <row r="50" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
-        <v>1122</v>
+        <v>1153</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>1122</v>
+        <v>1153</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D50" s="4">
         <v>46066</v>
@@ -34328,10 +35518,10 @@
         <v>61</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>1121</v>
+        <v>1152</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>1120</v>
+        <v>1151</v>
       </c>
       <c r="I50" s="2" t="s">
         <v>163</v>
@@ -34343,13 +35533,13 @@
         <v>632</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>1119</v>
+        <v>1150</v>
       </c>
       <c r="M50" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N50" s="2" t="s">
-        <v>1118</v>
+        <v>1149</v>
       </c>
       <c r="O50" s="5">
         <v>507</v>
@@ -34382,7 +35572,7 @@
         <v>51</v>
       </c>
       <c r="Y50" s="2" t="s">
-        <v>1117</v>
+        <v>1148</v>
       </c>
       <c r="Z50" s="2" t="s">
         <v>0</v>
@@ -34420,13 +35610,13 @@
     </row>
     <row r="51" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
-        <v>1116</v>
+        <v>1147</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>1116</v>
+        <v>1147</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D51" s="7">
         <v>46071</v>
@@ -34450,16 +35640,16 @@
         <v>164</v>
       </c>
       <c r="K51" s="3" t="s">
-        <v>1054</v>
+        <v>1086</v>
       </c>
       <c r="L51" s="3" t="s">
-        <v>1115</v>
+        <v>1146</v>
       </c>
       <c r="M51" s="3" t="s">
-        <v>1114</v>
+        <v>1145</v>
       </c>
       <c r="N51" s="3" t="s">
-        <v>1113</v>
+        <v>1144</v>
       </c>
       <c r="O51" s="8">
         <v>500</v>
@@ -34492,7 +35682,7 @@
         <v>51</v>
       </c>
       <c r="Y51" s="3" t="s">
-        <v>1112</v>
+        <v>1143</v>
       </c>
       <c r="Z51" s="3" t="s">
         <v>0</v>
@@ -34507,10 +35697,10 @@
         <v>111</v>
       </c>
       <c r="AD51" s="3" t="s">
-        <v>1049</v>
+        <v>1081</v>
       </c>
       <c r="AE51" s="3" t="s">
-        <v>1048</v>
+        <v>1080</v>
       </c>
       <c r="AF51" s="3" t="s">
         <v>77</v>
@@ -34530,13 +35720,13 @@
     </row>
     <row r="52" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>1111</v>
+        <v>1142</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>1111</v>
+        <v>1142</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D52" s="4">
         <v>46071</v>
@@ -34548,10 +35738,10 @@
         <v>61</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>1110</v>
+        <v>1141</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>1109</v>
+        <v>1140</v>
       </c>
       <c r="I52" s="2" t="s">
         <v>139</v>
@@ -34563,13 +35753,13 @@
         <v>446</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>1095</v>
+        <v>1126</v>
       </c>
       <c r="M52" s="2" t="s">
-        <v>1094</v>
+        <v>1125</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>1093</v>
+        <v>1124</v>
       </c>
       <c r="O52" s="5">
         <v>200</v>
@@ -34602,7 +35792,7 @@
         <v>51</v>
       </c>
       <c r="Y52" s="2" t="s">
-        <v>1108</v>
+        <v>1139</v>
       </c>
       <c r="Z52" s="2" t="s">
         <v>0</v>
@@ -34640,13 +35830,13 @@
     </row>
     <row r="53" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
-        <v>1107</v>
+        <v>1138</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>1107</v>
+        <v>1138</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D53" s="7">
         <v>46072</v>
@@ -34658,10 +35848,10 @@
         <v>40</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>1038</v>
+        <v>1070</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>1037</v>
+        <v>1069</v>
       </c>
       <c r="I53" s="3" t="s">
         <v>43</v>
@@ -34673,13 +35863,13 @@
         <v>440</v>
       </c>
       <c r="L53" s="3" t="s">
-        <v>1106</v>
+        <v>1137</v>
       </c>
       <c r="M53" s="3" t="s">
-        <v>1105</v>
+        <v>1136</v>
       </c>
       <c r="N53" s="3" t="s">
-        <v>1104</v>
+        <v>1135</v>
       </c>
       <c r="O53" s="8">
         <v>50</v>
@@ -34703,16 +35893,16 @@
         <v>0</v>
       </c>
       <c r="V53" s="3" t="s">
-        <v>1103</v>
+        <v>1134</v>
       </c>
       <c r="W53" s="3" t="s">
-        <v>1102</v>
+        <v>1133</v>
       </c>
       <c r="X53" s="3" t="s">
         <v>51</v>
       </c>
       <c r="Y53" s="3" t="s">
-        <v>1101</v>
+        <v>1132</v>
       </c>
       <c r="Z53" s="3" t="s">
         <v>0</v>
@@ -34750,13 +35940,13 @@
     </row>
     <row r="54" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>1100</v>
+        <v>1131</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>1100</v>
+        <v>1131</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D54" s="4">
         <v>46072</v>
@@ -34768,10 +35958,10 @@
         <v>61</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>1090</v>
+        <v>1121</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>1089</v>
+        <v>1120</v>
       </c>
       <c r="I54" s="2" t="s">
         <v>163</v>
@@ -34783,13 +35973,13 @@
         <v>417</v>
       </c>
       <c r="L54" s="2" t="s">
-        <v>1075</v>
+        <v>1106</v>
       </c>
       <c r="M54" s="2" t="s">
-        <v>1074</v>
+        <v>1105</v>
       </c>
       <c r="N54" s="2" t="s">
-        <v>1073</v>
+        <v>1104</v>
       </c>
       <c r="O54" s="5">
         <v>1600</v>
@@ -34822,7 +36012,7 @@
         <v>51</v>
       </c>
       <c r="Y54" s="2" t="s">
-        <v>1099</v>
+        <v>1130</v>
       </c>
       <c r="Z54" s="2" t="s">
         <v>0</v>
@@ -34860,13 +36050,13 @@
     </row>
     <row r="55" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
-        <v>1098</v>
+        <v>1129</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>1098</v>
+        <v>1129</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D55" s="7">
         <v>46072</v>
@@ -34878,10 +36068,10 @@
         <v>40</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>1097</v>
+        <v>1128</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>1096</v>
+        <v>1127</v>
       </c>
       <c r="I55" s="3" t="s">
         <v>43</v>
@@ -34893,13 +36083,13 @@
         <v>446</v>
       </c>
       <c r="L55" s="3" t="s">
-        <v>1095</v>
+        <v>1126</v>
       </c>
       <c r="M55" s="3" t="s">
-        <v>1094</v>
+        <v>1125</v>
       </c>
       <c r="N55" s="3" t="s">
-        <v>1093</v>
+        <v>1124</v>
       </c>
       <c r="O55" s="8">
         <v>500</v>
@@ -34932,7 +36122,7 @@
         <v>51</v>
       </c>
       <c r="Y55" s="3" t="s">
-        <v>1092</v>
+        <v>1123</v>
       </c>
       <c r="Z55" s="3" t="s">
         <v>0</v>
@@ -34970,13 +36160,13 @@
     </row>
     <row r="56" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
-        <v>1091</v>
+        <v>1122</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>1091</v>
+        <v>1122</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D56" s="4">
         <v>46076</v>
@@ -34988,10 +36178,10 @@
         <v>61</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>1090</v>
+        <v>1121</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>1089</v>
+        <v>1120</v>
       </c>
       <c r="I56" s="2" t="s">
         <v>163</v>
@@ -35003,13 +36193,13 @@
         <v>417</v>
       </c>
       <c r="L56" s="2" t="s">
-        <v>1075</v>
+        <v>1106</v>
       </c>
       <c r="M56" s="2" t="s">
-        <v>1074</v>
+        <v>1105</v>
       </c>
       <c r="N56" s="2" t="s">
-        <v>1073</v>
+        <v>1104</v>
       </c>
       <c r="O56" s="5">
         <v>1700</v>
@@ -35042,7 +36232,7 @@
         <v>51</v>
       </c>
       <c r="Y56" s="2" t="s">
-        <v>1088</v>
+        <v>1119</v>
       </c>
       <c r="Z56" s="2" t="s">
         <v>0</v>
@@ -35080,13 +36270,13 @@
     </row>
     <row r="57" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
-        <v>1085</v>
+        <v>1116</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>1085</v>
+        <v>1116</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D57" s="7">
         <v>46077</v>
@@ -35110,16 +36300,16 @@
         <v>164</v>
       </c>
       <c r="K57" s="3" t="s">
-        <v>1059</v>
+        <v>1091</v>
       </c>
       <c r="L57" s="3" t="s">
-        <v>1087</v>
+        <v>1118</v>
       </c>
       <c r="M57" s="3" t="s">
-        <v>1086</v>
+        <v>1117</v>
       </c>
       <c r="N57" s="3" t="s">
-        <v>1056</v>
+        <v>1088</v>
       </c>
       <c r="O57" s="8">
         <v>500</v>
@@ -35152,7 +36342,7 @@
         <v>51</v>
       </c>
       <c r="Y57" s="3" t="s">
-        <v>1084</v>
+        <v>1115</v>
       </c>
       <c r="Z57" s="3" t="s">
         <v>0</v>
@@ -35190,13 +36380,13 @@
     </row>
     <row r="58" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
-        <v>1085</v>
+        <v>1116</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>1085</v>
+        <v>1116</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D58" s="4">
         <v>46077</v>
@@ -35220,16 +36410,16 @@
         <v>164</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>1054</v>
+        <v>1086</v>
       </c>
       <c r="L58" s="2" t="s">
-        <v>1053</v>
+        <v>1085</v>
       </c>
       <c r="M58" s="2" t="s">
-        <v>1052</v>
+        <v>1084</v>
       </c>
       <c r="N58" s="2" t="s">
-        <v>1051</v>
+        <v>1083</v>
       </c>
       <c r="O58" s="5">
         <v>500</v>
@@ -35262,7 +36452,7 @@
         <v>51</v>
       </c>
       <c r="Y58" s="2" t="s">
-        <v>1084</v>
+        <v>1115</v>
       </c>
       <c r="Z58" s="2" t="s">
         <v>0</v>
@@ -35277,10 +36467,10 @@
         <v>111</v>
       </c>
       <c r="AD58" s="2" t="s">
-        <v>1049</v>
+        <v>1081</v>
       </c>
       <c r="AE58" s="2" t="s">
-        <v>1048</v>
+        <v>1080</v>
       </c>
       <c r="AF58" s="2" t="s">
         <v>77</v>
@@ -35300,13 +36490,13 @@
     </row>
     <row r="59" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
-        <v>1083</v>
+        <v>1114</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>1083</v>
+        <v>1114</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D59" s="7">
         <v>46078</v>
@@ -35318,10 +36508,10 @@
         <v>40</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>1082</v>
+        <v>1113</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>1081</v>
+        <v>1112</v>
       </c>
       <c r="I59" s="3" t="s">
         <v>139</v>
@@ -35333,13 +36523,13 @@
         <v>784</v>
       </c>
       <c r="L59" s="3" t="s">
-        <v>1080</v>
+        <v>1111</v>
       </c>
       <c r="M59" s="3" t="s">
-        <v>1079</v>
+        <v>1110</v>
       </c>
       <c r="N59" s="3" t="s">
-        <v>1078</v>
+        <v>1109</v>
       </c>
       <c r="O59" s="8">
         <v>225</v>
@@ -35372,7 +36562,7 @@
         <v>51</v>
       </c>
       <c r="Y59" s="3" t="s">
-        <v>1077</v>
+        <v>1108</v>
       </c>
       <c r="Z59" s="3" t="s">
         <v>0</v>
@@ -35410,13 +36600,13 @@
     </row>
     <row r="60" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
-        <v>1076</v>
+        <v>1107</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>1076</v>
+        <v>1107</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D60" s="4">
         <v>46079</v>
@@ -35443,13 +36633,13 @@
         <v>417</v>
       </c>
       <c r="L60" s="2" t="s">
-        <v>1075</v>
+        <v>1106</v>
       </c>
       <c r="M60" s="2" t="s">
-        <v>1074</v>
+        <v>1105</v>
       </c>
       <c r="N60" s="2" t="s">
-        <v>1073</v>
+        <v>1104</v>
       </c>
       <c r="O60" s="5">
         <v>5000</v>
@@ -35473,16 +36663,16 @@
         <v>2354</v>
       </c>
       <c r="V60" s="2" t="s">
-        <v>1072</v>
+        <v>1103</v>
       </c>
       <c r="W60" s="2" t="s">
-        <v>1071</v>
+        <v>1102</v>
       </c>
       <c r="X60" s="2" t="s">
         <v>51</v>
       </c>
       <c r="Y60" s="2" t="s">
-        <v>1070</v>
+        <v>1101</v>
       </c>
       <c r="Z60" s="2" t="s">
         <v>0</v>
@@ -35520,13 +36710,13 @@
     </row>
     <row r="61" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
-        <v>1069</v>
+        <v>1100</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>1069</v>
+        <v>1100</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D61" s="7">
         <v>46079</v>
@@ -35550,16 +36740,16 @@
         <v>912</v>
       </c>
       <c r="K61" s="3" t="s">
-        <v>1068</v>
+        <v>1060</v>
       </c>
       <c r="L61" s="3" t="s">
-        <v>1067</v>
+        <v>1099</v>
       </c>
       <c r="M61" s="3" t="s">
-        <v>1066</v>
+        <v>1098</v>
       </c>
       <c r="N61" s="3" t="s">
-        <v>1065</v>
+        <v>1097</v>
       </c>
       <c r="O61" s="8">
         <v>12000</v>
@@ -35592,7 +36782,7 @@
         <v>51</v>
       </c>
       <c r="Y61" s="3" t="s">
-        <v>1064</v>
+        <v>1096</v>
       </c>
       <c r="Z61" s="3" t="s">
         <v>0</v>
@@ -35630,13 +36820,13 @@
     </row>
     <row r="62" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
-        <v>1063</v>
+        <v>1095</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>1063</v>
+        <v>1095</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D62" s="4">
         <v>46085</v>
@@ -35663,13 +36853,13 @@
         <v>633</v>
       </c>
       <c r="L62" s="2" t="s">
-        <v>1062</v>
+        <v>1094</v>
       </c>
       <c r="M62" s="2" t="s">
         <v>652</v>
       </c>
       <c r="N62" s="2" t="s">
-        <v>1061</v>
+        <v>1093</v>
       </c>
       <c r="O62" s="5">
         <v>5005</v>
@@ -35702,7 +36892,7 @@
         <v>51</v>
       </c>
       <c r="Y62" s="2" t="s">
-        <v>1060</v>
+        <v>1092</v>
       </c>
       <c r="Z62" s="2" t="s">
         <v>0</v>
@@ -35740,13 +36930,13 @@
     </row>
     <row r="63" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
-        <v>1055</v>
+        <v>1087</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>1055</v>
+        <v>1087</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D63" s="7">
         <v>46085</v>
@@ -35770,16 +36960,16 @@
         <v>164</v>
       </c>
       <c r="K63" s="3" t="s">
-        <v>1059</v>
+        <v>1091</v>
       </c>
       <c r="L63" s="3" t="s">
-        <v>1058</v>
+        <v>1090</v>
       </c>
       <c r="M63" s="3" t="s">
-        <v>1057</v>
+        <v>1089</v>
       </c>
       <c r="N63" s="3" t="s">
-        <v>1056</v>
+        <v>1088</v>
       </c>
       <c r="O63" s="8">
         <v>500</v>
@@ -35812,7 +37002,7 @@
         <v>51</v>
       </c>
       <c r="Y63" s="3" t="s">
-        <v>1050</v>
+        <v>1082</v>
       </c>
       <c r="Z63" s="3" t="s">
         <v>0</v>
@@ -35850,13 +37040,13 @@
     </row>
     <row r="64" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
-        <v>1055</v>
+        <v>1087</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>1055</v>
+        <v>1087</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D64" s="4">
         <v>46085</v>
@@ -35880,16 +37070,16 @@
         <v>164</v>
       </c>
       <c r="K64" s="2" t="s">
-        <v>1054</v>
+        <v>1086</v>
       </c>
       <c r="L64" s="2" t="s">
-        <v>1053</v>
+        <v>1085</v>
       </c>
       <c r="M64" s="2" t="s">
-        <v>1052</v>
+        <v>1084</v>
       </c>
       <c r="N64" s="2" t="s">
-        <v>1051</v>
+        <v>1083</v>
       </c>
       <c r="O64" s="5">
         <v>500</v>
@@ -35922,7 +37112,7 @@
         <v>51</v>
       </c>
       <c r="Y64" s="2" t="s">
-        <v>1050</v>
+        <v>1082</v>
       </c>
       <c r="Z64" s="2" t="s">
         <v>0</v>
@@ -35937,10 +37127,10 @@
         <v>111</v>
       </c>
       <c r="AD64" s="2" t="s">
-        <v>1049</v>
+        <v>1081</v>
       </c>
       <c r="AE64" s="2" t="s">
-        <v>1048</v>
+        <v>1080</v>
       </c>
       <c r="AF64" s="2" t="s">
         <v>77</v>
@@ -35960,13 +37150,13 @@
     </row>
     <row r="65" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
-        <v>1047</v>
+        <v>1079</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>1047</v>
+        <v>1079</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D65" s="7">
         <v>46085</v>
@@ -35978,10 +37168,10 @@
         <v>40</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>1046</v>
+        <v>1078</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>1045</v>
+        <v>1077</v>
       </c>
       <c r="I65" s="3" t="s">
         <v>163</v>
@@ -35993,13 +37183,13 @@
         <v>154</v>
       </c>
       <c r="L65" s="3" t="s">
-        <v>1044</v>
+        <v>1076</v>
       </c>
       <c r="M65" s="3" t="s">
-        <v>1043</v>
+        <v>1075</v>
       </c>
       <c r="N65" s="3" t="s">
-        <v>1042</v>
+        <v>1074</v>
       </c>
       <c r="O65" s="8">
         <v>3700</v>
@@ -36032,7 +37222,7 @@
         <v>51</v>
       </c>
       <c r="Y65" s="3" t="s">
-        <v>1041</v>
+        <v>1073</v>
       </c>
       <c r="Z65" s="3" t="s">
         <v>0</v>
@@ -36070,13 +37260,13 @@
     </row>
     <row r="66" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
-        <v>1040</v>
+        <v>1072</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>1040</v>
+        <v>1072</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>1039</v>
+        <v>1071</v>
       </c>
       <c r="D66" s="4">
         <v>46085</v>
@@ -36088,10 +37278,10 @@
         <v>40</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>1038</v>
+        <v>1070</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>1037</v>
+        <v>1069</v>
       </c>
       <c r="I66" s="2" t="s">
         <v>139</v>
@@ -36100,7 +37290,7 @@
         <v>140</v>
       </c>
       <c r="K66" s="2" t="s">
-        <v>1036</v>
+        <v>1068</v>
       </c>
       <c r="L66" s="2" t="s">
         <v>0</v>
@@ -36142,7 +37332,7 @@
         <v>0</v>
       </c>
       <c r="Y66" s="2" t="s">
-        <v>1035</v>
+        <v>1067</v>
       </c>
       <c r="Z66" s="2" t="s">
         <v>0</v>
@@ -36157,10 +37347,10 @@
         <v>298</v>
       </c>
       <c r="AD66" s="2" t="s">
-        <v>1034</v>
+        <v>1066</v>
       </c>
       <c r="AE66" s="2" t="s">
-        <v>1033</v>
+        <v>1065</v>
       </c>
       <c r="AF66" s="2" t="s">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização da base de dados 10.03.2026
</commit_message>
<xml_diff>
--- a/BASE_KEMPARTS.xlsx
+++ b/BASE_KEMPARTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dash_kp_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CCDF60A6-0241-4C84-A5C9-0B6398B4F075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{97583B37-DC83-4DD0-9F4C-6CDFE6B33DC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{6FEA2588-5565-4B12-8C5E-E6FBB7E9CDF0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{CB469FB5-CC63-49DF-8F0A-CC2C928DC074}"/>
   </bookViews>
   <sheets>
     <sheet name="FSP" sheetId="3" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7397" uniqueCount="1288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7547" uniqueCount="1305">
   <si>
     <t/>
   </si>
@@ -3218,6 +3218,84 @@
     <t>153266</t>
   </si>
   <si>
+    <t>000015547</t>
+  </si>
+  <si>
+    <t>173837</t>
+  </si>
+  <si>
+    <t>000015548</t>
+  </si>
+  <si>
+    <t>C00113</t>
+  </si>
+  <si>
+    <t>EVERCOL INDUSTRIA E COMERCIO LTDA</t>
+  </si>
+  <si>
+    <t>173818</t>
+  </si>
+  <si>
+    <t>000015551</t>
+  </si>
+  <si>
+    <t>TRAN.24.004.10.24081025</t>
+  </si>
+  <si>
+    <t>24081025</t>
+  </si>
+  <si>
+    <t>TRAN.24.004.10.</t>
+  </si>
+  <si>
+    <t>153309</t>
+  </si>
+  <si>
+    <t>003301</t>
+  </si>
+  <si>
+    <t>2024.357.03.</t>
+  </si>
+  <si>
+    <t>240707</t>
+  </si>
+  <si>
+    <t>2024.357.03.240707</t>
+  </si>
+  <si>
+    <t>ALV INDUSTRIA E COMERCIO DE TINTAS LTDA</t>
+  </si>
+  <si>
+    <t>C00341</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>000002510</t>
+  </si>
+  <si>
+    <t>003293</t>
+  </si>
+  <si>
+    <t>TRANSPORTADORA NIMEC LT</t>
+  </si>
+  <si>
+    <t>T00213</t>
+  </si>
+  <si>
+    <t>2025.004.01.</t>
+  </si>
+  <si>
+    <t>25021048</t>
+  </si>
+  <si>
+    <t>2025.004.01.25021048</t>
+  </si>
+  <si>
+    <t>000002509</t>
+  </si>
+  <si>
     <t>GASTOS GERAIS</t>
   </si>
   <si>
@@ -3236,9 +3314,6 @@
     <t>C00591</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>000002508</t>
   </si>
   <si>
@@ -3329,15 +3404,6 @@
     <t>003169</t>
   </si>
   <si>
-    <t>TRANSPORTADORA NIMEC LT</t>
-  </si>
-  <si>
-    <t>T00213</t>
-  </si>
-  <si>
-    <t>2025.004.01.</t>
-  </si>
-  <si>
     <t>25021046</t>
   </si>
   <si>
@@ -3348,21 +3414,6 @@
   </si>
   <si>
     <t>003283</t>
-  </si>
-  <si>
-    <t>2024.357.03.</t>
-  </si>
-  <si>
-    <t>240707</t>
-  </si>
-  <si>
-    <t>2024.357.03.240707</t>
-  </si>
-  <si>
-    <t>ALV INDUSTRIA E COMERCIO DE TINTAS LTDA</t>
-  </si>
-  <si>
-    <t>C00341</t>
   </si>
   <si>
     <t>000002498</t>
@@ -4831,8 +4882,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{318A57C2-A3D9-48EA-BD6D-8BF7B0CE2ED1}">
-  <dimension ref="A1:AJ229"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B26A77ED-7CEE-4E89-8BE8-34DC8758E529}">
+  <dimension ref="A1:AJ233"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
@@ -30062,14 +30113,454 @@
         <v>9.8148</v>
       </c>
     </row>
+    <row r="230" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A230" s="2" t="s">
+        <v>1065</v>
+      </c>
+      <c r="B230" s="2" t="s">
+        <v>1065</v>
+      </c>
+      <c r="C230" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D230" s="4">
+        <v>46091</v>
+      </c>
+      <c r="E230" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F230" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G230" s="2" t="s">
+        <v>593</v>
+      </c>
+      <c r="H230" s="2" t="s">
+        <v>594</v>
+      </c>
+      <c r="I230" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="J230" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="K230" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="L230" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="M230" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="N230" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="O230" s="5">
+        <v>1000</v>
+      </c>
+      <c r="P230" s="5">
+        <v>25.2</v>
+      </c>
+      <c r="Q230" s="6">
+        <v>25200</v>
+      </c>
+      <c r="R230" s="6">
+        <v>819</v>
+      </c>
+      <c r="S230" s="6">
+        <v>26019</v>
+      </c>
+      <c r="T230" s="6">
+        <v>25200</v>
+      </c>
+      <c r="U230" s="6">
+        <v>4536</v>
+      </c>
+      <c r="V230" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="W230" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="X230" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y230" s="2" t="s">
+        <v>1066</v>
+      </c>
+      <c r="Z230" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA230" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB230" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="AC230" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD230" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="AE230" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="AF230" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AG230" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH230" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI230" s="6">
+        <v>18</v>
+      </c>
+      <c r="AJ230" s="5">
+        <v>7503.57</v>
+      </c>
+    </row>
+    <row r="231" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A231" s="3" t="s">
+        <v>1067</v>
+      </c>
+      <c r="B231" s="3" t="s">
+        <v>1067</v>
+      </c>
+      <c r="C231" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D231" s="7">
+        <v>46091</v>
+      </c>
+      <c r="E231" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F231" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G231" s="3" t="s">
+        <v>1068</v>
+      </c>
+      <c r="H231" s="3" t="s">
+        <v>1069</v>
+      </c>
+      <c r="I231" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J231" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="K231" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="L231" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="M231" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="N231" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="O231" s="8">
+        <v>1700</v>
+      </c>
+      <c r="P231" s="8">
+        <v>22.98</v>
+      </c>
+      <c r="Q231" s="9">
+        <v>39066</v>
+      </c>
+      <c r="R231" s="9">
+        <v>1269.6500000000001</v>
+      </c>
+      <c r="S231" s="9">
+        <v>40335.65</v>
+      </c>
+      <c r="T231" s="9">
+        <v>39066</v>
+      </c>
+      <c r="U231" s="9">
+        <v>7031.88</v>
+      </c>
+      <c r="V231" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="W231" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="X231" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y231" s="3" t="s">
+        <v>1070</v>
+      </c>
+      <c r="Z231" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA231" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB231" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC231" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD231" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE231" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="AF231" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="AG231" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH231" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI231" s="9">
+        <v>18</v>
+      </c>
+      <c r="AJ231" s="8">
+        <v>19786.912</v>
+      </c>
+    </row>
+    <row r="232" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A232" s="2" t="s">
+        <v>1071</v>
+      </c>
+      <c r="B232" s="2" t="s">
+        <v>1071</v>
+      </c>
+      <c r="C232" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D232" s="4">
+        <v>46091</v>
+      </c>
+      <c r="E232" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="F232" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="G232" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="H232" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="I232" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="J232" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="K232" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="L232" s="2" t="s">
+        <v>1072</v>
+      </c>
+      <c r="M232" s="2" t="s">
+        <v>1073</v>
+      </c>
+      <c r="N232" s="2" t="s">
+        <v>1074</v>
+      </c>
+      <c r="O232" s="5">
+        <v>1</v>
+      </c>
+      <c r="P232" s="5">
+        <v>10</v>
+      </c>
+      <c r="Q232" s="6">
+        <v>10</v>
+      </c>
+      <c r="R232" s="6">
+        <v>0</v>
+      </c>
+      <c r="S232" s="6">
+        <v>10</v>
+      </c>
+      <c r="T232" s="6">
+        <v>0</v>
+      </c>
+      <c r="U232" s="6">
+        <v>0</v>
+      </c>
+      <c r="V232" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="W232" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="X232" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y232" s="2" t="s">
+        <v>1075</v>
+      </c>
+      <c r="Z232" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA232" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB232" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC232" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD232" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="AE232" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="AF232" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="AG232" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH232" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI232" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ232" s="5">
+        <v>9.8976000000000006</v>
+      </c>
+    </row>
+    <row r="233" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A233" s="3" t="s">
+        <v>1071</v>
+      </c>
+      <c r="B233" s="3" t="s">
+        <v>1071</v>
+      </c>
+      <c r="C233" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D233" s="7">
+        <v>46091</v>
+      </c>
+      <c r="E233" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="F233" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="G233" s="3" t="s">
+        <v>622</v>
+      </c>
+      <c r="H233" s="3" t="s">
+        <v>623</v>
+      </c>
+      <c r="I233" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="J233" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="K233" s="3" t="s">
+        <v>631</v>
+      </c>
+      <c r="L233" s="3" t="s">
+        <v>703</v>
+      </c>
+      <c r="M233" s="3" t="s">
+        <v>704</v>
+      </c>
+      <c r="N233" s="3" t="s">
+        <v>705</v>
+      </c>
+      <c r="O233" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="P233" s="8">
+        <v>10</v>
+      </c>
+      <c r="Q233" s="9">
+        <v>5</v>
+      </c>
+      <c r="R233" s="9">
+        <v>0</v>
+      </c>
+      <c r="S233" s="9">
+        <v>5</v>
+      </c>
+      <c r="T233" s="9">
+        <v>0</v>
+      </c>
+      <c r="U233" s="9">
+        <v>0</v>
+      </c>
+      <c r="V233" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="W233" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="X233" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y233" s="3" t="s">
+        <v>1075</v>
+      </c>
+      <c r="Z233" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA233" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB233" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC233" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD233" s="3" t="s">
+        <v>517</v>
+      </c>
+      <c r="AE233" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="AF233" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="AG233" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH233" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI233" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ233" s="8">
+        <v>9.8208099999999998</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11535412-83B7-4F7D-A32C-87312564DCEE}">
-  <dimension ref="A1:AJ66"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49746817-01A4-4A9C-9061-C45AA702B917}">
+  <dimension ref="A1:AJ68"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
@@ -30220,13 +30711,13 @@
     </row>
     <row r="2" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>1287</v>
+        <v>1304</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>1287</v>
+        <v>1304</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D2" s="4">
         <v>46024</v>
@@ -30238,10 +30729,10 @@
         <v>40</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>1070</v>
+        <v>1096</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>1069</v>
+        <v>1095</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>43</v>
@@ -30253,13 +30744,13 @@
         <v>440</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>1137</v>
+        <v>1154</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>1136</v>
+        <v>1153</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>1135</v>
+        <v>1152</v>
       </c>
       <c r="O2" s="5">
         <v>50</v>
@@ -30283,16 +30774,16 @@
         <v>39.06</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>1134</v>
+        <v>1151</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>1133</v>
+        <v>1150</v>
       </c>
       <c r="X2" s="2" t="s">
         <v>51</v>
       </c>
       <c r="Y2" s="2" t="s">
-        <v>1286</v>
+        <v>1303</v>
       </c>
       <c r="Z2" s="2" t="s">
         <v>0</v>
@@ -30330,13 +30821,13 @@
     </row>
     <row r="3" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>1285</v>
+        <v>1302</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>1285</v>
+        <v>1302</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D3" s="7">
         <v>46027</v>
@@ -30348,10 +30839,10 @@
         <v>61</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>1152</v>
+        <v>1169</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>1151</v>
+        <v>1168</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>163</v>
@@ -30363,13 +30854,13 @@
         <v>632</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>1150</v>
+        <v>1167</v>
       </c>
       <c r="M3" s="3" t="s">
         <v>648</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>1149</v>
+        <v>1166</v>
       </c>
       <c r="O3" s="8">
         <v>1001</v>
@@ -30402,7 +30893,7 @@
         <v>51</v>
       </c>
       <c r="Y3" s="3" t="s">
-        <v>1284</v>
+        <v>1301</v>
       </c>
       <c r="Z3" s="3" t="s">
         <v>0</v>
@@ -30440,13 +30931,13 @@
     </row>
     <row r="4" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>1283</v>
+        <v>1300</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>1283</v>
+        <v>1300</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D4" s="4">
         <v>46027</v>
@@ -30458,10 +30949,10 @@
         <v>61</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>1282</v>
+        <v>1299</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>1281</v>
+        <v>1298</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>152</v>
@@ -30473,13 +30964,13 @@
         <v>342</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>1280</v>
+        <v>1297</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>1279</v>
+        <v>1296</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>1278</v>
+        <v>1295</v>
       </c>
       <c r="O4" s="5">
         <v>600</v>
@@ -30503,16 +30994,16 @@
         <v>355.68</v>
       </c>
       <c r="V4" s="2" t="s">
-        <v>1277</v>
+        <v>1294</v>
       </c>
       <c r="W4" s="2" t="s">
-        <v>1276</v>
+        <v>1293</v>
       </c>
       <c r="X4" s="2" t="s">
         <v>51</v>
       </c>
       <c r="Y4" s="2" t="s">
-        <v>1275</v>
+        <v>1292</v>
       </c>
       <c r="Z4" s="2" t="s">
         <v>0</v>
@@ -30550,13 +31041,13 @@
     </row>
     <row r="5" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>1274</v>
+        <v>1291</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1274</v>
+        <v>1291</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D5" s="7">
         <v>46029</v>
@@ -30568,10 +31059,10 @@
         <v>212</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>1193</v>
+        <v>1210</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>1192</v>
+        <v>1209</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>139</v>
@@ -30580,7 +31071,7 @@
         <v>140</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>1273</v>
+        <v>1290</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>0</v>
@@ -30622,7 +31113,7 @@
         <v>87</v>
       </c>
       <c r="Y5" s="3" t="s">
-        <v>1272</v>
+        <v>1289</v>
       </c>
       <c r="Z5" s="3" t="s">
         <v>0</v>
@@ -30660,13 +31151,13 @@
     </row>
     <row r="6" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>1274</v>
+        <v>1291</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1274</v>
+        <v>1291</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D6" s="4">
         <v>46029</v>
@@ -30678,10 +31169,10 @@
         <v>212</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>1193</v>
+        <v>1210</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>1192</v>
+        <v>1209</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>139</v>
@@ -30690,7 +31181,7 @@
         <v>140</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>1273</v>
+        <v>1290</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>0</v>
@@ -30732,7 +31223,7 @@
         <v>87</v>
       </c>
       <c r="Y6" s="2" t="s">
-        <v>1272</v>
+        <v>1289</v>
       </c>
       <c r="Z6" s="2" t="s">
         <v>0</v>
@@ -30770,13 +31261,13 @@
     </row>
     <row r="7" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>1271</v>
+        <v>1288</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1271</v>
+        <v>1288</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D7" s="7">
         <v>46029</v>
@@ -30794,22 +31285,22 @@
         <v>386</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>1156</v>
+        <v>1173</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>1155</v>
+        <v>1172</v>
       </c>
       <c r="K7" s="3" t="s">
         <v>1060</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>1270</v>
+        <v>1287</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>1269</v>
+        <v>1286</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>1268</v>
+        <v>1285</v>
       </c>
       <c r="O7" s="8">
         <v>1000</v>
@@ -30842,7 +31333,7 @@
         <v>51</v>
       </c>
       <c r="Y7" s="3" t="s">
-        <v>1267</v>
+        <v>1284</v>
       </c>
       <c r="Z7" s="3" t="s">
         <v>0</v>
@@ -30880,13 +31371,13 @@
     </row>
     <row r="8" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>1266</v>
+        <v>1283</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>1266</v>
+        <v>1283</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D8" s="4">
         <v>46036</v>
@@ -30898,10 +31389,10 @@
         <v>61</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>1152</v>
+        <v>1169</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>1151</v>
+        <v>1168</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>163</v>
@@ -30913,13 +31404,13 @@
         <v>632</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>1150</v>
+        <v>1167</v>
       </c>
       <c r="M8" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>1149</v>
+        <v>1166</v>
       </c>
       <c r="O8" s="5">
         <v>1001</v>
@@ -30952,7 +31443,7 @@
         <v>51</v>
       </c>
       <c r="Y8" s="2" t="s">
-        <v>1265</v>
+        <v>1282</v>
       </c>
       <c r="Z8" s="2" t="s">
         <v>0</v>
@@ -30990,13 +31481,13 @@
     </row>
     <row r="9" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
-        <v>1264</v>
+        <v>1281</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1264</v>
+        <v>1281</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D9" s="7">
         <v>46037</v>
@@ -31008,10 +31499,10 @@
         <v>61</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>1165</v>
+        <v>1182</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>1164</v>
+        <v>1181</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>163</v>
@@ -31023,13 +31514,13 @@
         <v>417</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>1263</v>
+        <v>1280</v>
       </c>
       <c r="M9" s="3" t="s">
         <v>1043</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>1161</v>
+        <v>1178</v>
       </c>
       <c r="O9" s="8">
         <v>1000</v>
@@ -31062,7 +31553,7 @@
         <v>51</v>
       </c>
       <c r="Y9" s="3" t="s">
-        <v>1262</v>
+        <v>1279</v>
       </c>
       <c r="Z9" s="3" t="s">
         <v>0</v>
@@ -31100,13 +31591,13 @@
     </row>
     <row r="10" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>1261</v>
+        <v>1278</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>1261</v>
+        <v>1278</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D10" s="4">
         <v>46037</v>
@@ -31118,10 +31609,10 @@
         <v>40</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>1113</v>
+        <v>1081</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>1112</v>
+        <v>1080</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>139</v>
@@ -31133,13 +31624,13 @@
         <v>784</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>1111</v>
+        <v>1079</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>1110</v>
+        <v>1078</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>1109</v>
+        <v>1077</v>
       </c>
       <c r="O10" s="5">
         <v>300</v>
@@ -31172,7 +31663,7 @@
         <v>51</v>
       </c>
       <c r="Y10" s="2" t="s">
-        <v>1260</v>
+        <v>1277</v>
       </c>
       <c r="Z10" s="2" t="s">
         <v>0</v>
@@ -31210,13 +31701,13 @@
     </row>
     <row r="11" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>1259</v>
+        <v>1276</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>1259</v>
+        <v>1276</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D11" s="7">
         <v>46037</v>
@@ -31228,10 +31719,10 @@
         <v>40</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>1203</v>
+        <v>1220</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>1202</v>
+        <v>1219</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>43</v>
@@ -31243,13 +31734,13 @@
         <v>300</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>1258</v>
+        <v>1275</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>1257</v>
+        <v>1274</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>1256</v>
+        <v>1273</v>
       </c>
       <c r="O11" s="8">
         <v>25</v>
@@ -31282,7 +31773,7 @@
         <v>51</v>
       </c>
       <c r="Y11" s="3" t="s">
-        <v>1255</v>
+        <v>1272</v>
       </c>
       <c r="Z11" s="3" t="s">
         <v>0</v>
@@ -31320,13 +31811,13 @@
     </row>
     <row r="12" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>1254</v>
+        <v>1271</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>1254</v>
+        <v>1271</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D12" s="4">
         <v>46041</v>
@@ -31338,10 +31829,10 @@
         <v>212</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>1193</v>
+        <v>1210</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>1192</v>
+        <v>1209</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>139</v>
@@ -31350,7 +31841,7 @@
         <v>140</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>1086</v>
+        <v>1111</v>
       </c>
       <c r="L12" s="2" t="s">
         <v>0</v>
@@ -31392,7 +31883,7 @@
         <v>87</v>
       </c>
       <c r="Y12" s="2" t="s">
-        <v>1253</v>
+        <v>1270</v>
       </c>
       <c r="Z12" s="2" t="s">
         <v>0</v>
@@ -31407,10 +31898,10 @@
         <v>55</v>
       </c>
       <c r="AD12" s="2" t="s">
-        <v>1081</v>
+        <v>1106</v>
       </c>
       <c r="AE12" s="2" t="s">
-        <v>1080</v>
+        <v>1105</v>
       </c>
       <c r="AF12" s="2" t="s">
         <v>442</v>
@@ -31430,13 +31921,13 @@
     </row>
     <row r="13" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>1252</v>
+        <v>1269</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>1252</v>
+        <v>1269</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D13" s="7">
         <v>46042</v>
@@ -31454,22 +31945,22 @@
         <v>386</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>1156</v>
+        <v>1173</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>1155</v>
+        <v>1172</v>
       </c>
       <c r="K13" s="3" t="s">
         <v>446</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>1159</v>
+        <v>1176</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>1158</v>
+        <v>1175</v>
       </c>
       <c r="N13" s="3" t="s">
-        <v>1124</v>
+        <v>1141</v>
       </c>
       <c r="O13" s="8">
         <v>2000</v>
@@ -31502,7 +31993,7 @@
         <v>51</v>
       </c>
       <c r="Y13" s="3" t="s">
-        <v>1251</v>
+        <v>1268</v>
       </c>
       <c r="Z13" s="3" t="s">
         <v>0</v>
@@ -31540,13 +32031,13 @@
     </row>
     <row r="14" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>1250</v>
+        <v>1267</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>1250</v>
+        <v>1267</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D14" s="4">
         <v>46042</v>
@@ -31570,16 +32061,16 @@
         <v>294</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>1086</v>
+        <v>1111</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>1218</v>
+        <v>1235</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>1217</v>
+        <v>1234</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>1083</v>
+        <v>1108</v>
       </c>
       <c r="O14" s="5">
         <v>6000</v>
@@ -31603,16 +32094,16 @@
         <v>12873.6</v>
       </c>
       <c r="V14" s="2" t="s">
-        <v>1249</v>
+        <v>1266</v>
       </c>
       <c r="W14" s="2" t="s">
-        <v>1248</v>
+        <v>1265</v>
       </c>
       <c r="X14" s="2" t="s">
         <v>51</v>
       </c>
       <c r="Y14" s="2" t="s">
-        <v>1247</v>
+        <v>1264</v>
       </c>
       <c r="Z14" s="2" t="s">
         <v>0</v>
@@ -31627,10 +32118,10 @@
         <v>298</v>
       </c>
       <c r="AD14" s="2" t="s">
-        <v>1081</v>
+        <v>1106</v>
       </c>
       <c r="AE14" s="2" t="s">
-        <v>1080</v>
+        <v>1105</v>
       </c>
       <c r="AF14" s="2" t="s">
         <v>77</v>
@@ -31650,13 +32141,13 @@
     </row>
     <row r="15" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>1246</v>
+        <v>1263</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>1246</v>
+        <v>1263</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D15" s="7">
         <v>46042</v>
@@ -31668,10 +32159,10 @@
         <v>212</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>1193</v>
+        <v>1210</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>1192</v>
+        <v>1209</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>139</v>
@@ -31722,7 +32213,7 @@
         <v>87</v>
       </c>
       <c r="Y15" s="3" t="s">
-        <v>1245</v>
+        <v>1262</v>
       </c>
       <c r="Z15" s="3" t="s">
         <v>0</v>
@@ -31743,7 +32234,7 @@
         <v>518</v>
       </c>
       <c r="AF15" s="3" t="s">
-        <v>1213</v>
+        <v>1230</v>
       </c>
       <c r="AG15" s="9">
         <v>0</v>
@@ -31760,13 +32251,13 @@
     </row>
     <row r="16" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>1246</v>
+        <v>1263</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>1246</v>
+        <v>1263</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D16" s="4">
         <v>46042</v>
@@ -31778,10 +32269,10 @@
         <v>212</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>1193</v>
+        <v>1210</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>1192</v>
+        <v>1209</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>139</v>
@@ -31832,7 +32323,7 @@
         <v>87</v>
       </c>
       <c r="Y16" s="2" t="s">
-        <v>1245</v>
+        <v>1262</v>
       </c>
       <c r="Z16" s="2" t="s">
         <v>0</v>
@@ -31853,7 +32344,7 @@
         <v>518</v>
       </c>
       <c r="AF16" s="2" t="s">
-        <v>1213</v>
+        <v>1230</v>
       </c>
       <c r="AG16" s="6">
         <v>0</v>
@@ -31870,13 +32361,13 @@
     </row>
     <row r="17" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
-        <v>1244</v>
+        <v>1261</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>1244</v>
+        <v>1261</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D17" s="7">
         <v>46043</v>
@@ -31903,13 +32394,13 @@
         <v>417</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>1163</v>
+        <v>1180</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>1162</v>
+        <v>1179</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>1161</v>
+        <v>1178</v>
       </c>
       <c r="O17" s="8">
         <v>1000</v>
@@ -31942,7 +32433,7 @@
         <v>51</v>
       </c>
       <c r="Y17" s="3" t="s">
-        <v>1243</v>
+        <v>1260</v>
       </c>
       <c r="Z17" s="3" t="s">
         <v>0</v>
@@ -31980,28 +32471,28 @@
     </row>
     <row r="18" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>1231</v>
+        <v>1248</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>1231</v>
+        <v>1248</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D18" s="4">
         <v>46045</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>1230</v>
+        <v>1247</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>1229</v>
+        <v>1246</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>1169</v>
+        <v>1186</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>1168</v>
+        <v>1185</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>139</v>
@@ -32013,13 +32504,13 @@
         <v>628</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>1242</v>
+        <v>1259</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>1241</v>
+        <v>1258</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>1240</v>
+        <v>1257</v>
       </c>
       <c r="O18" s="5">
         <v>2000</v>
@@ -32043,16 +32534,16 @@
         <v>0</v>
       </c>
       <c r="V18" s="2" t="s">
-        <v>1225</v>
+        <v>1242</v>
       </c>
       <c r="W18" s="2" t="s">
-        <v>1192</v>
+        <v>1209</v>
       </c>
       <c r="X18" s="2" t="s">
         <v>87</v>
       </c>
       <c r="Y18" s="2" t="s">
-        <v>1224</v>
+        <v>1241</v>
       </c>
       <c r="Z18" s="2" t="s">
         <v>0</v>
@@ -32090,28 +32581,28 @@
     </row>
     <row r="19" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
-        <v>1231</v>
+        <v>1248</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>1231</v>
+        <v>1248</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D19" s="7">
         <v>46045</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>1230</v>
+        <v>1247</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>1229</v>
+        <v>1246</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>1169</v>
+        <v>1186</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>1168</v>
+        <v>1185</v>
       </c>
       <c r="I19" s="3" t="s">
         <v>139</v>
@@ -32123,13 +32614,13 @@
         <v>631</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>1239</v>
+        <v>1256</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>1238</v>
+        <v>1255</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>1226</v>
+        <v>1243</v>
       </c>
       <c r="O19" s="8">
         <v>11725</v>
@@ -32153,16 +32644,16 @@
         <v>0</v>
       </c>
       <c r="V19" s="3" t="s">
-        <v>1225</v>
+        <v>1242</v>
       </c>
       <c r="W19" s="3" t="s">
-        <v>1192</v>
+        <v>1209</v>
       </c>
       <c r="X19" s="3" t="s">
         <v>87</v>
       </c>
       <c r="Y19" s="3" t="s">
-        <v>1224</v>
+        <v>1241</v>
       </c>
       <c r="Z19" s="3" t="s">
         <v>0</v>
@@ -32200,28 +32691,28 @@
     </row>
     <row r="20" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>1231</v>
+        <v>1248</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>1231</v>
+        <v>1248</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D20" s="4">
         <v>46045</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>1230</v>
+        <v>1247</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>1229</v>
+        <v>1246</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>1169</v>
+        <v>1186</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>1168</v>
+        <v>1185</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>139</v>
@@ -32233,13 +32724,13 @@
         <v>632</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>1150</v>
+        <v>1167</v>
       </c>
       <c r="M20" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>1149</v>
+        <v>1166</v>
       </c>
       <c r="O20" s="5">
         <v>2925</v>
@@ -32263,16 +32754,16 @@
         <v>0</v>
       </c>
       <c r="V20" s="2" t="s">
-        <v>1225</v>
+        <v>1242</v>
       </c>
       <c r="W20" s="2" t="s">
-        <v>1192</v>
+        <v>1209</v>
       </c>
       <c r="X20" s="2" t="s">
         <v>87</v>
       </c>
       <c r="Y20" s="2" t="s">
-        <v>1224</v>
+        <v>1241</v>
       </c>
       <c r="Z20" s="2" t="s">
         <v>0</v>
@@ -32310,28 +32801,28 @@
     </row>
     <row r="21" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
-        <v>1231</v>
+        <v>1248</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>1231</v>
+        <v>1248</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D21" s="7">
         <v>46045</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>1230</v>
+        <v>1247</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>1229</v>
+        <v>1246</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>1169</v>
+        <v>1186</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>1168</v>
+        <v>1185</v>
       </c>
       <c r="I21" s="3" t="s">
         <v>139</v>
@@ -32343,13 +32834,13 @@
         <v>633</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>1094</v>
+        <v>1119</v>
       </c>
       <c r="M21" s="3" t="s">
         <v>652</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>1093</v>
+        <v>1118</v>
       </c>
       <c r="O21" s="8">
         <v>2925</v>
@@ -32373,16 +32864,16 @@
         <v>0</v>
       </c>
       <c r="V21" s="3" t="s">
-        <v>1225</v>
+        <v>1242</v>
       </c>
       <c r="W21" s="3" t="s">
-        <v>1192</v>
+        <v>1209</v>
       </c>
       <c r="X21" s="3" t="s">
         <v>87</v>
       </c>
       <c r="Y21" s="3" t="s">
-        <v>1224</v>
+        <v>1241</v>
       </c>
       <c r="Z21" s="3" t="s">
         <v>0</v>
@@ -32420,28 +32911,28 @@
     </row>
     <row r="22" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>1231</v>
+        <v>1248</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>1231</v>
+        <v>1248</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D22" s="4">
         <v>46045</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>1230</v>
+        <v>1247</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>1229</v>
+        <v>1246</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>1169</v>
+        <v>1186</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>1168</v>
+        <v>1185</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>139</v>
@@ -32453,13 +32944,13 @@
         <v>465</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>1237</v>
+        <v>1254</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>1236</v>
+        <v>1253</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>1235</v>
+        <v>1252</v>
       </c>
       <c r="O22" s="5">
         <v>2400</v>
@@ -32483,16 +32974,16 @@
         <v>0</v>
       </c>
       <c r="V22" s="2" t="s">
-        <v>1225</v>
+        <v>1242</v>
       </c>
       <c r="W22" s="2" t="s">
-        <v>1192</v>
+        <v>1209</v>
       </c>
       <c r="X22" s="2" t="s">
         <v>87</v>
       </c>
       <c r="Y22" s="2" t="s">
-        <v>1224</v>
+        <v>1241</v>
       </c>
       <c r="Z22" s="2" t="s">
         <v>0</v>
@@ -32530,28 +33021,28 @@
     </row>
     <row r="23" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
-        <v>1231</v>
+        <v>1248</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>1231</v>
+        <v>1248</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D23" s="7">
         <v>46045</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>1230</v>
+        <v>1247</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>1229</v>
+        <v>1246</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>1169</v>
+        <v>1186</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>1168</v>
+        <v>1185</v>
       </c>
       <c r="I23" s="3" t="s">
         <v>139</v>
@@ -32563,13 +33054,13 @@
         <v>465</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>1234</v>
+        <v>1251</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>1233</v>
+        <v>1250</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>1232</v>
+        <v>1249</v>
       </c>
       <c r="O23" s="8">
         <v>1800</v>
@@ -32593,16 +33084,16 @@
         <v>0</v>
       </c>
       <c r="V23" s="3" t="s">
-        <v>1225</v>
+        <v>1242</v>
       </c>
       <c r="W23" s="3" t="s">
-        <v>1192</v>
+        <v>1209</v>
       </c>
       <c r="X23" s="3" t="s">
         <v>87</v>
       </c>
       <c r="Y23" s="3" t="s">
-        <v>1224</v>
+        <v>1241</v>
       </c>
       <c r="Z23" s="3" t="s">
         <v>0</v>
@@ -32640,28 +33131,28 @@
     </row>
     <row r="24" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>1231</v>
+        <v>1248</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>1231</v>
+        <v>1248</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D24" s="4">
         <v>46045</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>1230</v>
+        <v>1247</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>1229</v>
+        <v>1246</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>1169</v>
+        <v>1186</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>1168</v>
+        <v>1185</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>139</v>
@@ -32673,13 +33164,13 @@
         <v>634</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>1228</v>
+        <v>1245</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>1227</v>
+        <v>1244</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>1226</v>
+        <v>1243</v>
       </c>
       <c r="O24" s="5">
         <v>1400</v>
@@ -32703,16 +33194,16 @@
         <v>0</v>
       </c>
       <c r="V24" s="2" t="s">
-        <v>1225</v>
+        <v>1242</v>
       </c>
       <c r="W24" s="2" t="s">
-        <v>1192</v>
+        <v>1209</v>
       </c>
       <c r="X24" s="2" t="s">
         <v>87</v>
       </c>
       <c r="Y24" s="2" t="s">
-        <v>1224</v>
+        <v>1241</v>
       </c>
       <c r="Z24" s="2" t="s">
         <v>0</v>
@@ -32750,13 +33241,13 @@
     </row>
     <row r="25" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
-        <v>1223</v>
+        <v>1240</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>1223</v>
+        <v>1240</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D25" s="7">
         <v>46048</v>
@@ -32783,13 +33274,13 @@
         <v>417</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>1175</v>
+        <v>1192</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>1174</v>
+        <v>1191</v>
       </c>
       <c r="N25" s="3" t="s">
-        <v>1173</v>
+        <v>1190</v>
       </c>
       <c r="O25" s="8">
         <v>5000</v>
@@ -32813,16 +33304,16 @@
         <v>2354</v>
       </c>
       <c r="V25" s="3" t="s">
-        <v>1103</v>
+        <v>1086</v>
       </c>
       <c r="W25" s="3" t="s">
-        <v>1102</v>
+        <v>1085</v>
       </c>
       <c r="X25" s="3" t="s">
         <v>51</v>
       </c>
       <c r="Y25" s="3" t="s">
-        <v>1222</v>
+        <v>1239</v>
       </c>
       <c r="Z25" s="3" t="s">
         <v>0</v>
@@ -32860,13 +33351,13 @@
     </row>
     <row r="26" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>1221</v>
+        <v>1238</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>1221</v>
+        <v>1238</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D26" s="4">
         <v>46048</v>
@@ -32878,10 +33369,10 @@
         <v>40</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>1113</v>
+        <v>1081</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>1112</v>
+        <v>1080</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>139</v>
@@ -32893,13 +33384,13 @@
         <v>784</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>1111</v>
+        <v>1079</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>1110</v>
+        <v>1078</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>1109</v>
+        <v>1077</v>
       </c>
       <c r="O26" s="5">
         <v>300</v>
@@ -32932,7 +33423,7 @@
         <v>51</v>
       </c>
       <c r="Y26" s="2" t="s">
-        <v>1220</v>
+        <v>1237</v>
       </c>
       <c r="Z26" s="2" t="s">
         <v>0</v>
@@ -32970,13 +33461,13 @@
     </row>
     <row r="27" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
-        <v>1219</v>
+        <v>1236</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>1219</v>
+        <v>1236</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D27" s="7">
         <v>46048</v>
@@ -32988,10 +33479,10 @@
         <v>61</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>1152</v>
+        <v>1169</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>1151</v>
+        <v>1168</v>
       </c>
       <c r="I27" s="3" t="s">
         <v>163</v>
@@ -33003,13 +33494,13 @@
         <v>632</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>1150</v>
+        <v>1167</v>
       </c>
       <c r="M27" s="3" t="s">
         <v>648</v>
       </c>
       <c r="N27" s="3" t="s">
-        <v>1149</v>
+        <v>1166</v>
       </c>
       <c r="O27" s="8">
         <v>611</v>
@@ -33042,7 +33533,7 @@
         <v>51</v>
       </c>
       <c r="Y27" s="3" t="s">
-        <v>1216</v>
+        <v>1233</v>
       </c>
       <c r="Z27" s="3" t="s">
         <v>0</v>
@@ -33080,13 +33571,13 @@
     </row>
     <row r="28" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>1219</v>
+        <v>1236</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>1219</v>
+        <v>1236</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D28" s="4">
         <v>46048</v>
@@ -33098,10 +33589,10 @@
         <v>61</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>1152</v>
+        <v>1169</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>1151</v>
+        <v>1168</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>163</v>
@@ -33110,16 +33601,16 @@
         <v>164</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>1086</v>
+        <v>1111</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>1218</v>
+        <v>1235</v>
       </c>
       <c r="M28" s="2" t="s">
-        <v>1217</v>
+        <v>1234</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>1083</v>
+        <v>1108</v>
       </c>
       <c r="O28" s="5">
         <v>700</v>
@@ -33152,7 +33643,7 @@
         <v>51</v>
       </c>
       <c r="Y28" s="2" t="s">
-        <v>1216</v>
+        <v>1233</v>
       </c>
       <c r="Z28" s="2" t="s">
         <v>0</v>
@@ -33167,10 +33658,10 @@
         <v>55</v>
       </c>
       <c r="AD28" s="2" t="s">
-        <v>1081</v>
+        <v>1106</v>
       </c>
       <c r="AE28" s="2" t="s">
-        <v>1080</v>
+        <v>1105</v>
       </c>
       <c r="AF28" s="2" t="s">
         <v>77</v>
@@ -33190,13 +33681,13 @@
     </row>
     <row r="29" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
-        <v>1215</v>
+        <v>1232</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>1215</v>
+        <v>1232</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D29" s="7">
         <v>46048</v>
@@ -33208,10 +33699,10 @@
         <v>212</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>1193</v>
+        <v>1210</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>1192</v>
+        <v>1209</v>
       </c>
       <c r="I29" s="3" t="s">
         <v>139</v>
@@ -33262,7 +33753,7 @@
         <v>87</v>
       </c>
       <c r="Y29" s="3" t="s">
-        <v>1214</v>
+        <v>1231</v>
       </c>
       <c r="Z29" s="3" t="s">
         <v>0</v>
@@ -33283,7 +33774,7 @@
         <v>57</v>
       </c>
       <c r="AF29" s="3" t="s">
-        <v>1213</v>
+        <v>1230</v>
       </c>
       <c r="AG29" s="9">
         <v>0</v>
@@ -33300,13 +33791,13 @@
     </row>
     <row r="30" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>1212</v>
+        <v>1229</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>1212</v>
+        <v>1229</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D30" s="4">
         <v>46049</v>
@@ -33318,10 +33809,10 @@
         <v>212</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>1193</v>
+        <v>1210</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>1192</v>
+        <v>1209</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>139</v>
@@ -33372,7 +33863,7 @@
         <v>87</v>
       </c>
       <c r="Y30" s="2" t="s">
-        <v>1211</v>
+        <v>1228</v>
       </c>
       <c r="Z30" s="2" t="s">
         <v>0</v>
@@ -33410,13 +33901,13 @@
     </row>
     <row r="31" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
-        <v>1212</v>
+        <v>1229</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>1212</v>
+        <v>1229</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D31" s="7">
         <v>46049</v>
@@ -33428,10 +33919,10 @@
         <v>212</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>1193</v>
+        <v>1210</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>1192</v>
+        <v>1209</v>
       </c>
       <c r="I31" s="3" t="s">
         <v>139</v>
@@ -33482,7 +33973,7 @@
         <v>87</v>
       </c>
       <c r="Y31" s="3" t="s">
-        <v>1211</v>
+        <v>1228</v>
       </c>
       <c r="Z31" s="3" t="s">
         <v>0</v>
@@ -33520,13 +34011,13 @@
     </row>
     <row r="32" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>1208</v>
+        <v>1225</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>1208</v>
+        <v>1225</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D32" s="4">
         <v>46050</v>
@@ -33544,22 +34035,22 @@
         <v>386</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>1156</v>
+        <v>1173</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>1155</v>
+        <v>1172</v>
       </c>
       <c r="K32" s="2" t="s">
         <v>446</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>1210</v>
+        <v>1227</v>
       </c>
       <c r="M32" s="2" t="s">
         <v>448</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>1209</v>
+        <v>1226</v>
       </c>
       <c r="O32" s="5">
         <v>1000</v>
@@ -33592,7 +34083,7 @@
         <v>51</v>
       </c>
       <c r="Y32" s="2" t="s">
-        <v>1207</v>
+        <v>1224</v>
       </c>
       <c r="Z32" s="2" t="s">
         <v>0</v>
@@ -33630,13 +34121,13 @@
     </row>
     <row r="33" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
-        <v>1208</v>
+        <v>1225</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>1208</v>
+        <v>1225</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D33" s="7">
         <v>46050</v>
@@ -33654,22 +34145,22 @@
         <v>386</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>1156</v>
+        <v>1173</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>1155</v>
+        <v>1172</v>
       </c>
       <c r="K33" s="3" t="s">
         <v>446</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>1159</v>
+        <v>1176</v>
       </c>
       <c r="M33" s="3" t="s">
-        <v>1158</v>
+        <v>1175</v>
       </c>
       <c r="N33" s="3" t="s">
-        <v>1124</v>
+        <v>1141</v>
       </c>
       <c r="O33" s="8">
         <v>1000</v>
@@ -33702,7 +34193,7 @@
         <v>51</v>
       </c>
       <c r="Y33" s="3" t="s">
-        <v>1207</v>
+        <v>1224</v>
       </c>
       <c r="Z33" s="3" t="s">
         <v>0</v>
@@ -33740,13 +34231,13 @@
     </row>
     <row r="34" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>1206</v>
+        <v>1223</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>1206</v>
+        <v>1223</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D34" s="4">
         <v>46050</v>
@@ -33758,10 +34249,10 @@
         <v>212</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>1193</v>
+        <v>1210</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>1192</v>
+        <v>1209</v>
       </c>
       <c r="I34" s="2" t="s">
         <v>139</v>
@@ -33812,7 +34303,7 @@
         <v>87</v>
       </c>
       <c r="Y34" s="2" t="s">
-        <v>1205</v>
+        <v>1222</v>
       </c>
       <c r="Z34" s="2" t="s">
         <v>0</v>
@@ -33850,13 +34341,13 @@
     </row>
     <row r="35" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
-        <v>1204</v>
+        <v>1221</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>1204</v>
+        <v>1221</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D35" s="7">
         <v>46051</v>
@@ -33868,10 +34359,10 @@
         <v>40</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>1203</v>
+        <v>1220</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>1202</v>
+        <v>1219</v>
       </c>
       <c r="I35" s="3" t="s">
         <v>43</v>
@@ -33883,13 +34374,13 @@
         <v>632</v>
       </c>
       <c r="L35" s="3" t="s">
-        <v>1150</v>
+        <v>1167</v>
       </c>
       <c r="M35" s="3" t="s">
         <v>648</v>
       </c>
       <c r="N35" s="3" t="s">
-        <v>1149</v>
+        <v>1166</v>
       </c>
       <c r="O35" s="8">
         <v>26</v>
@@ -33922,7 +34413,7 @@
         <v>51</v>
       </c>
       <c r="Y35" s="3" t="s">
-        <v>1201</v>
+        <v>1218</v>
       </c>
       <c r="Z35" s="3" t="s">
         <v>0</v>
@@ -33960,13 +34451,13 @@
     </row>
     <row r="36" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>1200</v>
+        <v>1217</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>1200</v>
+        <v>1217</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D36" s="4">
         <v>46052</v>
@@ -33978,10 +34469,10 @@
         <v>61</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>1152</v>
+        <v>1169</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>1151</v>
+        <v>1168</v>
       </c>
       <c r="I36" s="2" t="s">
         <v>163</v>
@@ -33993,13 +34484,13 @@
         <v>632</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>1150</v>
+        <v>1167</v>
       </c>
       <c r="M36" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>1149</v>
+        <v>1166</v>
       </c>
       <c r="O36" s="5">
         <v>507</v>
@@ -34032,7 +34523,7 @@
         <v>51</v>
       </c>
       <c r="Y36" s="2" t="s">
-        <v>1199</v>
+        <v>1216</v>
       </c>
       <c r="Z36" s="2" t="s">
         <v>0</v>
@@ -34070,13 +34561,13 @@
     </row>
     <row r="37" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
-        <v>1198</v>
+        <v>1215</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>1198</v>
+        <v>1215</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D37" s="7">
         <v>46052</v>
@@ -34100,16 +34591,16 @@
         <v>164</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>1091</v>
+        <v>1116</v>
       </c>
       <c r="L37" s="3" t="s">
-        <v>1118</v>
+        <v>1135</v>
       </c>
       <c r="M37" s="3" t="s">
-        <v>1117</v>
+        <v>1134</v>
       </c>
       <c r="N37" s="3" t="s">
-        <v>1088</v>
+        <v>1113</v>
       </c>
       <c r="O37" s="8">
         <v>500</v>
@@ -34142,7 +34633,7 @@
         <v>51</v>
       </c>
       <c r="Y37" s="3" t="s">
-        <v>1197</v>
+        <v>1214</v>
       </c>
       <c r="Z37" s="3" t="s">
         <v>0</v>
@@ -34180,13 +34671,13 @@
     </row>
     <row r="38" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>1196</v>
+        <v>1213</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>1196</v>
+        <v>1213</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D38" s="4">
         <v>46052</v>
@@ -34198,10 +34689,10 @@
         <v>40</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>1113</v>
+        <v>1081</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>1112</v>
+        <v>1080</v>
       </c>
       <c r="I38" s="2" t="s">
         <v>139</v>
@@ -34213,13 +34704,13 @@
         <v>784</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>1111</v>
+        <v>1079</v>
       </c>
       <c r="M38" s="2" t="s">
-        <v>1110</v>
+        <v>1078</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>1109</v>
+        <v>1077</v>
       </c>
       <c r="O38" s="5">
         <v>300</v>
@@ -34252,7 +34743,7 @@
         <v>51</v>
       </c>
       <c r="Y38" s="2" t="s">
-        <v>1195</v>
+        <v>1212</v>
       </c>
       <c r="Z38" s="2" t="s">
         <v>0</v>
@@ -34290,13 +34781,13 @@
     </row>
     <row r="39" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
-        <v>1194</v>
+        <v>1211</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>1194</v>
+        <v>1211</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D39" s="7">
         <v>46055</v>
@@ -34308,10 +34799,10 @@
         <v>212</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>1193</v>
+        <v>1210</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>1192</v>
+        <v>1209</v>
       </c>
       <c r="I39" s="3" t="s">
         <v>139</v>
@@ -34320,7 +34811,7 @@
         <v>140</v>
       </c>
       <c r="K39" s="3" t="s">
-        <v>1191</v>
+        <v>1208</v>
       </c>
       <c r="L39" s="3" t="s">
         <v>0</v>
@@ -34362,7 +34853,7 @@
         <v>87</v>
       </c>
       <c r="Y39" s="3" t="s">
-        <v>1190</v>
+        <v>1207</v>
       </c>
       <c r="Z39" s="3" t="s">
         <v>0</v>
@@ -34400,13 +34891,13 @@
     </row>
     <row r="40" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>1189</v>
+        <v>1206</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>1189</v>
+        <v>1206</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D40" s="4">
         <v>46057</v>
@@ -34418,10 +34909,10 @@
         <v>61</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>1152</v>
+        <v>1169</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>1151</v>
+        <v>1168</v>
       </c>
       <c r="I40" s="2" t="s">
         <v>163</v>
@@ -34433,13 +34924,13 @@
         <v>632</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>1150</v>
+        <v>1167</v>
       </c>
       <c r="M40" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>1149</v>
+        <v>1166</v>
       </c>
       <c r="O40" s="5">
         <v>507</v>
@@ -34472,7 +34963,7 @@
         <v>51</v>
       </c>
       <c r="Y40" s="2" t="s">
-        <v>1188</v>
+        <v>1205</v>
       </c>
       <c r="Z40" s="2" t="s">
         <v>0</v>
@@ -34510,13 +35001,13 @@
     </row>
     <row r="41" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
-        <v>1187</v>
+        <v>1204</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>1187</v>
+        <v>1204</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D41" s="7">
         <v>46057</v>
@@ -34534,22 +35025,22 @@
         <v>386</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>1156</v>
+        <v>1173</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>1155</v>
+        <v>1172</v>
       </c>
       <c r="K41" s="3" t="s">
         <v>446</v>
       </c>
       <c r="L41" s="3" t="s">
-        <v>1159</v>
+        <v>1176</v>
       </c>
       <c r="M41" s="3" t="s">
-        <v>1158</v>
+        <v>1175</v>
       </c>
       <c r="N41" s="3" t="s">
-        <v>1124</v>
+        <v>1141</v>
       </c>
       <c r="O41" s="8">
         <v>2000</v>
@@ -34582,7 +35073,7 @@
         <v>51</v>
       </c>
       <c r="Y41" s="3" t="s">
-        <v>1154</v>
+        <v>1171</v>
       </c>
       <c r="Z41" s="3" t="s">
         <v>0</v>
@@ -34620,13 +35111,13 @@
     </row>
     <row r="42" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>1186</v>
+        <v>1203</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>1186</v>
+        <v>1203</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D42" s="4">
         <v>46058</v>
@@ -34638,10 +35129,10 @@
         <v>61</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>1152</v>
+        <v>1169</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>1151</v>
+        <v>1168</v>
       </c>
       <c r="I42" s="2" t="s">
         <v>163</v>
@@ -34653,13 +35144,13 @@
         <v>632</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>1150</v>
+        <v>1167</v>
       </c>
       <c r="M42" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>1149</v>
+        <v>1166</v>
       </c>
       <c r="O42" s="5">
         <v>507</v>
@@ -34692,7 +35183,7 @@
         <v>51</v>
       </c>
       <c r="Y42" s="2" t="s">
-        <v>1185</v>
+        <v>1202</v>
       </c>
       <c r="Z42" s="2" t="s">
         <v>0</v>
@@ -34730,13 +35221,13 @@
     </row>
     <row r="43" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
-        <v>1184</v>
+        <v>1201</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>1184</v>
+        <v>1201</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D43" s="7">
         <v>46058</v>
@@ -34748,10 +35239,10 @@
         <v>61</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>1121</v>
+        <v>1138</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>1120</v>
+        <v>1137</v>
       </c>
       <c r="I43" s="3" t="s">
         <v>163</v>
@@ -34763,13 +35254,13 @@
         <v>417</v>
       </c>
       <c r="L43" s="3" t="s">
-        <v>1175</v>
+        <v>1192</v>
       </c>
       <c r="M43" s="3" t="s">
-        <v>1174</v>
+        <v>1191</v>
       </c>
       <c r="N43" s="3" t="s">
-        <v>1173</v>
+        <v>1190</v>
       </c>
       <c r="O43" s="8">
         <v>1800</v>
@@ -34802,7 +35293,7 @@
         <v>51</v>
       </c>
       <c r="Y43" s="3" t="s">
-        <v>1183</v>
+        <v>1200</v>
       </c>
       <c r="Z43" s="3" t="s">
         <v>0</v>
@@ -34840,13 +35331,13 @@
     </row>
     <row r="44" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>1182</v>
+        <v>1199</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>1182</v>
+        <v>1199</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D44" s="4">
         <v>46059</v>
@@ -34858,10 +35349,10 @@
         <v>40</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>1181</v>
+        <v>1198</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>1180</v>
+        <v>1197</v>
       </c>
       <c r="I44" s="2" t="s">
         <v>43</v>
@@ -34873,13 +35364,13 @@
         <v>784</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>1111</v>
+        <v>1079</v>
       </c>
       <c r="M44" s="2" t="s">
-        <v>1110</v>
+        <v>1078</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>1109</v>
+        <v>1077</v>
       </c>
       <c r="O44" s="5">
         <v>500</v>
@@ -34912,7 +35403,7 @@
         <v>51</v>
       </c>
       <c r="Y44" s="2" t="s">
-        <v>1179</v>
+        <v>1196</v>
       </c>
       <c r="Z44" s="2" t="s">
         <v>0</v>
@@ -34950,13 +35441,13 @@
     </row>
     <row r="45" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="3" t="s">
-        <v>1178</v>
+        <v>1195</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>1178</v>
+        <v>1195</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D45" s="7">
         <v>46059</v>
@@ -34968,10 +35459,10 @@
         <v>40</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>1177</v>
+        <v>1194</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>1176</v>
+        <v>1193</v>
       </c>
       <c r="I45" s="3" t="s">
         <v>43</v>
@@ -34983,13 +35474,13 @@
         <v>417</v>
       </c>
       <c r="L45" s="3" t="s">
-        <v>1175</v>
+        <v>1192</v>
       </c>
       <c r="M45" s="3" t="s">
-        <v>1174</v>
+        <v>1191</v>
       </c>
       <c r="N45" s="3" t="s">
-        <v>1173</v>
+        <v>1190</v>
       </c>
       <c r="O45" s="8">
         <v>200</v>
@@ -35022,7 +35513,7 @@
         <v>51</v>
       </c>
       <c r="Y45" s="3" t="s">
-        <v>1172</v>
+        <v>1189</v>
       </c>
       <c r="Z45" s="3" t="s">
         <v>0</v>
@@ -35060,28 +35551,28 @@
     </row>
     <row r="46" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
-        <v>1171</v>
+        <v>1188</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>1171</v>
+        <v>1188</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D46" s="4">
         <v>46063</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>1170</v>
+        <v>1187</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>267</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>1169</v>
+        <v>1186</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>1168</v>
+        <v>1185</v>
       </c>
       <c r="I46" s="2" t="s">
         <v>139</v>
@@ -35090,7 +35581,7 @@
         <v>140</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>1068</v>
+        <v>1094</v>
       </c>
       <c r="L46" s="2" t="s">
         <v>0</v>
@@ -35132,7 +35623,7 @@
         <v>0</v>
       </c>
       <c r="Y46" s="2" t="s">
-        <v>1167</v>
+        <v>1184</v>
       </c>
       <c r="Z46" s="2" t="s">
         <v>0</v>
@@ -35147,10 +35638,10 @@
         <v>74</v>
       </c>
       <c r="AD46" s="2" t="s">
-        <v>1066</v>
+        <v>1092</v>
       </c>
       <c r="AE46" s="2" t="s">
-        <v>1065</v>
+        <v>1091</v>
       </c>
       <c r="AF46" s="2" t="s">
         <v>0</v>
@@ -35170,13 +35661,13 @@
     </row>
     <row r="47" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
-        <v>1166</v>
+        <v>1183</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>1166</v>
+        <v>1183</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D47" s="7">
         <v>46064</v>
@@ -35188,10 +35679,10 @@
         <v>61</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>1165</v>
+        <v>1182</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>1164</v>
+        <v>1181</v>
       </c>
       <c r="I47" s="3" t="s">
         <v>139</v>
@@ -35203,13 +35694,13 @@
         <v>417</v>
       </c>
       <c r="L47" s="3" t="s">
-        <v>1163</v>
+        <v>1180</v>
       </c>
       <c r="M47" s="3" t="s">
-        <v>1162</v>
+        <v>1179</v>
       </c>
       <c r="N47" s="3" t="s">
-        <v>1161</v>
+        <v>1178</v>
       </c>
       <c r="O47" s="8">
         <v>1000</v>
@@ -35242,7 +35733,7 @@
         <v>51</v>
       </c>
       <c r="Y47" s="3" t="s">
-        <v>1160</v>
+        <v>1177</v>
       </c>
       <c r="Z47" s="3" t="s">
         <v>0</v>
@@ -35280,13 +35771,13 @@
     </row>
     <row r="48" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
-        <v>1157</v>
+        <v>1174</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>1157</v>
+        <v>1174</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D48" s="4">
         <v>46064</v>
@@ -35304,22 +35795,22 @@
         <v>386</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>1156</v>
+        <v>1173</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>1155</v>
+        <v>1172</v>
       </c>
       <c r="K48" s="2" t="s">
         <v>446</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>1159</v>
+        <v>1176</v>
       </c>
       <c r="M48" s="2" t="s">
-        <v>1158</v>
+        <v>1175</v>
       </c>
       <c r="N48" s="2" t="s">
-        <v>1124</v>
+        <v>1141</v>
       </c>
       <c r="O48" s="5">
         <v>1000</v>
@@ -35352,7 +35843,7 @@
         <v>51</v>
       </c>
       <c r="Y48" s="2" t="s">
-        <v>1154</v>
+        <v>1171</v>
       </c>
       <c r="Z48" s="2" t="s">
         <v>0</v>
@@ -35390,13 +35881,13 @@
     </row>
     <row r="49" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
-        <v>1157</v>
+        <v>1174</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>1157</v>
+        <v>1174</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D49" s="7">
         <v>46064</v>
@@ -35414,22 +35905,22 @@
         <v>386</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>1156</v>
+        <v>1173</v>
       </c>
       <c r="J49" s="3" t="s">
-        <v>1155</v>
+        <v>1172</v>
       </c>
       <c r="K49" s="3" t="s">
         <v>446</v>
       </c>
       <c r="L49" s="3" t="s">
-        <v>1126</v>
+        <v>1143</v>
       </c>
       <c r="M49" s="3" t="s">
-        <v>1125</v>
+        <v>1142</v>
       </c>
       <c r="N49" s="3" t="s">
-        <v>1124</v>
+        <v>1141</v>
       </c>
       <c r="O49" s="8">
         <v>1000</v>
@@ -35462,7 +35953,7 @@
         <v>51</v>
       </c>
       <c r="Y49" s="3" t="s">
-        <v>1154</v>
+        <v>1171</v>
       </c>
       <c r="Z49" s="3" t="s">
         <v>0</v>
@@ -35500,13 +35991,13 @@
     </row>
     <row r="50" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
-        <v>1153</v>
+        <v>1170</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>1153</v>
+        <v>1170</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D50" s="4">
         <v>46066</v>
@@ -35518,10 +36009,10 @@
         <v>61</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>1152</v>
+        <v>1169</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>1151</v>
+        <v>1168</v>
       </c>
       <c r="I50" s="2" t="s">
         <v>163</v>
@@ -35533,13 +36024,13 @@
         <v>632</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>1150</v>
+        <v>1167</v>
       </c>
       <c r="M50" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N50" s="2" t="s">
-        <v>1149</v>
+        <v>1166</v>
       </c>
       <c r="O50" s="5">
         <v>507</v>
@@ -35572,7 +36063,7 @@
         <v>51</v>
       </c>
       <c r="Y50" s="2" t="s">
-        <v>1148</v>
+        <v>1165</v>
       </c>
       <c r="Z50" s="2" t="s">
         <v>0</v>
@@ -35610,13 +36101,13 @@
     </row>
     <row r="51" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
-        <v>1147</v>
+        <v>1164</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>1147</v>
+        <v>1164</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D51" s="7">
         <v>46071</v>
@@ -35640,16 +36131,16 @@
         <v>164</v>
       </c>
       <c r="K51" s="3" t="s">
-        <v>1086</v>
+        <v>1111</v>
       </c>
       <c r="L51" s="3" t="s">
-        <v>1146</v>
+        <v>1163</v>
       </c>
       <c r="M51" s="3" t="s">
-        <v>1145</v>
+        <v>1162</v>
       </c>
       <c r="N51" s="3" t="s">
-        <v>1144</v>
+        <v>1161</v>
       </c>
       <c r="O51" s="8">
         <v>500</v>
@@ -35682,7 +36173,7 @@
         <v>51</v>
       </c>
       <c r="Y51" s="3" t="s">
-        <v>1143</v>
+        <v>1160</v>
       </c>
       <c r="Z51" s="3" t="s">
         <v>0</v>
@@ -35697,10 +36188,10 @@
         <v>111</v>
       </c>
       <c r="AD51" s="3" t="s">
-        <v>1081</v>
+        <v>1106</v>
       </c>
       <c r="AE51" s="3" t="s">
-        <v>1080</v>
+        <v>1105</v>
       </c>
       <c r="AF51" s="3" t="s">
         <v>77</v>
@@ -35720,13 +36211,13 @@
     </row>
     <row r="52" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>1142</v>
+        <v>1159</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>1142</v>
+        <v>1159</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D52" s="4">
         <v>46071</v>
@@ -35738,10 +36229,10 @@
         <v>61</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>1141</v>
+        <v>1158</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>1140</v>
+        <v>1157</v>
       </c>
       <c r="I52" s="2" t="s">
         <v>139</v>
@@ -35753,13 +36244,13 @@
         <v>446</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>1126</v>
+        <v>1143</v>
       </c>
       <c r="M52" s="2" t="s">
-        <v>1125</v>
+        <v>1142</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>1124</v>
+        <v>1141</v>
       </c>
       <c r="O52" s="5">
         <v>200</v>
@@ -35792,7 +36283,7 @@
         <v>51</v>
       </c>
       <c r="Y52" s="2" t="s">
-        <v>1139</v>
+        <v>1156</v>
       </c>
       <c r="Z52" s="2" t="s">
         <v>0</v>
@@ -35830,13 +36321,13 @@
     </row>
     <row r="53" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
-        <v>1138</v>
+        <v>1155</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>1138</v>
+        <v>1155</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D53" s="7">
         <v>46072</v>
@@ -35848,10 +36339,10 @@
         <v>40</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>1070</v>
+        <v>1096</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>1069</v>
+        <v>1095</v>
       </c>
       <c r="I53" s="3" t="s">
         <v>43</v>
@@ -35863,13 +36354,13 @@
         <v>440</v>
       </c>
       <c r="L53" s="3" t="s">
-        <v>1137</v>
+        <v>1154</v>
       </c>
       <c r="M53" s="3" t="s">
-        <v>1136</v>
+        <v>1153</v>
       </c>
       <c r="N53" s="3" t="s">
-        <v>1135</v>
+        <v>1152</v>
       </c>
       <c r="O53" s="8">
         <v>50</v>
@@ -35893,16 +36384,16 @@
         <v>0</v>
       </c>
       <c r="V53" s="3" t="s">
-        <v>1134</v>
+        <v>1151</v>
       </c>
       <c r="W53" s="3" t="s">
-        <v>1133</v>
+        <v>1150</v>
       </c>
       <c r="X53" s="3" t="s">
         <v>51</v>
       </c>
       <c r="Y53" s="3" t="s">
-        <v>1132</v>
+        <v>1149</v>
       </c>
       <c r="Z53" s="3" t="s">
         <v>0</v>
@@ -35940,13 +36431,13 @@
     </row>
     <row r="54" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>1131</v>
+        <v>1148</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>1131</v>
+        <v>1148</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D54" s="4">
         <v>46072</v>
@@ -35958,10 +36449,10 @@
         <v>61</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>1121</v>
+        <v>1138</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>1120</v>
+        <v>1137</v>
       </c>
       <c r="I54" s="2" t="s">
         <v>163</v>
@@ -35973,13 +36464,13 @@
         <v>417</v>
       </c>
       <c r="L54" s="2" t="s">
-        <v>1106</v>
+        <v>1128</v>
       </c>
       <c r="M54" s="2" t="s">
-        <v>1105</v>
+        <v>1127</v>
       </c>
       <c r="N54" s="2" t="s">
-        <v>1104</v>
+        <v>1087</v>
       </c>
       <c r="O54" s="5">
         <v>1600</v>
@@ -36012,7 +36503,7 @@
         <v>51</v>
       </c>
       <c r="Y54" s="2" t="s">
-        <v>1130</v>
+        <v>1147</v>
       </c>
       <c r="Z54" s="2" t="s">
         <v>0</v>
@@ -36050,13 +36541,13 @@
     </row>
     <row r="55" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
-        <v>1129</v>
+        <v>1146</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>1129</v>
+        <v>1146</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D55" s="7">
         <v>46072</v>
@@ -36068,10 +36559,10 @@
         <v>40</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>1128</v>
+        <v>1145</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>1127</v>
+        <v>1144</v>
       </c>
       <c r="I55" s="3" t="s">
         <v>43</v>
@@ -36083,13 +36574,13 @@
         <v>446</v>
       </c>
       <c r="L55" s="3" t="s">
-        <v>1126</v>
+        <v>1143</v>
       </c>
       <c r="M55" s="3" t="s">
-        <v>1125</v>
+        <v>1142</v>
       </c>
       <c r="N55" s="3" t="s">
-        <v>1124</v>
+        <v>1141</v>
       </c>
       <c r="O55" s="8">
         <v>500</v>
@@ -36122,7 +36613,7 @@
         <v>51</v>
       </c>
       <c r="Y55" s="3" t="s">
-        <v>1123</v>
+        <v>1140</v>
       </c>
       <c r="Z55" s="3" t="s">
         <v>0</v>
@@ -36160,13 +36651,13 @@
     </row>
     <row r="56" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
-        <v>1122</v>
+        <v>1139</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>1122</v>
+        <v>1139</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D56" s="4">
         <v>46076</v>
@@ -36178,10 +36669,10 @@
         <v>61</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>1121</v>
+        <v>1138</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>1120</v>
+        <v>1137</v>
       </c>
       <c r="I56" s="2" t="s">
         <v>163</v>
@@ -36193,13 +36684,13 @@
         <v>417</v>
       </c>
       <c r="L56" s="2" t="s">
-        <v>1106</v>
+        <v>1128</v>
       </c>
       <c r="M56" s="2" t="s">
-        <v>1105</v>
+        <v>1127</v>
       </c>
       <c r="N56" s="2" t="s">
-        <v>1104</v>
+        <v>1087</v>
       </c>
       <c r="O56" s="5">
         <v>1700</v>
@@ -36232,7 +36723,7 @@
         <v>51</v>
       </c>
       <c r="Y56" s="2" t="s">
-        <v>1119</v>
+        <v>1136</v>
       </c>
       <c r="Z56" s="2" t="s">
         <v>0</v>
@@ -36270,13 +36761,13 @@
     </row>
     <row r="57" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
-        <v>1116</v>
+        <v>1133</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>1116</v>
+        <v>1133</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D57" s="7">
         <v>46077</v>
@@ -36300,16 +36791,16 @@
         <v>164</v>
       </c>
       <c r="K57" s="3" t="s">
-        <v>1091</v>
+        <v>1116</v>
       </c>
       <c r="L57" s="3" t="s">
-        <v>1118</v>
+        <v>1135</v>
       </c>
       <c r="M57" s="3" t="s">
-        <v>1117</v>
+        <v>1134</v>
       </c>
       <c r="N57" s="3" t="s">
-        <v>1088</v>
+        <v>1113</v>
       </c>
       <c r="O57" s="8">
         <v>500</v>
@@ -36342,7 +36833,7 @@
         <v>51</v>
       </c>
       <c r="Y57" s="3" t="s">
-        <v>1115</v>
+        <v>1132</v>
       </c>
       <c r="Z57" s="3" t="s">
         <v>0</v>
@@ -36380,13 +36871,13 @@
     </row>
     <row r="58" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
-        <v>1116</v>
+        <v>1133</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>1116</v>
+        <v>1133</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D58" s="4">
         <v>46077</v>
@@ -36410,16 +36901,16 @@
         <v>164</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>1086</v>
+        <v>1111</v>
       </c>
       <c r="L58" s="2" t="s">
-        <v>1085</v>
+        <v>1110</v>
       </c>
       <c r="M58" s="2" t="s">
-        <v>1084</v>
+        <v>1109</v>
       </c>
       <c r="N58" s="2" t="s">
-        <v>1083</v>
+        <v>1108</v>
       </c>
       <c r="O58" s="5">
         <v>500</v>
@@ -36452,7 +36943,7 @@
         <v>51</v>
       </c>
       <c r="Y58" s="2" t="s">
-        <v>1115</v>
+        <v>1132</v>
       </c>
       <c r="Z58" s="2" t="s">
         <v>0</v>
@@ -36467,10 +36958,10 @@
         <v>111</v>
       </c>
       <c r="AD58" s="2" t="s">
-        <v>1081</v>
+        <v>1106</v>
       </c>
       <c r="AE58" s="2" t="s">
-        <v>1080</v>
+        <v>1105</v>
       </c>
       <c r="AF58" s="2" t="s">
         <v>77</v>
@@ -36490,13 +36981,13 @@
     </row>
     <row r="59" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
-        <v>1114</v>
+        <v>1131</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>1114</v>
+        <v>1131</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D59" s="7">
         <v>46078</v>
@@ -36508,10 +36999,10 @@
         <v>40</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>1113</v>
+        <v>1081</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>1112</v>
+        <v>1080</v>
       </c>
       <c r="I59" s="3" t="s">
         <v>139</v>
@@ -36523,13 +37014,13 @@
         <v>784</v>
       </c>
       <c r="L59" s="3" t="s">
-        <v>1111</v>
+        <v>1079</v>
       </c>
       <c r="M59" s="3" t="s">
-        <v>1110</v>
+        <v>1078</v>
       </c>
       <c r="N59" s="3" t="s">
-        <v>1109</v>
+        <v>1077</v>
       </c>
       <c r="O59" s="8">
         <v>225</v>
@@ -36562,7 +37053,7 @@
         <v>51</v>
       </c>
       <c r="Y59" s="3" t="s">
-        <v>1108</v>
+        <v>1130</v>
       </c>
       <c r="Z59" s="3" t="s">
         <v>0</v>
@@ -36600,13 +37091,13 @@
     </row>
     <row r="60" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
-        <v>1107</v>
+        <v>1129</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>1107</v>
+        <v>1129</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D60" s="4">
         <v>46079</v>
@@ -36633,13 +37124,13 @@
         <v>417</v>
       </c>
       <c r="L60" s="2" t="s">
-        <v>1106</v>
+        <v>1128</v>
       </c>
       <c r="M60" s="2" t="s">
-        <v>1105</v>
+        <v>1127</v>
       </c>
       <c r="N60" s="2" t="s">
-        <v>1104</v>
+        <v>1087</v>
       </c>
       <c r="O60" s="5">
         <v>5000</v>
@@ -36663,16 +37154,16 @@
         <v>2354</v>
       </c>
       <c r="V60" s="2" t="s">
-        <v>1103</v>
+        <v>1086</v>
       </c>
       <c r="W60" s="2" t="s">
-        <v>1102</v>
+        <v>1085</v>
       </c>
       <c r="X60" s="2" t="s">
         <v>51</v>
       </c>
       <c r="Y60" s="2" t="s">
-        <v>1101</v>
+        <v>1126</v>
       </c>
       <c r="Z60" s="2" t="s">
         <v>0</v>
@@ -36710,13 +37201,13 @@
     </row>
     <row r="61" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
-        <v>1100</v>
+        <v>1125</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>1100</v>
+        <v>1125</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D61" s="7">
         <v>46079</v>
@@ -36743,13 +37234,13 @@
         <v>1060</v>
       </c>
       <c r="L61" s="3" t="s">
-        <v>1099</v>
+        <v>1124</v>
       </c>
       <c r="M61" s="3" t="s">
-        <v>1098</v>
+        <v>1123</v>
       </c>
       <c r="N61" s="3" t="s">
-        <v>1097</v>
+        <v>1122</v>
       </c>
       <c r="O61" s="8">
         <v>12000</v>
@@ -36782,7 +37273,7 @@
         <v>51</v>
       </c>
       <c r="Y61" s="3" t="s">
-        <v>1096</v>
+        <v>1121</v>
       </c>
       <c r="Z61" s="3" t="s">
         <v>0</v>
@@ -36820,13 +37311,13 @@
     </row>
     <row r="62" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
-        <v>1095</v>
+        <v>1120</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>1095</v>
+        <v>1120</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D62" s="4">
         <v>46085</v>
@@ -36853,13 +37344,13 @@
         <v>633</v>
       </c>
       <c r="L62" s="2" t="s">
-        <v>1094</v>
+        <v>1119</v>
       </c>
       <c r="M62" s="2" t="s">
         <v>652</v>
       </c>
       <c r="N62" s="2" t="s">
-        <v>1093</v>
+        <v>1118</v>
       </c>
       <c r="O62" s="5">
         <v>5005</v>
@@ -36892,7 +37383,7 @@
         <v>51</v>
       </c>
       <c r="Y62" s="2" t="s">
-        <v>1092</v>
+        <v>1117</v>
       </c>
       <c r="Z62" s="2" t="s">
         <v>0</v>
@@ -36930,13 +37421,13 @@
     </row>
     <row r="63" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
-        <v>1087</v>
+        <v>1112</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>1087</v>
+        <v>1112</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D63" s="7">
         <v>46085</v>
@@ -36960,16 +37451,16 @@
         <v>164</v>
       </c>
       <c r="K63" s="3" t="s">
-        <v>1091</v>
+        <v>1116</v>
       </c>
       <c r="L63" s="3" t="s">
-        <v>1090</v>
+        <v>1115</v>
       </c>
       <c r="M63" s="3" t="s">
-        <v>1089</v>
+        <v>1114</v>
       </c>
       <c r="N63" s="3" t="s">
-        <v>1088</v>
+        <v>1113</v>
       </c>
       <c r="O63" s="8">
         <v>500</v>
@@ -37002,7 +37493,7 @@
         <v>51</v>
       </c>
       <c r="Y63" s="3" t="s">
-        <v>1082</v>
+        <v>1107</v>
       </c>
       <c r="Z63" s="3" t="s">
         <v>0</v>
@@ -37040,13 +37531,13 @@
     </row>
     <row r="64" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
-        <v>1087</v>
+        <v>1112</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>1087</v>
+        <v>1112</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D64" s="4">
         <v>46085</v>
@@ -37070,16 +37561,16 @@
         <v>164</v>
       </c>
       <c r="K64" s="2" t="s">
-        <v>1086</v>
+        <v>1111</v>
       </c>
       <c r="L64" s="2" t="s">
-        <v>1085</v>
+        <v>1110</v>
       </c>
       <c r="M64" s="2" t="s">
-        <v>1084</v>
+        <v>1109</v>
       </c>
       <c r="N64" s="2" t="s">
-        <v>1083</v>
+        <v>1108</v>
       </c>
       <c r="O64" s="5">
         <v>500</v>
@@ -37112,7 +37603,7 @@
         <v>51</v>
       </c>
       <c r="Y64" s="2" t="s">
-        <v>1082</v>
+        <v>1107</v>
       </c>
       <c r="Z64" s="2" t="s">
         <v>0</v>
@@ -37127,10 +37618,10 @@
         <v>111</v>
       </c>
       <c r="AD64" s="2" t="s">
-        <v>1081</v>
+        <v>1106</v>
       </c>
       <c r="AE64" s="2" t="s">
-        <v>1080</v>
+        <v>1105</v>
       </c>
       <c r="AF64" s="2" t="s">
         <v>77</v>
@@ -37150,13 +37641,13 @@
     </row>
     <row r="65" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
-        <v>1079</v>
+        <v>1104</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>1079</v>
+        <v>1104</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D65" s="7">
         <v>46085</v>
@@ -37168,10 +37659,10 @@
         <v>40</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>1078</v>
+        <v>1103</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>1077</v>
+        <v>1102</v>
       </c>
       <c r="I65" s="3" t="s">
         <v>163</v>
@@ -37183,13 +37674,13 @@
         <v>154</v>
       </c>
       <c r="L65" s="3" t="s">
-        <v>1076</v>
+        <v>1101</v>
       </c>
       <c r="M65" s="3" t="s">
-        <v>1075</v>
+        <v>1100</v>
       </c>
       <c r="N65" s="3" t="s">
-        <v>1074</v>
+        <v>1099</v>
       </c>
       <c r="O65" s="8">
         <v>3700</v>
@@ -37222,7 +37713,7 @@
         <v>51</v>
       </c>
       <c r="Y65" s="3" t="s">
-        <v>1073</v>
+        <v>1098</v>
       </c>
       <c r="Z65" s="3" t="s">
         <v>0</v>
@@ -37260,13 +37751,13 @@
     </row>
     <row r="66" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
-        <v>1072</v>
+        <v>1097</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>1072</v>
+        <v>1097</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D66" s="4">
         <v>46085</v>
@@ -37278,10 +37769,10 @@
         <v>40</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>1070</v>
+        <v>1096</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>1069</v>
+        <v>1095</v>
       </c>
       <c r="I66" s="2" t="s">
         <v>139</v>
@@ -37290,7 +37781,7 @@
         <v>140</v>
       </c>
       <c r="K66" s="2" t="s">
-        <v>1068</v>
+        <v>1094</v>
       </c>
       <c r="L66" s="2" t="s">
         <v>0</v>
@@ -37332,7 +37823,7 @@
         <v>0</v>
       </c>
       <c r="Y66" s="2" t="s">
-        <v>1067</v>
+        <v>1093</v>
       </c>
       <c r="Z66" s="2" t="s">
         <v>0</v>
@@ -37347,10 +37838,10 @@
         <v>298</v>
       </c>
       <c r="AD66" s="2" t="s">
-        <v>1066</v>
+        <v>1092</v>
       </c>
       <c r="AE66" s="2" t="s">
-        <v>1065</v>
+        <v>1091</v>
       </c>
       <c r="AF66" s="2" t="s">
         <v>0</v>
@@ -37366,6 +37857,226 @@
       </c>
       <c r="AJ66" s="5">
         <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A67" s="3" t="s">
+        <v>1090</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>1090</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>1082</v>
+      </c>
+      <c r="D67" s="7">
+        <v>46091</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F67" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G67" s="3" t="s">
+        <v>782</v>
+      </c>
+      <c r="H67" s="3" t="s">
+        <v>783</v>
+      </c>
+      <c r="I67" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="J67" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="K67" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="L67" s="3" t="s">
+        <v>1089</v>
+      </c>
+      <c r="M67" s="3" t="s">
+        <v>1088</v>
+      </c>
+      <c r="N67" s="3" t="s">
+        <v>1087</v>
+      </c>
+      <c r="O67" s="8">
+        <v>5000</v>
+      </c>
+      <c r="P67" s="8">
+        <v>11.77</v>
+      </c>
+      <c r="Q67" s="9">
+        <v>58850</v>
+      </c>
+      <c r="R67" s="9">
+        <v>1912.63</v>
+      </c>
+      <c r="S67" s="9">
+        <v>60762.63</v>
+      </c>
+      <c r="T67" s="9">
+        <v>58850</v>
+      </c>
+      <c r="U67" s="9">
+        <v>2354</v>
+      </c>
+      <c r="V67" s="3" t="s">
+        <v>1086</v>
+      </c>
+      <c r="W67" s="3" t="s">
+        <v>1085</v>
+      </c>
+      <c r="X67" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y67" s="3" t="s">
+        <v>1084</v>
+      </c>
+      <c r="Z67" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA67" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB67" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="AC67" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="AD67" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="AE67" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="AF67" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="AG67" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH67" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI67" s="9">
+        <v>4</v>
+      </c>
+      <c r="AJ67" s="8">
+        <v>48943.45</v>
+      </c>
+    </row>
+    <row r="68" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A68" s="2" t="s">
+        <v>1083</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>1083</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>1082</v>
+      </c>
+      <c r="D68" s="4">
+        <v>46091</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>1081</v>
+      </c>
+      <c r="H68" s="2" t="s">
+        <v>1080</v>
+      </c>
+      <c r="I68" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="J68" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="K68" s="2" t="s">
+        <v>784</v>
+      </c>
+      <c r="L68" s="2" t="s">
+        <v>1079</v>
+      </c>
+      <c r="M68" s="2" t="s">
+        <v>1078</v>
+      </c>
+      <c r="N68" s="2" t="s">
+        <v>1077</v>
+      </c>
+      <c r="O68" s="5">
+        <v>225</v>
+      </c>
+      <c r="P68" s="5">
+        <v>12.25</v>
+      </c>
+      <c r="Q68" s="6">
+        <v>2756.25</v>
+      </c>
+      <c r="R68" s="6">
+        <v>89.58</v>
+      </c>
+      <c r="S68" s="6">
+        <v>2845.83</v>
+      </c>
+      <c r="T68" s="6">
+        <v>2756.25</v>
+      </c>
+      <c r="U68" s="6">
+        <v>110.25</v>
+      </c>
+      <c r="V68" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="W68" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="X68" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y68" s="2" t="s">
+        <v>1076</v>
+      </c>
+      <c r="Z68" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA68" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB68" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC68" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD68" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="AE68" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="AF68" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AG68" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH68" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI68" s="6">
+        <v>4</v>
+      </c>
+      <c r="AJ68" s="5">
+        <v>2225.1802499999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização da base de dados 11.03.2026
</commit_message>
<xml_diff>
--- a/BASE_KEMPARTS.xlsx
+++ b/BASE_KEMPARTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dash_kp_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{97583B37-DC83-4DD0-9F4C-6CDFE6B33DC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4411F3B8-10E0-4D1D-BC04-9B36A6AE8EC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{CB469FB5-CC63-49DF-8F0A-CC2C928DC074}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{54047E8A-2573-47AA-9902-914A4DC7D30A}"/>
   </bookViews>
   <sheets>
     <sheet name="FSP" sheetId="3" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7547" uniqueCount="1305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7722" uniqueCount="1325">
   <si>
     <t/>
   </si>
@@ -3251,6 +3251,102 @@
     <t>153309</t>
   </si>
   <si>
+    <t>000015554</t>
+  </si>
+  <si>
+    <t>173734</t>
+  </si>
+  <si>
+    <t>000015555</t>
+  </si>
+  <si>
+    <t>T00166</t>
+  </si>
+  <si>
+    <t>IBERICO TRANSPORTES E LOGISTICA EIRELI</t>
+  </si>
+  <si>
+    <t>173852</t>
+  </si>
+  <si>
+    <t>000015556</t>
+  </si>
+  <si>
+    <t>C00481</t>
+  </si>
+  <si>
+    <t>FLEXCOR TINTAS EIRELLI</t>
+  </si>
+  <si>
+    <t>T00151</t>
+  </si>
+  <si>
+    <t>LUSEANNA TRANSP ARMAZ LTDA</t>
+  </si>
+  <si>
+    <t>173853</t>
+  </si>
+  <si>
+    <t>003309</t>
+  </si>
+  <si>
+    <t>TRANSPARE TRANSPORTES ARMAZENS GERAIS LT</t>
+  </si>
+  <si>
+    <t>T00258</t>
+  </si>
+  <si>
+    <t>2024.357.04.</t>
+  </si>
+  <si>
+    <t>240706</t>
+  </si>
+  <si>
+    <t>2024.357.04.240706</t>
+  </si>
+  <si>
+    <t>KEMPARTS COMERCIO INTERNACIONAL DE PRODU</t>
+  </si>
+  <si>
+    <t>C00001</t>
+  </si>
+  <si>
+    <t>TRANSFERENCIA DE MERC. ADQUIRIDA/RECEBIDA DE TERCEIROS</t>
+  </si>
+  <si>
+    <t>6152</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>000002511</t>
+  </si>
+  <si>
+    <t>2025.357.05.</t>
+  </si>
+  <si>
+    <t>20250903</t>
+  </si>
+  <si>
+    <t>2025.357.05.20250903</t>
+  </si>
+  <si>
+    <t>2025.004.01.</t>
+  </si>
+  <si>
+    <t>25021048</t>
+  </si>
+  <si>
+    <t>2025.004.01.25021048</t>
+  </si>
+  <si>
+    <t>2024.004.14.</t>
+  </si>
+  <si>
+    <t>2024.004.14.24121064</t>
+  </si>
+  <si>
     <t>003301</t>
   </si>
   <si>
@@ -3269,9 +3365,6 @@
     <t>C00341</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>000002510</t>
   </si>
   <si>
@@ -3284,15 +3377,6 @@
     <t>T00213</t>
   </si>
   <si>
-    <t>2025.004.01.</t>
-  </si>
-  <si>
-    <t>25021048</t>
-  </si>
-  <si>
-    <t>2025.004.01.25021048</t>
-  </si>
-  <si>
     <t>000002509</t>
   </si>
   <si>
@@ -3578,12 +3662,6 @@
     <t>003257</t>
   </si>
   <si>
-    <t>KEMPARTS COMERCIO INTERNACIONAL DE PRODU</t>
-  </si>
-  <si>
-    <t>C00001</t>
-  </si>
-  <si>
     <t>6101</t>
   </si>
   <si>
@@ -3593,9 +3671,6 @@
     <t>003253</t>
   </si>
   <si>
-    <t>2024.004.14.</t>
-  </si>
-  <si>
     <t>24121037</t>
   </si>
   <si>
@@ -3650,9 +3725,6 @@
     <t>CH 332</t>
   </si>
   <si>
-    <t>TRANSPARE TRANSPORTES ARMAZENS GERAIS LT</t>
-  </si>
-  <si>
     <t>F00813</t>
   </si>
   <si>
@@ -3749,9 +3821,6 @@
     <t>003219</t>
   </si>
   <si>
-    <t>T00258</t>
-  </si>
-  <si>
     <t>2025.435.</t>
   </si>
   <si>
@@ -3761,12 +3830,6 @@
     <t>2025.435.030001006106</t>
   </si>
   <si>
-    <t>TRANSFERENCIA DE MERC. ADQUIRIDA/RECEBIDA DE TERCEIROS</t>
-  </si>
-  <si>
-    <t>6152</t>
-  </si>
-  <si>
     <t>000002456</t>
   </si>
   <si>
@@ -3876,9 +3939,6 @@
   </si>
   <si>
     <t>003200</t>
-  </si>
-  <si>
-    <t>2025.357.05.</t>
   </si>
   <si>
     <t>250501</t>
@@ -4882,8 +4942,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B26A77ED-7CEE-4E89-8BE8-34DC8758E529}">
-  <dimension ref="A1:AJ233"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91811D7F-73CA-4BD0-A771-919B24F863E7}">
+  <dimension ref="A1:AJ236"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
@@ -30553,14 +30613,344 @@
         <v>9.8208099999999998</v>
       </c>
     </row>
+    <row r="234" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A234" s="2" t="s">
+        <v>1076</v>
+      </c>
+      <c r="B234" s="2" t="s">
+        <v>1076</v>
+      </c>
+      <c r="C234" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D234" s="4">
+        <v>46092</v>
+      </c>
+      <c r="E234" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F234" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G234" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="H234" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="I234" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="J234" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="K234" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="L234" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="M234" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="N234" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="O234" s="5">
+        <v>370</v>
+      </c>
+      <c r="P234" s="5">
+        <v>25.75</v>
+      </c>
+      <c r="Q234" s="6">
+        <v>9527.5</v>
+      </c>
+      <c r="R234" s="6">
+        <v>309.64</v>
+      </c>
+      <c r="S234" s="6">
+        <v>9837.14</v>
+      </c>
+      <c r="T234" s="6">
+        <v>9527.5</v>
+      </c>
+      <c r="U234" s="6">
+        <v>381.1</v>
+      </c>
+      <c r="V234" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="W234" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="X234" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y234" s="2" t="s">
+        <v>1077</v>
+      </c>
+      <c r="Z234" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA234" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB234" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC234" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="AD234" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE234" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="AF234" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AG234" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH234" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI234" s="6">
+        <v>4</v>
+      </c>
+      <c r="AJ234" s="5">
+        <v>4912.8082000000004</v>
+      </c>
+    </row>
+    <row r="235" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A235" s="3" t="s">
+        <v>1078</v>
+      </c>
+      <c r="B235" s="3" t="s">
+        <v>1078</v>
+      </c>
+      <c r="C235" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D235" s="7">
+        <v>46092</v>
+      </c>
+      <c r="E235" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F235" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="G235" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="H235" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I235" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="J235" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="K235" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="L235" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="M235" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="N235" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="O235" s="8">
+        <v>14800</v>
+      </c>
+      <c r="P235" s="8">
+        <v>12.23531</v>
+      </c>
+      <c r="Q235" s="9">
+        <v>181082.59</v>
+      </c>
+      <c r="R235" s="9">
+        <v>0</v>
+      </c>
+      <c r="S235" s="9">
+        <v>181082.59</v>
+      </c>
+      <c r="T235" s="9">
+        <v>0</v>
+      </c>
+      <c r="U235" s="9">
+        <v>0</v>
+      </c>
+      <c r="V235" s="3" t="s">
+        <v>1079</v>
+      </c>
+      <c r="W235" s="3" t="s">
+        <v>1080</v>
+      </c>
+      <c r="X235" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y235" s="3" t="s">
+        <v>1081</v>
+      </c>
+      <c r="Z235" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA235" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB235" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="AC235" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD235" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE235" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="AF235" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AG235" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH235" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI235" s="9">
+        <v>0</v>
+      </c>
+      <c r="AJ235" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="236" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A236" s="2" t="s">
+        <v>1082</v>
+      </c>
+      <c r="B236" s="2" t="s">
+        <v>1082</v>
+      </c>
+      <c r="C236" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D236" s="4">
+        <v>46092</v>
+      </c>
+      <c r="E236" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F236" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G236" s="2" t="s">
+        <v>1083</v>
+      </c>
+      <c r="H236" s="2" t="s">
+        <v>1084</v>
+      </c>
+      <c r="I236" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="J236" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="K236" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="L236" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="M236" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="N236" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="O236" s="5">
+        <v>1000</v>
+      </c>
+      <c r="P236" s="5">
+        <v>15.02</v>
+      </c>
+      <c r="Q236" s="6">
+        <v>15020</v>
+      </c>
+      <c r="R236" s="6">
+        <v>488.15</v>
+      </c>
+      <c r="S236" s="6">
+        <v>15508.15</v>
+      </c>
+      <c r="T236" s="6">
+        <v>15020</v>
+      </c>
+      <c r="U236" s="6">
+        <v>600.79999999999995</v>
+      </c>
+      <c r="V236" s="2" t="s">
+        <v>1085</v>
+      </c>
+      <c r="W236" s="2" t="s">
+        <v>1086</v>
+      </c>
+      <c r="X236" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y236" s="2" t="s">
+        <v>1087</v>
+      </c>
+      <c r="Z236" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA236" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB236" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="AC236" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="AD236" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="AE236" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="AF236" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AG236" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH236" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI236" s="6">
+        <v>4</v>
+      </c>
+      <c r="AJ236" s="5">
+        <v>10341.27</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49746817-01A4-4A9C-9061-C45AA702B917}">
-  <dimension ref="A1:AJ68"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7F5C9F-1B8B-4223-BCB6-9F8E23135EC6}">
+  <dimension ref="A1:AJ72"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
@@ -30711,13 +31101,13 @@
     </row>
     <row r="2" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>1304</v>
+        <v>1324</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>1304</v>
+        <v>1324</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D2" s="4">
         <v>46024</v>
@@ -30729,10 +31119,10 @@
         <v>40</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>1096</v>
+        <v>1124</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>1095</v>
+        <v>1123</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>43</v>
@@ -30744,13 +31134,13 @@
         <v>440</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>1154</v>
+        <v>1182</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>1153</v>
+        <v>1181</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>1152</v>
+        <v>1180</v>
       </c>
       <c r="O2" s="5">
         <v>50</v>
@@ -30774,16 +31164,16 @@
         <v>39.06</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>1151</v>
+        <v>1179</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>1150</v>
+        <v>1178</v>
       </c>
       <c r="X2" s="2" t="s">
         <v>51</v>
       </c>
       <c r="Y2" s="2" t="s">
-        <v>1303</v>
+        <v>1323</v>
       </c>
       <c r="Z2" s="2" t="s">
         <v>0</v>
@@ -30821,13 +31211,13 @@
     </row>
     <row r="3" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>1302</v>
+        <v>1322</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>1302</v>
+        <v>1322</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D3" s="7">
         <v>46027</v>
@@ -30839,10 +31229,10 @@
         <v>61</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>1169</v>
+        <v>1197</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>1168</v>
+        <v>1196</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>163</v>
@@ -30854,13 +31244,13 @@
         <v>632</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>1167</v>
+        <v>1195</v>
       </c>
       <c r="M3" s="3" t="s">
         <v>648</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>1166</v>
+        <v>1194</v>
       </c>
       <c r="O3" s="8">
         <v>1001</v>
@@ -30893,7 +31283,7 @@
         <v>51</v>
       </c>
       <c r="Y3" s="3" t="s">
-        <v>1301</v>
+        <v>1321</v>
       </c>
       <c r="Z3" s="3" t="s">
         <v>0</v>
@@ -30931,13 +31321,13 @@
     </row>
     <row r="4" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>1300</v>
+        <v>1320</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>1300</v>
+        <v>1320</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D4" s="4">
         <v>46027</v>
@@ -30949,10 +31339,10 @@
         <v>61</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>1299</v>
+        <v>1319</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>1298</v>
+        <v>1318</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>152</v>
@@ -30964,13 +31354,13 @@
         <v>342</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>1297</v>
+        <v>1317</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>1296</v>
+        <v>1316</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>1295</v>
+        <v>1315</v>
       </c>
       <c r="O4" s="5">
         <v>600</v>
@@ -30994,16 +31384,16 @@
         <v>355.68</v>
       </c>
       <c r="V4" s="2" t="s">
-        <v>1294</v>
+        <v>1314</v>
       </c>
       <c r="W4" s="2" t="s">
-        <v>1293</v>
+        <v>1313</v>
       </c>
       <c r="X4" s="2" t="s">
         <v>51</v>
       </c>
       <c r="Y4" s="2" t="s">
-        <v>1292</v>
+        <v>1312</v>
       </c>
       <c r="Z4" s="2" t="s">
         <v>0</v>
@@ -31041,13 +31431,13 @@
     </row>
     <row r="5" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>1291</v>
+        <v>1311</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1291</v>
+        <v>1311</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D5" s="7">
         <v>46029</v>
@@ -31059,10 +31449,10 @@
         <v>212</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>1210</v>
+        <v>1234</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>1209</v>
+        <v>1089</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>139</v>
@@ -31071,7 +31461,7 @@
         <v>140</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>1290</v>
+        <v>1310</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>0</v>
@@ -31113,7 +31503,7 @@
         <v>87</v>
       </c>
       <c r="Y5" s="3" t="s">
-        <v>1289</v>
+        <v>1309</v>
       </c>
       <c r="Z5" s="3" t="s">
         <v>0</v>
@@ -31151,13 +31541,13 @@
     </row>
     <row r="6" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>1291</v>
+        <v>1311</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1291</v>
+        <v>1311</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D6" s="4">
         <v>46029</v>
@@ -31169,10 +31559,10 @@
         <v>212</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>1210</v>
+        <v>1234</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>1209</v>
+        <v>1089</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>139</v>
@@ -31181,7 +31571,7 @@
         <v>140</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>1290</v>
+        <v>1310</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>0</v>
@@ -31223,7 +31613,7 @@
         <v>87</v>
       </c>
       <c r="Y6" s="2" t="s">
-        <v>1289</v>
+        <v>1309</v>
       </c>
       <c r="Z6" s="2" t="s">
         <v>0</v>
@@ -31261,13 +31651,13 @@
     </row>
     <row r="7" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>1288</v>
+        <v>1308</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1288</v>
+        <v>1308</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D7" s="7">
         <v>46029</v>
@@ -31285,22 +31675,22 @@
         <v>386</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>1173</v>
+        <v>1201</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>1172</v>
+        <v>1200</v>
       </c>
       <c r="K7" s="3" t="s">
         <v>1060</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>1287</v>
+        <v>1307</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>1286</v>
+        <v>1306</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>1285</v>
+        <v>1100</v>
       </c>
       <c r="O7" s="8">
         <v>1000</v>
@@ -31333,7 +31723,7 @@
         <v>51</v>
       </c>
       <c r="Y7" s="3" t="s">
-        <v>1284</v>
+        <v>1305</v>
       </c>
       <c r="Z7" s="3" t="s">
         <v>0</v>
@@ -31371,13 +31761,13 @@
     </row>
     <row r="8" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>1283</v>
+        <v>1304</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>1283</v>
+        <v>1304</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D8" s="4">
         <v>46036</v>
@@ -31389,10 +31779,10 @@
         <v>61</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>1169</v>
+        <v>1197</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>1168</v>
+        <v>1196</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>163</v>
@@ -31404,13 +31794,13 @@
         <v>632</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>1167</v>
+        <v>1195</v>
       </c>
       <c r="M8" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>1166</v>
+        <v>1194</v>
       </c>
       <c r="O8" s="5">
         <v>1001</v>
@@ -31443,7 +31833,7 @@
         <v>51</v>
       </c>
       <c r="Y8" s="2" t="s">
-        <v>1282</v>
+        <v>1303</v>
       </c>
       <c r="Z8" s="2" t="s">
         <v>0</v>
@@ -31481,13 +31871,13 @@
     </row>
     <row r="9" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
-        <v>1281</v>
+        <v>1302</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1281</v>
+        <v>1302</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D9" s="7">
         <v>46037</v>
@@ -31499,10 +31889,10 @@
         <v>61</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>1182</v>
+        <v>1210</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>1181</v>
+        <v>1209</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>163</v>
@@ -31514,13 +31904,13 @@
         <v>417</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>1280</v>
+        <v>1301</v>
       </c>
       <c r="M9" s="3" t="s">
         <v>1043</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>1178</v>
+        <v>1206</v>
       </c>
       <c r="O9" s="8">
         <v>1000</v>
@@ -31553,7 +31943,7 @@
         <v>51</v>
       </c>
       <c r="Y9" s="3" t="s">
-        <v>1279</v>
+        <v>1300</v>
       </c>
       <c r="Z9" s="3" t="s">
         <v>0</v>
@@ -31591,13 +31981,13 @@
     </row>
     <row r="10" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>1278</v>
+        <v>1299</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>1278</v>
+        <v>1299</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D10" s="4">
         <v>46037</v>
@@ -31609,10 +31999,10 @@
         <v>40</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>1081</v>
+        <v>1113</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>1080</v>
+        <v>1112</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>139</v>
@@ -31624,13 +32014,13 @@
         <v>784</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>1079</v>
+        <v>1111</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>1078</v>
+        <v>1110</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>1077</v>
+        <v>1109</v>
       </c>
       <c r="O10" s="5">
         <v>300</v>
@@ -31663,7 +32053,7 @@
         <v>51</v>
       </c>
       <c r="Y10" s="2" t="s">
-        <v>1277</v>
+        <v>1298</v>
       </c>
       <c r="Z10" s="2" t="s">
         <v>0</v>
@@ -31701,13 +32091,13 @@
     </row>
     <row r="11" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>1276</v>
+        <v>1297</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>1276</v>
+        <v>1297</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D11" s="7">
         <v>46037</v>
@@ -31719,10 +32109,10 @@
         <v>40</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>1220</v>
+        <v>1244</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>1219</v>
+        <v>1243</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>43</v>
@@ -31734,13 +32124,13 @@
         <v>300</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>1275</v>
+        <v>1296</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>1274</v>
+        <v>1295</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>1273</v>
+        <v>1294</v>
       </c>
       <c r="O11" s="8">
         <v>25</v>
@@ -31773,7 +32163,7 @@
         <v>51</v>
       </c>
       <c r="Y11" s="3" t="s">
-        <v>1272</v>
+        <v>1293</v>
       </c>
       <c r="Z11" s="3" t="s">
         <v>0</v>
@@ -31811,13 +32201,13 @@
     </row>
     <row r="12" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>1271</v>
+        <v>1292</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>1271</v>
+        <v>1292</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D12" s="4">
         <v>46041</v>
@@ -31829,10 +32219,10 @@
         <v>212</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>1210</v>
+        <v>1234</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>1209</v>
+        <v>1089</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>139</v>
@@ -31841,7 +32231,7 @@
         <v>140</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>1111</v>
+        <v>1139</v>
       </c>
       <c r="L12" s="2" t="s">
         <v>0</v>
@@ -31883,7 +32273,7 @@
         <v>87</v>
       </c>
       <c r="Y12" s="2" t="s">
-        <v>1270</v>
+        <v>1291</v>
       </c>
       <c r="Z12" s="2" t="s">
         <v>0</v>
@@ -31898,10 +32288,10 @@
         <v>55</v>
       </c>
       <c r="AD12" s="2" t="s">
-        <v>1106</v>
+        <v>1134</v>
       </c>
       <c r="AE12" s="2" t="s">
-        <v>1105</v>
+        <v>1133</v>
       </c>
       <c r="AF12" s="2" t="s">
         <v>442</v>
@@ -31921,13 +32311,13 @@
     </row>
     <row r="13" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>1269</v>
+        <v>1290</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>1269</v>
+        <v>1290</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D13" s="7">
         <v>46042</v>
@@ -31945,22 +32335,22 @@
         <v>386</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>1173</v>
+        <v>1201</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>1172</v>
+        <v>1200</v>
       </c>
       <c r="K13" s="3" t="s">
         <v>446</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>1176</v>
+        <v>1204</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>1175</v>
+        <v>1203</v>
       </c>
       <c r="N13" s="3" t="s">
-        <v>1141</v>
+        <v>1169</v>
       </c>
       <c r="O13" s="8">
         <v>2000</v>
@@ -31993,7 +32383,7 @@
         <v>51</v>
       </c>
       <c r="Y13" s="3" t="s">
-        <v>1268</v>
+        <v>1289</v>
       </c>
       <c r="Z13" s="3" t="s">
         <v>0</v>
@@ -32031,13 +32421,13 @@
     </row>
     <row r="14" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>1267</v>
+        <v>1288</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>1267</v>
+        <v>1288</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D14" s="4">
         <v>46042</v>
@@ -32061,16 +32451,16 @@
         <v>294</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>1111</v>
+        <v>1139</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>1235</v>
+        <v>1259</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>1234</v>
+        <v>1258</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>1108</v>
+        <v>1136</v>
       </c>
       <c r="O14" s="5">
         <v>6000</v>
@@ -32094,16 +32484,16 @@
         <v>12873.6</v>
       </c>
       <c r="V14" s="2" t="s">
-        <v>1266</v>
+        <v>1287</v>
       </c>
       <c r="W14" s="2" t="s">
-        <v>1265</v>
+        <v>1286</v>
       </c>
       <c r="X14" s="2" t="s">
         <v>51</v>
       </c>
       <c r="Y14" s="2" t="s">
-        <v>1264</v>
+        <v>1285</v>
       </c>
       <c r="Z14" s="2" t="s">
         <v>0</v>
@@ -32118,10 +32508,10 @@
         <v>298</v>
       </c>
       <c r="AD14" s="2" t="s">
-        <v>1106</v>
+        <v>1134</v>
       </c>
       <c r="AE14" s="2" t="s">
-        <v>1105</v>
+        <v>1133</v>
       </c>
       <c r="AF14" s="2" t="s">
         <v>77</v>
@@ -32141,13 +32531,13 @@
     </row>
     <row r="15" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>1263</v>
+        <v>1284</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>1263</v>
+        <v>1284</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D15" s="7">
         <v>46042</v>
@@ -32159,10 +32549,10 @@
         <v>212</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>1210</v>
+        <v>1234</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>1209</v>
+        <v>1089</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>139</v>
@@ -32213,7 +32603,7 @@
         <v>87</v>
       </c>
       <c r="Y15" s="3" t="s">
-        <v>1262</v>
+        <v>1283</v>
       </c>
       <c r="Z15" s="3" t="s">
         <v>0</v>
@@ -32234,7 +32624,7 @@
         <v>518</v>
       </c>
       <c r="AF15" s="3" t="s">
-        <v>1230</v>
+        <v>1254</v>
       </c>
       <c r="AG15" s="9">
         <v>0</v>
@@ -32251,13 +32641,13 @@
     </row>
     <row r="16" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>1263</v>
+        <v>1284</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>1263</v>
+        <v>1284</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D16" s="4">
         <v>46042</v>
@@ -32269,10 +32659,10 @@
         <v>212</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>1210</v>
+        <v>1234</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>1209</v>
+        <v>1089</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>139</v>
@@ -32323,7 +32713,7 @@
         <v>87</v>
       </c>
       <c r="Y16" s="2" t="s">
-        <v>1262</v>
+        <v>1283</v>
       </c>
       <c r="Z16" s="2" t="s">
         <v>0</v>
@@ -32344,7 +32734,7 @@
         <v>518</v>
       </c>
       <c r="AF16" s="2" t="s">
-        <v>1230</v>
+        <v>1254</v>
       </c>
       <c r="AG16" s="6">
         <v>0</v>
@@ -32361,13 +32751,13 @@
     </row>
     <row r="17" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
-        <v>1261</v>
+        <v>1282</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>1261</v>
+        <v>1282</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D17" s="7">
         <v>46043</v>
@@ -32394,13 +32784,13 @@
         <v>417</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>1180</v>
+        <v>1208</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>1179</v>
+        <v>1207</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>1178</v>
+        <v>1206</v>
       </c>
       <c r="O17" s="8">
         <v>1000</v>
@@ -32433,7 +32823,7 @@
         <v>51</v>
       </c>
       <c r="Y17" s="3" t="s">
-        <v>1260</v>
+        <v>1281</v>
       </c>
       <c r="Z17" s="3" t="s">
         <v>0</v>
@@ -32471,28 +32861,28 @@
     </row>
     <row r="18" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>1248</v>
+        <v>1269</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>1248</v>
+        <v>1269</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D18" s="4">
         <v>46045</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>1247</v>
+        <v>1097</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>1246</v>
+        <v>1096</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>1186</v>
+        <v>1095</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>1185</v>
+        <v>1094</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>139</v>
@@ -32504,13 +32894,13 @@
         <v>628</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>1259</v>
+        <v>1280</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>1258</v>
+        <v>1279</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>1257</v>
+        <v>1278</v>
       </c>
       <c r="O18" s="5">
         <v>2000</v>
@@ -32534,16 +32924,16 @@
         <v>0</v>
       </c>
       <c r="V18" s="2" t="s">
-        <v>1242</v>
+        <v>1090</v>
       </c>
       <c r="W18" s="2" t="s">
-        <v>1209</v>
+        <v>1089</v>
       </c>
       <c r="X18" s="2" t="s">
         <v>87</v>
       </c>
       <c r="Y18" s="2" t="s">
-        <v>1241</v>
+        <v>1265</v>
       </c>
       <c r="Z18" s="2" t="s">
         <v>0</v>
@@ -32581,28 +32971,28 @@
     </row>
     <row r="19" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
-        <v>1248</v>
+        <v>1269</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>1248</v>
+        <v>1269</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D19" s="7">
         <v>46045</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>1247</v>
+        <v>1097</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>1246</v>
+        <v>1096</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>1186</v>
+        <v>1095</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>1185</v>
+        <v>1094</v>
       </c>
       <c r="I19" s="3" t="s">
         <v>139</v>
@@ -32614,13 +33004,13 @@
         <v>631</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>1256</v>
+        <v>1277</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>1255</v>
+        <v>1276</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>1243</v>
+        <v>1266</v>
       </c>
       <c r="O19" s="8">
         <v>11725</v>
@@ -32644,16 +33034,16 @@
         <v>0</v>
       </c>
       <c r="V19" s="3" t="s">
-        <v>1242</v>
+        <v>1090</v>
       </c>
       <c r="W19" s="3" t="s">
-        <v>1209</v>
+        <v>1089</v>
       </c>
       <c r="X19" s="3" t="s">
         <v>87</v>
       </c>
       <c r="Y19" s="3" t="s">
-        <v>1241</v>
+        <v>1265</v>
       </c>
       <c r="Z19" s="3" t="s">
         <v>0</v>
@@ -32691,28 +33081,28 @@
     </row>
     <row r="20" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>1248</v>
+        <v>1269</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>1248</v>
+        <v>1269</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D20" s="4">
         <v>46045</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>1247</v>
+        <v>1097</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>1246</v>
+        <v>1096</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>1186</v>
+        <v>1095</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>1185</v>
+        <v>1094</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>139</v>
@@ -32724,13 +33114,13 @@
         <v>632</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>1167</v>
+        <v>1195</v>
       </c>
       <c r="M20" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>1166</v>
+        <v>1194</v>
       </c>
       <c r="O20" s="5">
         <v>2925</v>
@@ -32754,16 +33144,16 @@
         <v>0</v>
       </c>
       <c r="V20" s="2" t="s">
-        <v>1242</v>
+        <v>1090</v>
       </c>
       <c r="W20" s="2" t="s">
-        <v>1209</v>
+        <v>1089</v>
       </c>
       <c r="X20" s="2" t="s">
         <v>87</v>
       </c>
       <c r="Y20" s="2" t="s">
-        <v>1241</v>
+        <v>1265</v>
       </c>
       <c r="Z20" s="2" t="s">
         <v>0</v>
@@ -32801,28 +33191,28 @@
     </row>
     <row r="21" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
-        <v>1248</v>
+        <v>1269</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>1248</v>
+        <v>1269</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D21" s="7">
         <v>46045</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>1247</v>
+        <v>1097</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>1246</v>
+        <v>1096</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>1186</v>
+        <v>1095</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>1185</v>
+        <v>1094</v>
       </c>
       <c r="I21" s="3" t="s">
         <v>139</v>
@@ -32834,13 +33224,13 @@
         <v>633</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>1119</v>
+        <v>1147</v>
       </c>
       <c r="M21" s="3" t="s">
         <v>652</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>1118</v>
+        <v>1146</v>
       </c>
       <c r="O21" s="8">
         <v>2925</v>
@@ -32864,16 +33254,16 @@
         <v>0</v>
       </c>
       <c r="V21" s="3" t="s">
-        <v>1242</v>
+        <v>1090</v>
       </c>
       <c r="W21" s="3" t="s">
-        <v>1209</v>
+        <v>1089</v>
       </c>
       <c r="X21" s="3" t="s">
         <v>87</v>
       </c>
       <c r="Y21" s="3" t="s">
-        <v>1241</v>
+        <v>1265</v>
       </c>
       <c r="Z21" s="3" t="s">
         <v>0</v>
@@ -32911,28 +33301,28 @@
     </row>
     <row r="22" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>1248</v>
+        <v>1269</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>1248</v>
+        <v>1269</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D22" s="4">
         <v>46045</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>1247</v>
+        <v>1097</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>1246</v>
+        <v>1096</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>1186</v>
+        <v>1095</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>1185</v>
+        <v>1094</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>139</v>
@@ -32944,13 +33334,13 @@
         <v>465</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>1254</v>
+        <v>1275</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>1253</v>
+        <v>1274</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>1252</v>
+        <v>1273</v>
       </c>
       <c r="O22" s="5">
         <v>2400</v>
@@ -32974,16 +33364,16 @@
         <v>0</v>
       </c>
       <c r="V22" s="2" t="s">
-        <v>1242</v>
+        <v>1090</v>
       </c>
       <c r="W22" s="2" t="s">
-        <v>1209</v>
+        <v>1089</v>
       </c>
       <c r="X22" s="2" t="s">
         <v>87</v>
       </c>
       <c r="Y22" s="2" t="s">
-        <v>1241</v>
+        <v>1265</v>
       </c>
       <c r="Z22" s="2" t="s">
         <v>0</v>
@@ -33021,28 +33411,28 @@
     </row>
     <row r="23" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
-        <v>1248</v>
+        <v>1269</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>1248</v>
+        <v>1269</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D23" s="7">
         <v>46045</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>1247</v>
+        <v>1097</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>1246</v>
+        <v>1096</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>1186</v>
+        <v>1095</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>1185</v>
+        <v>1094</v>
       </c>
       <c r="I23" s="3" t="s">
         <v>139</v>
@@ -33054,13 +33444,13 @@
         <v>465</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>1251</v>
+        <v>1272</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>1250</v>
+        <v>1271</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>1249</v>
+        <v>1270</v>
       </c>
       <c r="O23" s="8">
         <v>1800</v>
@@ -33084,16 +33474,16 @@
         <v>0</v>
       </c>
       <c r="V23" s="3" t="s">
-        <v>1242</v>
+        <v>1090</v>
       </c>
       <c r="W23" s="3" t="s">
-        <v>1209</v>
+        <v>1089</v>
       </c>
       <c r="X23" s="3" t="s">
         <v>87</v>
       </c>
       <c r="Y23" s="3" t="s">
-        <v>1241</v>
+        <v>1265</v>
       </c>
       <c r="Z23" s="3" t="s">
         <v>0</v>
@@ -33131,28 +33521,28 @@
     </row>
     <row r="24" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>1248</v>
+        <v>1269</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>1248</v>
+        <v>1269</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D24" s="4">
         <v>46045</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>1247</v>
+        <v>1097</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>1246</v>
+        <v>1096</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>1186</v>
+        <v>1095</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>1185</v>
+        <v>1094</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>139</v>
@@ -33164,13 +33554,13 @@
         <v>634</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>1245</v>
+        <v>1268</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>1244</v>
+        <v>1267</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>1243</v>
+        <v>1266</v>
       </c>
       <c r="O24" s="5">
         <v>1400</v>
@@ -33194,16 +33584,16 @@
         <v>0</v>
       </c>
       <c r="V24" s="2" t="s">
-        <v>1242</v>
+        <v>1090</v>
       </c>
       <c r="W24" s="2" t="s">
-        <v>1209</v>
+        <v>1089</v>
       </c>
       <c r="X24" s="2" t="s">
         <v>87</v>
       </c>
       <c r="Y24" s="2" t="s">
-        <v>1241</v>
+        <v>1265</v>
       </c>
       <c r="Z24" s="2" t="s">
         <v>0</v>
@@ -33241,13 +33631,13 @@
     </row>
     <row r="25" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
-        <v>1240</v>
+        <v>1264</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>1240</v>
+        <v>1264</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D25" s="7">
         <v>46048</v>
@@ -33274,13 +33664,13 @@
         <v>417</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>1192</v>
+        <v>1217</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>1191</v>
+        <v>1216</v>
       </c>
       <c r="N25" s="3" t="s">
-        <v>1190</v>
+        <v>1106</v>
       </c>
       <c r="O25" s="8">
         <v>5000</v>
@@ -33304,16 +33694,16 @@
         <v>2354</v>
       </c>
       <c r="V25" s="3" t="s">
-        <v>1086</v>
+        <v>1117</v>
       </c>
       <c r="W25" s="3" t="s">
-        <v>1085</v>
+        <v>1116</v>
       </c>
       <c r="X25" s="3" t="s">
         <v>51</v>
       </c>
       <c r="Y25" s="3" t="s">
-        <v>1239</v>
+        <v>1263</v>
       </c>
       <c r="Z25" s="3" t="s">
         <v>0</v>
@@ -33351,13 +33741,13 @@
     </row>
     <row r="26" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>1238</v>
+        <v>1262</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>1238</v>
+        <v>1262</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D26" s="4">
         <v>46048</v>
@@ -33369,10 +33759,10 @@
         <v>40</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>1081</v>
+        <v>1113</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>1080</v>
+        <v>1112</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>139</v>
@@ -33384,13 +33774,13 @@
         <v>784</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>1079</v>
+        <v>1111</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>1078</v>
+        <v>1110</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>1077</v>
+        <v>1109</v>
       </c>
       <c r="O26" s="5">
         <v>300</v>
@@ -33423,7 +33813,7 @@
         <v>51</v>
       </c>
       <c r="Y26" s="2" t="s">
-        <v>1237</v>
+        <v>1261</v>
       </c>
       <c r="Z26" s="2" t="s">
         <v>0</v>
@@ -33461,13 +33851,13 @@
     </row>
     <row r="27" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
-        <v>1236</v>
+        <v>1260</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>1236</v>
+        <v>1260</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D27" s="7">
         <v>46048</v>
@@ -33479,10 +33869,10 @@
         <v>61</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>1169</v>
+        <v>1197</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>1168</v>
+        <v>1196</v>
       </c>
       <c r="I27" s="3" t="s">
         <v>163</v>
@@ -33494,13 +33884,13 @@
         <v>632</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>1167</v>
+        <v>1195</v>
       </c>
       <c r="M27" s="3" t="s">
         <v>648</v>
       </c>
       <c r="N27" s="3" t="s">
-        <v>1166</v>
+        <v>1194</v>
       </c>
       <c r="O27" s="8">
         <v>611</v>
@@ -33533,7 +33923,7 @@
         <v>51</v>
       </c>
       <c r="Y27" s="3" t="s">
-        <v>1233</v>
+        <v>1257</v>
       </c>
       <c r="Z27" s="3" t="s">
         <v>0</v>
@@ -33571,13 +33961,13 @@
     </row>
     <row r="28" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>1236</v>
+        <v>1260</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>1236</v>
+        <v>1260</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D28" s="4">
         <v>46048</v>
@@ -33589,10 +33979,10 @@
         <v>61</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>1169</v>
+        <v>1197</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>1168</v>
+        <v>1196</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>163</v>
@@ -33601,16 +33991,16 @@
         <v>164</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>1111</v>
+        <v>1139</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>1235</v>
+        <v>1259</v>
       </c>
       <c r="M28" s="2" t="s">
-        <v>1234</v>
+        <v>1258</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>1108</v>
+        <v>1136</v>
       </c>
       <c r="O28" s="5">
         <v>700</v>
@@ -33643,7 +34033,7 @@
         <v>51</v>
       </c>
       <c r="Y28" s="2" t="s">
-        <v>1233</v>
+        <v>1257</v>
       </c>
       <c r="Z28" s="2" t="s">
         <v>0</v>
@@ -33658,10 +34048,10 @@
         <v>55</v>
       </c>
       <c r="AD28" s="2" t="s">
-        <v>1106</v>
+        <v>1134</v>
       </c>
       <c r="AE28" s="2" t="s">
-        <v>1105</v>
+        <v>1133</v>
       </c>
       <c r="AF28" s="2" t="s">
         <v>77</v>
@@ -33681,13 +34071,13 @@
     </row>
     <row r="29" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
-        <v>1232</v>
+        <v>1256</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>1232</v>
+        <v>1256</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D29" s="7">
         <v>46048</v>
@@ -33699,10 +34089,10 @@
         <v>212</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>1210</v>
+        <v>1234</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>1209</v>
+        <v>1089</v>
       </c>
       <c r="I29" s="3" t="s">
         <v>139</v>
@@ -33753,7 +34143,7 @@
         <v>87</v>
       </c>
       <c r="Y29" s="3" t="s">
-        <v>1231</v>
+        <v>1255</v>
       </c>
       <c r="Z29" s="3" t="s">
         <v>0</v>
@@ -33774,7 +34164,7 @@
         <v>57</v>
       </c>
       <c r="AF29" s="3" t="s">
-        <v>1230</v>
+        <v>1254</v>
       </c>
       <c r="AG29" s="9">
         <v>0</v>
@@ -33791,13 +34181,13 @@
     </row>
     <row r="30" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>1229</v>
+        <v>1253</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>1229</v>
+        <v>1253</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D30" s="4">
         <v>46049</v>
@@ -33809,10 +34199,10 @@
         <v>212</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>1210</v>
+        <v>1234</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>1209</v>
+        <v>1089</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>139</v>
@@ -33863,7 +34253,7 @@
         <v>87</v>
       </c>
       <c r="Y30" s="2" t="s">
-        <v>1228</v>
+        <v>1252</v>
       </c>
       <c r="Z30" s="2" t="s">
         <v>0</v>
@@ -33901,13 +34291,13 @@
     </row>
     <row r="31" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
-        <v>1229</v>
+        <v>1253</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>1229</v>
+        <v>1253</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D31" s="7">
         <v>46049</v>
@@ -33919,10 +34309,10 @@
         <v>212</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>1210</v>
+        <v>1234</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>1209</v>
+        <v>1089</v>
       </c>
       <c r="I31" s="3" t="s">
         <v>139</v>
@@ -33973,7 +34363,7 @@
         <v>87</v>
       </c>
       <c r="Y31" s="3" t="s">
-        <v>1228</v>
+        <v>1252</v>
       </c>
       <c r="Z31" s="3" t="s">
         <v>0</v>
@@ -34011,13 +34401,13 @@
     </row>
     <row r="32" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>1225</v>
+        <v>1249</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>1225</v>
+        <v>1249</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D32" s="4">
         <v>46050</v>
@@ -34035,22 +34425,22 @@
         <v>386</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>1173</v>
+        <v>1201</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>1172</v>
+        <v>1200</v>
       </c>
       <c r="K32" s="2" t="s">
         <v>446</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>1227</v>
+        <v>1251</v>
       </c>
       <c r="M32" s="2" t="s">
         <v>448</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>1226</v>
+        <v>1250</v>
       </c>
       <c r="O32" s="5">
         <v>1000</v>
@@ -34083,7 +34473,7 @@
         <v>51</v>
       </c>
       <c r="Y32" s="2" t="s">
-        <v>1224</v>
+        <v>1248</v>
       </c>
       <c r="Z32" s="2" t="s">
         <v>0</v>
@@ -34121,13 +34511,13 @@
     </row>
     <row r="33" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
-        <v>1225</v>
+        <v>1249</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>1225</v>
+        <v>1249</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D33" s="7">
         <v>46050</v>
@@ -34145,22 +34535,22 @@
         <v>386</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>1173</v>
+        <v>1201</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>1172</v>
+        <v>1200</v>
       </c>
       <c r="K33" s="3" t="s">
         <v>446</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>1176</v>
+        <v>1204</v>
       </c>
       <c r="M33" s="3" t="s">
-        <v>1175</v>
+        <v>1203</v>
       </c>
       <c r="N33" s="3" t="s">
-        <v>1141</v>
+        <v>1169</v>
       </c>
       <c r="O33" s="8">
         <v>1000</v>
@@ -34193,7 +34583,7 @@
         <v>51</v>
       </c>
       <c r="Y33" s="3" t="s">
-        <v>1224</v>
+        <v>1248</v>
       </c>
       <c r="Z33" s="3" t="s">
         <v>0</v>
@@ -34231,13 +34621,13 @@
     </row>
     <row r="34" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>1223</v>
+        <v>1247</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>1223</v>
+        <v>1247</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D34" s="4">
         <v>46050</v>
@@ -34249,10 +34639,10 @@
         <v>212</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>1210</v>
+        <v>1234</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>1209</v>
+        <v>1089</v>
       </c>
       <c r="I34" s="2" t="s">
         <v>139</v>
@@ -34303,7 +34693,7 @@
         <v>87</v>
       </c>
       <c r="Y34" s="2" t="s">
-        <v>1222</v>
+        <v>1246</v>
       </c>
       <c r="Z34" s="2" t="s">
         <v>0</v>
@@ -34341,13 +34731,13 @@
     </row>
     <row r="35" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
-        <v>1221</v>
+        <v>1245</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>1221</v>
+        <v>1245</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D35" s="7">
         <v>46051</v>
@@ -34359,10 +34749,10 @@
         <v>40</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>1220</v>
+        <v>1244</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>1219</v>
+        <v>1243</v>
       </c>
       <c r="I35" s="3" t="s">
         <v>43</v>
@@ -34374,13 +34764,13 @@
         <v>632</v>
       </c>
       <c r="L35" s="3" t="s">
-        <v>1167</v>
+        <v>1195</v>
       </c>
       <c r="M35" s="3" t="s">
         <v>648</v>
       </c>
       <c r="N35" s="3" t="s">
-        <v>1166</v>
+        <v>1194</v>
       </c>
       <c r="O35" s="8">
         <v>26</v>
@@ -34413,7 +34803,7 @@
         <v>51</v>
       </c>
       <c r="Y35" s="3" t="s">
-        <v>1218</v>
+        <v>1242</v>
       </c>
       <c r="Z35" s="3" t="s">
         <v>0</v>
@@ -34451,13 +34841,13 @@
     </row>
     <row r="36" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>1217</v>
+        <v>1241</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>1217</v>
+        <v>1241</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D36" s="4">
         <v>46052</v>
@@ -34469,10 +34859,10 @@
         <v>61</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>1169</v>
+        <v>1197</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>1168</v>
+        <v>1196</v>
       </c>
       <c r="I36" s="2" t="s">
         <v>163</v>
@@ -34484,13 +34874,13 @@
         <v>632</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>1167</v>
+        <v>1195</v>
       </c>
       <c r="M36" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>1166</v>
+        <v>1194</v>
       </c>
       <c r="O36" s="5">
         <v>507</v>
@@ -34523,7 +34913,7 @@
         <v>51</v>
       </c>
       <c r="Y36" s="2" t="s">
-        <v>1216</v>
+        <v>1240</v>
       </c>
       <c r="Z36" s="2" t="s">
         <v>0</v>
@@ -34561,13 +34951,13 @@
     </row>
     <row r="37" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
-        <v>1215</v>
+        <v>1239</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>1215</v>
+        <v>1239</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D37" s="7">
         <v>46052</v>
@@ -34591,16 +34981,16 @@
         <v>164</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>1116</v>
+        <v>1144</v>
       </c>
       <c r="L37" s="3" t="s">
-        <v>1135</v>
+        <v>1163</v>
       </c>
       <c r="M37" s="3" t="s">
-        <v>1134</v>
+        <v>1162</v>
       </c>
       <c r="N37" s="3" t="s">
-        <v>1113</v>
+        <v>1141</v>
       </c>
       <c r="O37" s="8">
         <v>500</v>
@@ -34633,7 +35023,7 @@
         <v>51</v>
       </c>
       <c r="Y37" s="3" t="s">
-        <v>1214</v>
+        <v>1238</v>
       </c>
       <c r="Z37" s="3" t="s">
         <v>0</v>
@@ -34671,13 +35061,13 @@
     </row>
     <row r="38" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>1213</v>
+        <v>1237</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>1213</v>
+        <v>1237</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D38" s="4">
         <v>46052</v>
@@ -34689,10 +35079,10 @@
         <v>40</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>1081</v>
+        <v>1113</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>1080</v>
+        <v>1112</v>
       </c>
       <c r="I38" s="2" t="s">
         <v>139</v>
@@ -34704,13 +35094,13 @@
         <v>784</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>1079</v>
+        <v>1111</v>
       </c>
       <c r="M38" s="2" t="s">
-        <v>1078</v>
+        <v>1110</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>1077</v>
+        <v>1109</v>
       </c>
       <c r="O38" s="5">
         <v>300</v>
@@ -34743,7 +35133,7 @@
         <v>51</v>
       </c>
       <c r="Y38" s="2" t="s">
-        <v>1212</v>
+        <v>1236</v>
       </c>
       <c r="Z38" s="2" t="s">
         <v>0</v>
@@ -34781,13 +35171,13 @@
     </row>
     <row r="39" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
-        <v>1211</v>
+        <v>1235</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>1211</v>
+        <v>1235</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D39" s="7">
         <v>46055</v>
@@ -34799,10 +35189,10 @@
         <v>212</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>1210</v>
+        <v>1234</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>1209</v>
+        <v>1089</v>
       </c>
       <c r="I39" s="3" t="s">
         <v>139</v>
@@ -34811,7 +35201,7 @@
         <v>140</v>
       </c>
       <c r="K39" s="3" t="s">
-        <v>1208</v>
+        <v>1233</v>
       </c>
       <c r="L39" s="3" t="s">
         <v>0</v>
@@ -34853,7 +35243,7 @@
         <v>87</v>
       </c>
       <c r="Y39" s="3" t="s">
-        <v>1207</v>
+        <v>1232</v>
       </c>
       <c r="Z39" s="3" t="s">
         <v>0</v>
@@ -34891,13 +35281,13 @@
     </row>
     <row r="40" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>1206</v>
+        <v>1231</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>1206</v>
+        <v>1231</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D40" s="4">
         <v>46057</v>
@@ -34909,10 +35299,10 @@
         <v>61</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>1169</v>
+        <v>1197</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>1168</v>
+        <v>1196</v>
       </c>
       <c r="I40" s="2" t="s">
         <v>163</v>
@@ -34924,13 +35314,13 @@
         <v>632</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>1167</v>
+        <v>1195</v>
       </c>
       <c r="M40" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>1166</v>
+        <v>1194</v>
       </c>
       <c r="O40" s="5">
         <v>507</v>
@@ -34963,7 +35353,7 @@
         <v>51</v>
       </c>
       <c r="Y40" s="2" t="s">
-        <v>1205</v>
+        <v>1230</v>
       </c>
       <c r="Z40" s="2" t="s">
         <v>0</v>
@@ -35001,13 +35391,13 @@
     </row>
     <row r="41" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
-        <v>1204</v>
+        <v>1229</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>1204</v>
+        <v>1229</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D41" s="7">
         <v>46057</v>
@@ -35025,22 +35415,22 @@
         <v>386</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>1173</v>
+        <v>1201</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>1172</v>
+        <v>1200</v>
       </c>
       <c r="K41" s="3" t="s">
         <v>446</v>
       </c>
       <c r="L41" s="3" t="s">
-        <v>1176</v>
+        <v>1204</v>
       </c>
       <c r="M41" s="3" t="s">
-        <v>1175</v>
+        <v>1203</v>
       </c>
       <c r="N41" s="3" t="s">
-        <v>1141</v>
+        <v>1169</v>
       </c>
       <c r="O41" s="8">
         <v>2000</v>
@@ -35073,7 +35463,7 @@
         <v>51</v>
       </c>
       <c r="Y41" s="3" t="s">
-        <v>1171</v>
+        <v>1199</v>
       </c>
       <c r="Z41" s="3" t="s">
         <v>0</v>
@@ -35111,13 +35501,13 @@
     </row>
     <row r="42" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>1203</v>
+        <v>1228</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>1203</v>
+        <v>1228</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D42" s="4">
         <v>46058</v>
@@ -35129,10 +35519,10 @@
         <v>61</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>1169</v>
+        <v>1197</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>1168</v>
+        <v>1196</v>
       </c>
       <c r="I42" s="2" t="s">
         <v>163</v>
@@ -35144,13 +35534,13 @@
         <v>632</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>1167</v>
+        <v>1195</v>
       </c>
       <c r="M42" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>1166</v>
+        <v>1194</v>
       </c>
       <c r="O42" s="5">
         <v>507</v>
@@ -35183,7 +35573,7 @@
         <v>51</v>
       </c>
       <c r="Y42" s="2" t="s">
-        <v>1202</v>
+        <v>1227</v>
       </c>
       <c r="Z42" s="2" t="s">
         <v>0</v>
@@ -35221,13 +35611,13 @@
     </row>
     <row r="43" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
-        <v>1201</v>
+        <v>1226</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>1201</v>
+        <v>1226</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D43" s="7">
         <v>46058</v>
@@ -35239,10 +35629,10 @@
         <v>61</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>1138</v>
+        <v>1166</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>1137</v>
+        <v>1165</v>
       </c>
       <c r="I43" s="3" t="s">
         <v>163</v>
@@ -35254,13 +35644,13 @@
         <v>417</v>
       </c>
       <c r="L43" s="3" t="s">
-        <v>1192</v>
+        <v>1217</v>
       </c>
       <c r="M43" s="3" t="s">
-        <v>1191</v>
+        <v>1216</v>
       </c>
       <c r="N43" s="3" t="s">
-        <v>1190</v>
+        <v>1106</v>
       </c>
       <c r="O43" s="8">
         <v>1800</v>
@@ -35293,7 +35683,7 @@
         <v>51</v>
       </c>
       <c r="Y43" s="3" t="s">
-        <v>1200</v>
+        <v>1225</v>
       </c>
       <c r="Z43" s="3" t="s">
         <v>0</v>
@@ -35331,13 +35721,13 @@
     </row>
     <row r="44" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>1199</v>
+        <v>1224</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>1199</v>
+        <v>1224</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D44" s="4">
         <v>46059</v>
@@ -35349,10 +35739,10 @@
         <v>40</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>1198</v>
+        <v>1223</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>1197</v>
+        <v>1222</v>
       </c>
       <c r="I44" s="2" t="s">
         <v>43</v>
@@ -35364,13 +35754,13 @@
         <v>784</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>1079</v>
+        <v>1111</v>
       </c>
       <c r="M44" s="2" t="s">
-        <v>1078</v>
+        <v>1110</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>1077</v>
+        <v>1109</v>
       </c>
       <c r="O44" s="5">
         <v>500</v>
@@ -35403,7 +35793,7 @@
         <v>51</v>
       </c>
       <c r="Y44" s="2" t="s">
-        <v>1196</v>
+        <v>1221</v>
       </c>
       <c r="Z44" s="2" t="s">
         <v>0</v>
@@ -35441,13 +35831,13 @@
     </row>
     <row r="45" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="3" t="s">
-        <v>1195</v>
+        <v>1220</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>1195</v>
+        <v>1220</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D45" s="7">
         <v>46059</v>
@@ -35459,10 +35849,10 @@
         <v>40</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>1194</v>
+        <v>1219</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>1193</v>
+        <v>1218</v>
       </c>
       <c r="I45" s="3" t="s">
         <v>43</v>
@@ -35474,13 +35864,13 @@
         <v>417</v>
       </c>
       <c r="L45" s="3" t="s">
-        <v>1192</v>
+        <v>1217</v>
       </c>
       <c r="M45" s="3" t="s">
-        <v>1191</v>
+        <v>1216</v>
       </c>
       <c r="N45" s="3" t="s">
-        <v>1190</v>
+        <v>1106</v>
       </c>
       <c r="O45" s="8">
         <v>200</v>
@@ -35513,7 +35903,7 @@
         <v>51</v>
       </c>
       <c r="Y45" s="3" t="s">
-        <v>1189</v>
+        <v>1215</v>
       </c>
       <c r="Z45" s="3" t="s">
         <v>0</v>
@@ -35551,28 +35941,28 @@
     </row>
     <row r="46" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
-        <v>1188</v>
+        <v>1214</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>1188</v>
+        <v>1214</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D46" s="4">
         <v>46063</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>1187</v>
+        <v>1213</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>267</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>1186</v>
+        <v>1095</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>1185</v>
+        <v>1094</v>
       </c>
       <c r="I46" s="2" t="s">
         <v>139</v>
@@ -35581,7 +35971,7 @@
         <v>140</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>1094</v>
+        <v>1122</v>
       </c>
       <c r="L46" s="2" t="s">
         <v>0</v>
@@ -35623,7 +36013,7 @@
         <v>0</v>
       </c>
       <c r="Y46" s="2" t="s">
-        <v>1184</v>
+        <v>1212</v>
       </c>
       <c r="Z46" s="2" t="s">
         <v>0</v>
@@ -35638,10 +36028,10 @@
         <v>74</v>
       </c>
       <c r="AD46" s="2" t="s">
-        <v>1092</v>
+        <v>1120</v>
       </c>
       <c r="AE46" s="2" t="s">
-        <v>1091</v>
+        <v>1119</v>
       </c>
       <c r="AF46" s="2" t="s">
         <v>0</v>
@@ -35661,13 +36051,13 @@
     </row>
     <row r="47" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
-        <v>1183</v>
+        <v>1211</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>1183</v>
+        <v>1211</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D47" s="7">
         <v>46064</v>
@@ -35679,10 +36069,10 @@
         <v>61</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>1182</v>
+        <v>1210</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>1181</v>
+        <v>1209</v>
       </c>
       <c r="I47" s="3" t="s">
         <v>139</v>
@@ -35694,13 +36084,13 @@
         <v>417</v>
       </c>
       <c r="L47" s="3" t="s">
-        <v>1180</v>
+        <v>1208</v>
       </c>
       <c r="M47" s="3" t="s">
-        <v>1179</v>
+        <v>1207</v>
       </c>
       <c r="N47" s="3" t="s">
-        <v>1178</v>
+        <v>1206</v>
       </c>
       <c r="O47" s="8">
         <v>1000</v>
@@ -35733,7 +36123,7 @@
         <v>51</v>
       </c>
       <c r="Y47" s="3" t="s">
-        <v>1177</v>
+        <v>1205</v>
       </c>
       <c r="Z47" s="3" t="s">
         <v>0</v>
@@ -35771,13 +36161,13 @@
     </row>
     <row r="48" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
-        <v>1174</v>
+        <v>1202</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>1174</v>
+        <v>1202</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D48" s="4">
         <v>46064</v>
@@ -35795,22 +36185,22 @@
         <v>386</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>1173</v>
+        <v>1201</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>1172</v>
+        <v>1200</v>
       </c>
       <c r="K48" s="2" t="s">
         <v>446</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>1176</v>
+        <v>1204</v>
       </c>
       <c r="M48" s="2" t="s">
-        <v>1175</v>
+        <v>1203</v>
       </c>
       <c r="N48" s="2" t="s">
-        <v>1141</v>
+        <v>1169</v>
       </c>
       <c r="O48" s="5">
         <v>1000</v>
@@ -35843,7 +36233,7 @@
         <v>51</v>
       </c>
       <c r="Y48" s="2" t="s">
-        <v>1171</v>
+        <v>1199</v>
       </c>
       <c r="Z48" s="2" t="s">
         <v>0</v>
@@ -35881,13 +36271,13 @@
     </row>
     <row r="49" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
-        <v>1174</v>
+        <v>1202</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>1174</v>
+        <v>1202</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D49" s="7">
         <v>46064</v>
@@ -35905,22 +36295,22 @@
         <v>386</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>1173</v>
+        <v>1201</v>
       </c>
       <c r="J49" s="3" t="s">
-        <v>1172</v>
+        <v>1200</v>
       </c>
       <c r="K49" s="3" t="s">
         <v>446</v>
       </c>
       <c r="L49" s="3" t="s">
-        <v>1143</v>
+        <v>1171</v>
       </c>
       <c r="M49" s="3" t="s">
-        <v>1142</v>
+        <v>1170</v>
       </c>
       <c r="N49" s="3" t="s">
-        <v>1141</v>
+        <v>1169</v>
       </c>
       <c r="O49" s="8">
         <v>1000</v>
@@ -35953,7 +36343,7 @@
         <v>51</v>
       </c>
       <c r="Y49" s="3" t="s">
-        <v>1171</v>
+        <v>1199</v>
       </c>
       <c r="Z49" s="3" t="s">
         <v>0</v>
@@ -35991,13 +36381,13 @@
     </row>
     <row r="50" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
-        <v>1170</v>
+        <v>1198</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>1170</v>
+        <v>1198</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D50" s="4">
         <v>46066</v>
@@ -36009,10 +36399,10 @@
         <v>61</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>1169</v>
+        <v>1197</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>1168</v>
+        <v>1196</v>
       </c>
       <c r="I50" s="2" t="s">
         <v>163</v>
@@ -36024,13 +36414,13 @@
         <v>632</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>1167</v>
+        <v>1195</v>
       </c>
       <c r="M50" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N50" s="2" t="s">
-        <v>1166</v>
+        <v>1194</v>
       </c>
       <c r="O50" s="5">
         <v>507</v>
@@ -36063,7 +36453,7 @@
         <v>51</v>
       </c>
       <c r="Y50" s="2" t="s">
-        <v>1165</v>
+        <v>1193</v>
       </c>
       <c r="Z50" s="2" t="s">
         <v>0</v>
@@ -36101,13 +36491,13 @@
     </row>
     <row r="51" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
-        <v>1164</v>
+        <v>1192</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>1164</v>
+        <v>1192</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D51" s="7">
         <v>46071</v>
@@ -36131,16 +36521,16 @@
         <v>164</v>
       </c>
       <c r="K51" s="3" t="s">
-        <v>1111</v>
+        <v>1139</v>
       </c>
       <c r="L51" s="3" t="s">
-        <v>1163</v>
+        <v>1191</v>
       </c>
       <c r="M51" s="3" t="s">
-        <v>1162</v>
+        <v>1190</v>
       </c>
       <c r="N51" s="3" t="s">
-        <v>1161</v>
+        <v>1189</v>
       </c>
       <c r="O51" s="8">
         <v>500</v>
@@ -36173,7 +36563,7 @@
         <v>51</v>
       </c>
       <c r="Y51" s="3" t="s">
-        <v>1160</v>
+        <v>1188</v>
       </c>
       <c r="Z51" s="3" t="s">
         <v>0</v>
@@ -36188,10 +36578,10 @@
         <v>111</v>
       </c>
       <c r="AD51" s="3" t="s">
-        <v>1106</v>
+        <v>1134</v>
       </c>
       <c r="AE51" s="3" t="s">
-        <v>1105</v>
+        <v>1133</v>
       </c>
       <c r="AF51" s="3" t="s">
         <v>77</v>
@@ -36211,13 +36601,13 @@
     </row>
     <row r="52" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>1159</v>
+        <v>1187</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>1159</v>
+        <v>1187</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D52" s="4">
         <v>46071</v>
@@ -36229,10 +36619,10 @@
         <v>61</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>1158</v>
+        <v>1186</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>1157</v>
+        <v>1185</v>
       </c>
       <c r="I52" s="2" t="s">
         <v>139</v>
@@ -36244,13 +36634,13 @@
         <v>446</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>1143</v>
+        <v>1171</v>
       </c>
       <c r="M52" s="2" t="s">
-        <v>1142</v>
+        <v>1170</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>1141</v>
+        <v>1169</v>
       </c>
       <c r="O52" s="5">
         <v>200</v>
@@ -36283,7 +36673,7 @@
         <v>51</v>
       </c>
       <c r="Y52" s="2" t="s">
-        <v>1156</v>
+        <v>1184</v>
       </c>
       <c r="Z52" s="2" t="s">
         <v>0</v>
@@ -36321,13 +36711,13 @@
     </row>
     <row r="53" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
-        <v>1155</v>
+        <v>1183</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>1155</v>
+        <v>1183</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D53" s="7">
         <v>46072</v>
@@ -36339,10 +36729,10 @@
         <v>40</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>1096</v>
+        <v>1124</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>1095</v>
+        <v>1123</v>
       </c>
       <c r="I53" s="3" t="s">
         <v>43</v>
@@ -36354,13 +36744,13 @@
         <v>440</v>
       </c>
       <c r="L53" s="3" t="s">
-        <v>1154</v>
+        <v>1182</v>
       </c>
       <c r="M53" s="3" t="s">
-        <v>1153</v>
+        <v>1181</v>
       </c>
       <c r="N53" s="3" t="s">
-        <v>1152</v>
+        <v>1180</v>
       </c>
       <c r="O53" s="8">
         <v>50</v>
@@ -36384,16 +36774,16 @@
         <v>0</v>
       </c>
       <c r="V53" s="3" t="s">
-        <v>1151</v>
+        <v>1179</v>
       </c>
       <c r="W53" s="3" t="s">
-        <v>1150</v>
+        <v>1178</v>
       </c>
       <c r="X53" s="3" t="s">
         <v>51</v>
       </c>
       <c r="Y53" s="3" t="s">
-        <v>1149</v>
+        <v>1177</v>
       </c>
       <c r="Z53" s="3" t="s">
         <v>0</v>
@@ -36431,13 +36821,13 @@
     </row>
     <row r="54" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>1148</v>
+        <v>1176</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>1148</v>
+        <v>1176</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D54" s="4">
         <v>46072</v>
@@ -36449,10 +36839,10 @@
         <v>61</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>1138</v>
+        <v>1166</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>1137</v>
+        <v>1165</v>
       </c>
       <c r="I54" s="2" t="s">
         <v>163</v>
@@ -36464,13 +36854,13 @@
         <v>417</v>
       </c>
       <c r="L54" s="2" t="s">
-        <v>1128</v>
+        <v>1156</v>
       </c>
       <c r="M54" s="2" t="s">
-        <v>1127</v>
+        <v>1155</v>
       </c>
       <c r="N54" s="2" t="s">
-        <v>1087</v>
+        <v>1103</v>
       </c>
       <c r="O54" s="5">
         <v>1600</v>
@@ -36503,7 +36893,7 @@
         <v>51</v>
       </c>
       <c r="Y54" s="2" t="s">
-        <v>1147</v>
+        <v>1175</v>
       </c>
       <c r="Z54" s="2" t="s">
         <v>0</v>
@@ -36541,13 +36931,13 @@
     </row>
     <row r="55" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
-        <v>1146</v>
+        <v>1174</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>1146</v>
+        <v>1174</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D55" s="7">
         <v>46072</v>
@@ -36559,10 +36949,10 @@
         <v>40</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>1145</v>
+        <v>1173</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>1144</v>
+        <v>1172</v>
       </c>
       <c r="I55" s="3" t="s">
         <v>43</v>
@@ -36574,13 +36964,13 @@
         <v>446</v>
       </c>
       <c r="L55" s="3" t="s">
-        <v>1143</v>
+        <v>1171</v>
       </c>
       <c r="M55" s="3" t="s">
-        <v>1142</v>
+        <v>1170</v>
       </c>
       <c r="N55" s="3" t="s">
-        <v>1141</v>
+        <v>1169</v>
       </c>
       <c r="O55" s="8">
         <v>500</v>
@@ -36613,7 +37003,7 @@
         <v>51</v>
       </c>
       <c r="Y55" s="3" t="s">
-        <v>1140</v>
+        <v>1168</v>
       </c>
       <c r="Z55" s="3" t="s">
         <v>0</v>
@@ -36651,13 +37041,13 @@
     </row>
     <row r="56" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
-        <v>1139</v>
+        <v>1167</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>1139</v>
+        <v>1167</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D56" s="4">
         <v>46076</v>
@@ -36669,10 +37059,10 @@
         <v>61</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>1138</v>
+        <v>1166</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>1137</v>
+        <v>1165</v>
       </c>
       <c r="I56" s="2" t="s">
         <v>163</v>
@@ -36684,13 +37074,13 @@
         <v>417</v>
       </c>
       <c r="L56" s="2" t="s">
-        <v>1128</v>
+        <v>1156</v>
       </c>
       <c r="M56" s="2" t="s">
-        <v>1127</v>
+        <v>1155</v>
       </c>
       <c r="N56" s="2" t="s">
-        <v>1087</v>
+        <v>1103</v>
       </c>
       <c r="O56" s="5">
         <v>1700</v>
@@ -36723,7 +37113,7 @@
         <v>51</v>
       </c>
       <c r="Y56" s="2" t="s">
-        <v>1136</v>
+        <v>1164</v>
       </c>
       <c r="Z56" s="2" t="s">
         <v>0</v>
@@ -36761,13 +37151,13 @@
     </row>
     <row r="57" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
-        <v>1133</v>
+        <v>1161</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>1133</v>
+        <v>1161</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D57" s="7">
         <v>46077</v>
@@ -36791,16 +37181,16 @@
         <v>164</v>
       </c>
       <c r="K57" s="3" t="s">
-        <v>1116</v>
+        <v>1144</v>
       </c>
       <c r="L57" s="3" t="s">
-        <v>1135</v>
+        <v>1163</v>
       </c>
       <c r="M57" s="3" t="s">
-        <v>1134</v>
+        <v>1162</v>
       </c>
       <c r="N57" s="3" t="s">
-        <v>1113</v>
+        <v>1141</v>
       </c>
       <c r="O57" s="8">
         <v>500</v>
@@ -36833,7 +37223,7 @@
         <v>51</v>
       </c>
       <c r="Y57" s="3" t="s">
-        <v>1132</v>
+        <v>1160</v>
       </c>
       <c r="Z57" s="3" t="s">
         <v>0</v>
@@ -36871,13 +37261,13 @@
     </row>
     <row r="58" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
-        <v>1133</v>
+        <v>1161</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>1133</v>
+        <v>1161</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D58" s="4">
         <v>46077</v>
@@ -36901,16 +37291,16 @@
         <v>164</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>1111</v>
+        <v>1139</v>
       </c>
       <c r="L58" s="2" t="s">
-        <v>1110</v>
+        <v>1138</v>
       </c>
       <c r="M58" s="2" t="s">
-        <v>1109</v>
+        <v>1137</v>
       </c>
       <c r="N58" s="2" t="s">
-        <v>1108</v>
+        <v>1136</v>
       </c>
       <c r="O58" s="5">
         <v>500</v>
@@ -36943,7 +37333,7 @@
         <v>51</v>
       </c>
       <c r="Y58" s="2" t="s">
-        <v>1132</v>
+        <v>1160</v>
       </c>
       <c r="Z58" s="2" t="s">
         <v>0</v>
@@ -36958,10 +37348,10 @@
         <v>111</v>
       </c>
       <c r="AD58" s="2" t="s">
-        <v>1106</v>
+        <v>1134</v>
       </c>
       <c r="AE58" s="2" t="s">
-        <v>1105</v>
+        <v>1133</v>
       </c>
       <c r="AF58" s="2" t="s">
         <v>77</v>
@@ -36981,13 +37371,13 @@
     </row>
     <row r="59" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
-        <v>1131</v>
+        <v>1159</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>1131</v>
+        <v>1159</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D59" s="7">
         <v>46078</v>
@@ -36999,10 +37389,10 @@
         <v>40</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>1081</v>
+        <v>1113</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>1080</v>
+        <v>1112</v>
       </c>
       <c r="I59" s="3" t="s">
         <v>139</v>
@@ -37014,13 +37404,13 @@
         <v>784</v>
       </c>
       <c r="L59" s="3" t="s">
-        <v>1079</v>
+        <v>1111</v>
       </c>
       <c r="M59" s="3" t="s">
-        <v>1078</v>
+        <v>1110</v>
       </c>
       <c r="N59" s="3" t="s">
-        <v>1077</v>
+        <v>1109</v>
       </c>
       <c r="O59" s="8">
         <v>225</v>
@@ -37053,7 +37443,7 @@
         <v>51</v>
       </c>
       <c r="Y59" s="3" t="s">
-        <v>1130</v>
+        <v>1158</v>
       </c>
       <c r="Z59" s="3" t="s">
         <v>0</v>
@@ -37091,13 +37481,13 @@
     </row>
     <row r="60" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
-        <v>1129</v>
+        <v>1157</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>1129</v>
+        <v>1157</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D60" s="4">
         <v>46079</v>
@@ -37124,13 +37514,13 @@
         <v>417</v>
       </c>
       <c r="L60" s="2" t="s">
-        <v>1128</v>
+        <v>1156</v>
       </c>
       <c r="M60" s="2" t="s">
-        <v>1127</v>
+        <v>1155</v>
       </c>
       <c r="N60" s="2" t="s">
-        <v>1087</v>
+        <v>1103</v>
       </c>
       <c r="O60" s="5">
         <v>5000</v>
@@ -37154,16 +37544,16 @@
         <v>2354</v>
       </c>
       <c r="V60" s="2" t="s">
-        <v>1086</v>
+        <v>1117</v>
       </c>
       <c r="W60" s="2" t="s">
-        <v>1085</v>
+        <v>1116</v>
       </c>
       <c r="X60" s="2" t="s">
         <v>51</v>
       </c>
       <c r="Y60" s="2" t="s">
-        <v>1126</v>
+        <v>1154</v>
       </c>
       <c r="Z60" s="2" t="s">
         <v>0</v>
@@ -37201,13 +37591,13 @@
     </row>
     <row r="61" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
-        <v>1125</v>
+        <v>1153</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>1125</v>
+        <v>1153</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D61" s="7">
         <v>46079</v>
@@ -37234,13 +37624,13 @@
         <v>1060</v>
       </c>
       <c r="L61" s="3" t="s">
-        <v>1124</v>
+        <v>1152</v>
       </c>
       <c r="M61" s="3" t="s">
-        <v>1123</v>
+        <v>1151</v>
       </c>
       <c r="N61" s="3" t="s">
-        <v>1122</v>
+        <v>1150</v>
       </c>
       <c r="O61" s="8">
         <v>12000</v>
@@ -37273,7 +37663,7 @@
         <v>51</v>
       </c>
       <c r="Y61" s="3" t="s">
-        <v>1121</v>
+        <v>1149</v>
       </c>
       <c r="Z61" s="3" t="s">
         <v>0</v>
@@ -37311,13 +37701,13 @@
     </row>
     <row r="62" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
-        <v>1120</v>
+        <v>1148</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>1120</v>
+        <v>1148</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D62" s="4">
         <v>46085</v>
@@ -37344,13 +37734,13 @@
         <v>633</v>
       </c>
       <c r="L62" s="2" t="s">
-        <v>1119</v>
+        <v>1147</v>
       </c>
       <c r="M62" s="2" t="s">
         <v>652</v>
       </c>
       <c r="N62" s="2" t="s">
-        <v>1118</v>
+        <v>1146</v>
       </c>
       <c r="O62" s="5">
         <v>5005</v>
@@ -37383,7 +37773,7 @@
         <v>51</v>
       </c>
       <c r="Y62" s="2" t="s">
-        <v>1117</v>
+        <v>1145</v>
       </c>
       <c r="Z62" s="2" t="s">
         <v>0</v>
@@ -37421,13 +37811,13 @@
     </row>
     <row r="63" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
-        <v>1112</v>
+        <v>1140</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>1112</v>
+        <v>1140</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D63" s="7">
         <v>46085</v>
@@ -37451,16 +37841,16 @@
         <v>164</v>
       </c>
       <c r="K63" s="3" t="s">
-        <v>1116</v>
+        <v>1144</v>
       </c>
       <c r="L63" s="3" t="s">
-        <v>1115</v>
+        <v>1143</v>
       </c>
       <c r="M63" s="3" t="s">
-        <v>1114</v>
+        <v>1142</v>
       </c>
       <c r="N63" s="3" t="s">
-        <v>1113</v>
+        <v>1141</v>
       </c>
       <c r="O63" s="8">
         <v>500</v>
@@ -37493,7 +37883,7 @@
         <v>51</v>
       </c>
       <c r="Y63" s="3" t="s">
-        <v>1107</v>
+        <v>1135</v>
       </c>
       <c r="Z63" s="3" t="s">
         <v>0</v>
@@ -37531,13 +37921,13 @@
     </row>
     <row r="64" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
-        <v>1112</v>
+        <v>1140</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>1112</v>
+        <v>1140</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D64" s="4">
         <v>46085</v>
@@ -37561,16 +37951,16 @@
         <v>164</v>
       </c>
       <c r="K64" s="2" t="s">
-        <v>1111</v>
+        <v>1139</v>
       </c>
       <c r="L64" s="2" t="s">
-        <v>1110</v>
+        <v>1138</v>
       </c>
       <c r="M64" s="2" t="s">
-        <v>1109</v>
+        <v>1137</v>
       </c>
       <c r="N64" s="2" t="s">
-        <v>1108</v>
+        <v>1136</v>
       </c>
       <c r="O64" s="5">
         <v>500</v>
@@ -37603,7 +37993,7 @@
         <v>51</v>
       </c>
       <c r="Y64" s="2" t="s">
-        <v>1107</v>
+        <v>1135</v>
       </c>
       <c r="Z64" s="2" t="s">
         <v>0</v>
@@ -37618,10 +38008,10 @@
         <v>111</v>
       </c>
       <c r="AD64" s="2" t="s">
-        <v>1106</v>
+        <v>1134</v>
       </c>
       <c r="AE64" s="2" t="s">
-        <v>1105</v>
+        <v>1133</v>
       </c>
       <c r="AF64" s="2" t="s">
         <v>77</v>
@@ -37641,13 +38031,13 @@
     </row>
     <row r="65" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
-        <v>1104</v>
+        <v>1132</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>1104</v>
+        <v>1132</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D65" s="7">
         <v>46085</v>
@@ -37659,10 +38049,10 @@
         <v>40</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>1103</v>
+        <v>1131</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>1102</v>
+        <v>1130</v>
       </c>
       <c r="I65" s="3" t="s">
         <v>163</v>
@@ -37674,13 +38064,13 @@
         <v>154</v>
       </c>
       <c r="L65" s="3" t="s">
-        <v>1101</v>
+        <v>1129</v>
       </c>
       <c r="M65" s="3" t="s">
-        <v>1100</v>
+        <v>1128</v>
       </c>
       <c r="N65" s="3" t="s">
-        <v>1099</v>
+        <v>1127</v>
       </c>
       <c r="O65" s="8">
         <v>3700</v>
@@ -37713,7 +38103,7 @@
         <v>51</v>
       </c>
       <c r="Y65" s="3" t="s">
-        <v>1098</v>
+        <v>1126</v>
       </c>
       <c r="Z65" s="3" t="s">
         <v>0</v>
@@ -37751,13 +38141,13 @@
     </row>
     <row r="66" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
-        <v>1097</v>
+        <v>1125</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>1097</v>
+        <v>1125</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D66" s="4">
         <v>46085</v>
@@ -37769,10 +38159,10 @@
         <v>40</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>1096</v>
+        <v>1124</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>1095</v>
+        <v>1123</v>
       </c>
       <c r="I66" s="2" t="s">
         <v>139</v>
@@ -37781,7 +38171,7 @@
         <v>140</v>
       </c>
       <c r="K66" s="2" t="s">
-        <v>1094</v>
+        <v>1122</v>
       </c>
       <c r="L66" s="2" t="s">
         <v>0</v>
@@ -37823,7 +38213,7 @@
         <v>0</v>
       </c>
       <c r="Y66" s="2" t="s">
-        <v>1093</v>
+        <v>1121</v>
       </c>
       <c r="Z66" s="2" t="s">
         <v>0</v>
@@ -37838,10 +38228,10 @@
         <v>298</v>
       </c>
       <c r="AD66" s="2" t="s">
-        <v>1092</v>
+        <v>1120</v>
       </c>
       <c r="AE66" s="2" t="s">
-        <v>1091</v>
+        <v>1119</v>
       </c>
       <c r="AF66" s="2" t="s">
         <v>0</v>
@@ -37861,13 +38251,13 @@
     </row>
     <row r="67" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
-        <v>1090</v>
+        <v>1118</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>1090</v>
+        <v>1118</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D67" s="7">
         <v>46091</v>
@@ -37894,13 +38284,13 @@
         <v>417</v>
       </c>
       <c r="L67" s="3" t="s">
-        <v>1089</v>
+        <v>1105</v>
       </c>
       <c r="M67" s="3" t="s">
-        <v>1088</v>
+        <v>1104</v>
       </c>
       <c r="N67" s="3" t="s">
-        <v>1087</v>
+        <v>1103</v>
       </c>
       <c r="O67" s="8">
         <v>5000</v>
@@ -37924,16 +38314,16 @@
         <v>2354</v>
       </c>
       <c r="V67" s="3" t="s">
-        <v>1086</v>
+        <v>1117</v>
       </c>
       <c r="W67" s="3" t="s">
-        <v>1085</v>
+        <v>1116</v>
       </c>
       <c r="X67" s="3" t="s">
         <v>51</v>
       </c>
       <c r="Y67" s="3" t="s">
-        <v>1084</v>
+        <v>1115</v>
       </c>
       <c r="Z67" s="3" t="s">
         <v>0</v>
@@ -37971,13 +38361,13 @@
     </row>
     <row r="68" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
-        <v>1083</v>
+        <v>1114</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>1083</v>
+        <v>1114</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>1082</v>
+        <v>1098</v>
       </c>
       <c r="D68" s="4">
         <v>46091</v>
@@ -37989,10 +38379,10 @@
         <v>40</v>
       </c>
       <c r="G68" s="2" t="s">
-        <v>1081</v>
+        <v>1113</v>
       </c>
       <c r="H68" s="2" t="s">
-        <v>1080</v>
+        <v>1112</v>
       </c>
       <c r="I68" s="2" t="s">
         <v>139</v>
@@ -38004,13 +38394,13 @@
         <v>784</v>
       </c>
       <c r="L68" s="2" t="s">
-        <v>1079</v>
+        <v>1111</v>
       </c>
       <c r="M68" s="2" t="s">
-        <v>1078</v>
+        <v>1110</v>
       </c>
       <c r="N68" s="2" t="s">
-        <v>1077</v>
+        <v>1109</v>
       </c>
       <c r="O68" s="5">
         <v>225</v>
@@ -38043,7 +38433,7 @@
         <v>51</v>
       </c>
       <c r="Y68" s="2" t="s">
-        <v>1076</v>
+        <v>1108</v>
       </c>
       <c r="Z68" s="2" t="s">
         <v>0</v>
@@ -38077,6 +38467,446 @@
       </c>
       <c r="AJ68" s="5">
         <v>2225.1802499999999</v>
+      </c>
+    </row>
+    <row r="69" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="3" t="s">
+        <v>1099</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>1099</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>1098</v>
+      </c>
+      <c r="D69" s="7">
+        <v>46092</v>
+      </c>
+      <c r="E69" s="3" t="s">
+        <v>1097</v>
+      </c>
+      <c r="F69" s="3" t="s">
+        <v>1096</v>
+      </c>
+      <c r="G69" s="3" t="s">
+        <v>1095</v>
+      </c>
+      <c r="H69" s="3" t="s">
+        <v>1094</v>
+      </c>
+      <c r="I69" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="J69" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="K69" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="L69" s="3" t="s">
+        <v>1107</v>
+      </c>
+      <c r="M69" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="N69" s="3" t="s">
+        <v>1106</v>
+      </c>
+      <c r="O69" s="8">
+        <v>10000</v>
+      </c>
+      <c r="P69" s="8">
+        <v>8.2807300000000001</v>
+      </c>
+      <c r="Q69" s="9">
+        <v>82807.3</v>
+      </c>
+      <c r="R69" s="9">
+        <v>2691.23</v>
+      </c>
+      <c r="S69" s="9">
+        <v>85498.53</v>
+      </c>
+      <c r="T69" s="9">
+        <v>205676.76</v>
+      </c>
+      <c r="U69" s="9">
+        <v>3312.29</v>
+      </c>
+      <c r="V69" s="3" t="s">
+        <v>1090</v>
+      </c>
+      <c r="W69" s="3" t="s">
+        <v>1089</v>
+      </c>
+      <c r="X69" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y69" s="3" t="s">
+        <v>1088</v>
+      </c>
+      <c r="Z69" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA69" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB69" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="AC69" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD69" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="AE69" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="AF69" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="AG69" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH69" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI69" s="9">
+        <v>4</v>
+      </c>
+      <c r="AJ69" s="8">
+        <v>101325.9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A70" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>1098</v>
+      </c>
+      <c r="D70" s="4">
+        <v>46092</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>1097</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>1096</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>1095</v>
+      </c>
+      <c r="H70" s="2" t="s">
+        <v>1094</v>
+      </c>
+      <c r="I70" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="J70" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="K70" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="L70" s="2" t="s">
+        <v>1105</v>
+      </c>
+      <c r="M70" s="2" t="s">
+        <v>1104</v>
+      </c>
+      <c r="N70" s="2" t="s">
+        <v>1103</v>
+      </c>
+      <c r="O70" s="5">
+        <v>5000</v>
+      </c>
+      <c r="P70" s="5">
+        <v>7.7957700000000001</v>
+      </c>
+      <c r="Q70" s="6">
+        <v>38978.85</v>
+      </c>
+      <c r="R70" s="6">
+        <v>1266.81</v>
+      </c>
+      <c r="S70" s="6">
+        <v>40245.660000000003</v>
+      </c>
+      <c r="T70" s="6">
+        <v>205676.76</v>
+      </c>
+      <c r="U70" s="6">
+        <v>1559.15</v>
+      </c>
+      <c r="V70" s="2" t="s">
+        <v>1090</v>
+      </c>
+      <c r="W70" s="2" t="s">
+        <v>1089</v>
+      </c>
+      <c r="X70" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y70" s="2" t="s">
+        <v>1088</v>
+      </c>
+      <c r="Z70" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA70" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB70" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="AC70" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD70" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="AE70" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="AF70" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AG70" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH70" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI70" s="6">
+        <v>4</v>
+      </c>
+      <c r="AJ70" s="5">
+        <v>48943.45</v>
+      </c>
+    </row>
+    <row r="71" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A71" s="3" t="s">
+        <v>1099</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>1099</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>1098</v>
+      </c>
+      <c r="D71" s="7">
+        <v>46092</v>
+      </c>
+      <c r="E71" s="3" t="s">
+        <v>1097</v>
+      </c>
+      <c r="F71" s="3" t="s">
+        <v>1096</v>
+      </c>
+      <c r="G71" s="3" t="s">
+        <v>1095</v>
+      </c>
+      <c r="H71" s="3" t="s">
+        <v>1094</v>
+      </c>
+      <c r="I71" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="J71" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="K71" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="L71" s="3" t="s">
+        <v>1102</v>
+      </c>
+      <c r="M71" s="3" t="s">
+        <v>1101</v>
+      </c>
+      <c r="N71" s="3" t="s">
+        <v>1100</v>
+      </c>
+      <c r="O71" s="8">
+        <v>8400</v>
+      </c>
+      <c r="P71" s="8">
+        <v>7.6801399999999997</v>
+      </c>
+      <c r="Q71" s="9">
+        <v>64513.18</v>
+      </c>
+      <c r="R71" s="9">
+        <v>2096.6799999999998</v>
+      </c>
+      <c r="S71" s="9">
+        <v>66609.86</v>
+      </c>
+      <c r="T71" s="9">
+        <v>205676.76</v>
+      </c>
+      <c r="U71" s="9">
+        <v>2580.5300000000002</v>
+      </c>
+      <c r="V71" s="3" t="s">
+        <v>1090</v>
+      </c>
+      <c r="W71" s="3" t="s">
+        <v>1089</v>
+      </c>
+      <c r="X71" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y71" s="3" t="s">
+        <v>1088</v>
+      </c>
+      <c r="Z71" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA71" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB71" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="AC71" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD71" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="AE71" s="3" t="s">
+        <v>351</v>
+      </c>
+      <c r="AF71" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="AG71" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH71" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI71" s="9">
+        <v>4</v>
+      </c>
+      <c r="AJ71" s="8">
+        <v>70249.703999999998</v>
+      </c>
+    </row>
+    <row r="72" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A72" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>1098</v>
+      </c>
+      <c r="D72" s="4">
+        <v>46092</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>1097</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>1096</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>1095</v>
+      </c>
+      <c r="H72" s="2" t="s">
+        <v>1094</v>
+      </c>
+      <c r="I72" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="J72" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="K72" s="2" t="s">
+        <v>784</v>
+      </c>
+      <c r="L72" s="2" t="s">
+        <v>1093</v>
+      </c>
+      <c r="M72" s="2" t="s">
+        <v>1092</v>
+      </c>
+      <c r="N72" s="2" t="s">
+        <v>1091</v>
+      </c>
+      <c r="O72" s="5">
+        <v>2400</v>
+      </c>
+      <c r="P72" s="5">
+        <v>8.0739300000000007</v>
+      </c>
+      <c r="Q72" s="6">
+        <v>19377.43</v>
+      </c>
+      <c r="R72" s="6">
+        <v>629.77</v>
+      </c>
+      <c r="S72" s="6">
+        <v>20007.2</v>
+      </c>
+      <c r="T72" s="6">
+        <v>205676.76</v>
+      </c>
+      <c r="U72" s="6">
+        <v>775.1</v>
+      </c>
+      <c r="V72" s="2" t="s">
+        <v>1090</v>
+      </c>
+      <c r="W72" s="2" t="s">
+        <v>1089</v>
+      </c>
+      <c r="X72" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y72" s="2" t="s">
+        <v>1088</v>
+      </c>
+      <c r="Z72" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA72" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB72" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="AC72" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD72" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="AE72" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="AF72" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AG72" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH72" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI72" s="6">
+        <v>4</v>
+      </c>
+      <c r="AJ72" s="5">
+        <v>23735.256000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização da base de dados 13.03.2026
</commit_message>
<xml_diff>
--- a/BASE_KEMPARTS.xlsx
+++ b/BASE_KEMPARTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dash_kp_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B3665815-13D9-4495-BE2A-87C9BDF3712C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A5645B91-F09B-49FB-B37D-BD81249B5F37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{AA580DC9-C95C-4DA9-B895-704AEDCE78B9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{78875E9F-F8B2-45C9-B510-7C6062415979}"/>
   </bookViews>
   <sheets>
     <sheet name="FSP" sheetId="3" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7772" uniqueCount="1339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7797" uniqueCount="1342">
   <si>
     <t/>
   </si>
@@ -3321,6 +3321,15 @@
   </si>
   <si>
     <t>173873</t>
+  </si>
+  <si>
+    <t>000015566</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>173878</t>
   </si>
   <si>
     <t>003310</t>
@@ -4984,8 +4993,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{721A248D-7949-4F08-ACA9-1D45E33E30C7}">
-  <dimension ref="A1:AJ237"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1C22518-2E03-4AF8-94AF-81F32468EBBC}">
+  <dimension ref="A1:AJ238"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
@@ -31095,13 +31104,123 @@
         <v>0</v>
       </c>
     </row>
+    <row r="238" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A238" s="2" t="s">
+        <v>1100</v>
+      </c>
+      <c r="B238" s="2" t="s">
+        <v>1100</v>
+      </c>
+      <c r="C238" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D238" s="4">
+        <v>46094</v>
+      </c>
+      <c r="E238" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F238" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G238" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="H238" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="I238" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="J238" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="K238" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="L238" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="M238" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="N238" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="O238" s="5">
+        <v>0</v>
+      </c>
+      <c r="P238" s="5">
+        <v>2103.25</v>
+      </c>
+      <c r="Q238" s="6">
+        <v>2103.25</v>
+      </c>
+      <c r="R238" s="6">
+        <v>68.36</v>
+      </c>
+      <c r="S238" s="6">
+        <v>2171.61</v>
+      </c>
+      <c r="T238" s="6">
+        <v>2103.25</v>
+      </c>
+      <c r="U238" s="6">
+        <v>378.59</v>
+      </c>
+      <c r="V238" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="W238" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="X238" s="2" t="s">
+        <v>1101</v>
+      </c>
+      <c r="Y238" s="2" t="s">
+        <v>1102</v>
+      </c>
+      <c r="Z238" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA238" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB238" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="AC238" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD238" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE238" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="AF238" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="AG238" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH238" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AI238" s="6">
+        <v>18</v>
+      </c>
+      <c r="AJ238" s="5">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66E8590A-227B-4AA7-93BD-7C8719288B78}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26A9CA2A-55CB-4E16-8C38-D221AD8EA67E}">
   <dimension ref="A1:AJ73"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
@@ -31253,13 +31372,13 @@
     </row>
     <row r="2" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>1338</v>
+        <v>1341</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>1338</v>
+        <v>1341</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D2" s="4">
         <v>46024</v>
@@ -31271,10 +31390,10 @@
         <v>40</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>1142</v>
+        <v>1145</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>1141</v>
+        <v>1144</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>43</v>
@@ -31286,13 +31405,13 @@
         <v>440</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>1198</v>
+        <v>1201</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>1197</v>
+        <v>1200</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>1196</v>
+        <v>1199</v>
       </c>
       <c r="O2" s="5">
         <v>50</v>
@@ -31316,16 +31435,16 @@
         <v>39.06</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>1195</v>
+        <v>1198</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>1194</v>
+        <v>1197</v>
       </c>
       <c r="X2" s="2" t="s">
         <v>51</v>
       </c>
       <c r="Y2" s="2" t="s">
-        <v>1337</v>
+        <v>1340</v>
       </c>
       <c r="Z2" s="2" t="s">
         <v>0</v>
@@ -31363,13 +31482,13 @@
     </row>
     <row r="3" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>1336</v>
+        <v>1339</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>1336</v>
+        <v>1339</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D3" s="7">
         <v>46027</v>
@@ -31381,10 +31500,10 @@
         <v>61</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>1104</v>
+        <v>1107</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>1103</v>
+        <v>1106</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>163</v>
@@ -31396,13 +31515,13 @@
         <v>632</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>1211</v>
+        <v>1214</v>
       </c>
       <c r="M3" s="3" t="s">
         <v>648</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>1210</v>
+        <v>1213</v>
       </c>
       <c r="O3" s="8">
         <v>1001</v>
@@ -31435,7 +31554,7 @@
         <v>51</v>
       </c>
       <c r="Y3" s="3" t="s">
-        <v>1335</v>
+        <v>1338</v>
       </c>
       <c r="Z3" s="3" t="s">
         <v>0</v>
@@ -31473,13 +31592,13 @@
     </row>
     <row r="4" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>1334</v>
+        <v>1337</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>1334</v>
+        <v>1337</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D4" s="4">
         <v>46027</v>
@@ -31491,10 +31610,10 @@
         <v>61</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>1333</v>
+        <v>1336</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>1332</v>
+        <v>1335</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>152</v>
@@ -31506,13 +31625,13 @@
         <v>342</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>1331</v>
+        <v>1334</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>1330</v>
+        <v>1333</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>1329</v>
+        <v>1332</v>
       </c>
       <c r="O4" s="5">
         <v>600</v>
@@ -31536,16 +31655,16 @@
         <v>355.68</v>
       </c>
       <c r="V4" s="2" t="s">
-        <v>1328</v>
+        <v>1331</v>
       </c>
       <c r="W4" s="2" t="s">
-        <v>1327</v>
+        <v>1330</v>
       </c>
       <c r="X4" s="2" t="s">
         <v>51</v>
       </c>
       <c r="Y4" s="2" t="s">
-        <v>1326</v>
+        <v>1329</v>
       </c>
       <c r="Z4" s="2" t="s">
         <v>0</v>
@@ -31583,13 +31702,13 @@
     </row>
     <row r="5" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>1325</v>
+        <v>1328</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1325</v>
+        <v>1328</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D5" s="7">
         <v>46029</v>
@@ -31601,10 +31720,10 @@
         <v>212</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>1248</v>
+        <v>1251</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>139</v>
@@ -31613,7 +31732,7 @@
         <v>140</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>1324</v>
+        <v>1327</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>0</v>
@@ -31655,7 +31774,7 @@
         <v>87</v>
       </c>
       <c r="Y5" s="3" t="s">
-        <v>1323</v>
+        <v>1326</v>
       </c>
       <c r="Z5" s="3" t="s">
         <v>0</v>
@@ -31693,13 +31812,13 @@
     </row>
     <row r="6" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>1325</v>
+        <v>1328</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1325</v>
+        <v>1328</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D6" s="4">
         <v>46029</v>
@@ -31711,10 +31830,10 @@
         <v>212</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>1248</v>
+        <v>1251</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>139</v>
@@ -31723,7 +31842,7 @@
         <v>140</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>1324</v>
+        <v>1327</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>0</v>
@@ -31765,7 +31884,7 @@
         <v>87</v>
       </c>
       <c r="Y6" s="2" t="s">
-        <v>1323</v>
+        <v>1326</v>
       </c>
       <c r="Z6" s="2" t="s">
         <v>0</v>
@@ -31803,13 +31922,13 @@
     </row>
     <row r="7" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>1322</v>
+        <v>1325</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1322</v>
+        <v>1325</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D7" s="7">
         <v>46029</v>
@@ -31827,22 +31946,22 @@
         <v>386</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>1215</v>
+        <v>1218</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>1214</v>
+        <v>1217</v>
       </c>
       <c r="K7" s="3" t="s">
         <v>1058</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>1321</v>
+        <v>1324</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>1320</v>
+        <v>1323</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>1118</v>
+        <v>1121</v>
       </c>
       <c r="O7" s="8">
         <v>1000</v>
@@ -31875,7 +31994,7 @@
         <v>51</v>
       </c>
       <c r="Y7" s="3" t="s">
-        <v>1319</v>
+        <v>1322</v>
       </c>
       <c r="Z7" s="3" t="s">
         <v>0</v>
@@ -31913,13 +32032,13 @@
     </row>
     <row r="8" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>1318</v>
+        <v>1321</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>1318</v>
+        <v>1321</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D8" s="4">
         <v>46036</v>
@@ -31931,10 +32050,10 @@
         <v>61</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>1104</v>
+        <v>1107</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>1103</v>
+        <v>1106</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>163</v>
@@ -31946,13 +32065,13 @@
         <v>632</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>1211</v>
+        <v>1214</v>
       </c>
       <c r="M8" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>1210</v>
+        <v>1213</v>
       </c>
       <c r="O8" s="5">
         <v>1001</v>
@@ -31985,7 +32104,7 @@
         <v>51</v>
       </c>
       <c r="Y8" s="2" t="s">
-        <v>1317</v>
+        <v>1320</v>
       </c>
       <c r="Z8" s="2" t="s">
         <v>0</v>
@@ -32023,13 +32142,13 @@
     </row>
     <row r="9" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
-        <v>1316</v>
+        <v>1319</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1316</v>
+        <v>1319</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D9" s="7">
         <v>46037</v>
@@ -32041,10 +32160,10 @@
         <v>61</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>1224</v>
+        <v>1227</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>1223</v>
+        <v>1226</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>163</v>
@@ -32056,13 +32175,13 @@
         <v>417</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>1315</v>
+        <v>1318</v>
       </c>
       <c r="M9" s="3" t="s">
         <v>1041</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>1220</v>
+        <v>1223</v>
       </c>
       <c r="O9" s="8">
         <v>1000</v>
@@ -32095,7 +32214,7 @@
         <v>51</v>
       </c>
       <c r="Y9" s="3" t="s">
-        <v>1314</v>
+        <v>1317</v>
       </c>
       <c r="Z9" s="3" t="s">
         <v>0</v>
@@ -32133,13 +32252,13 @@
     </row>
     <row r="10" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>1313</v>
+        <v>1316</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>1313</v>
+        <v>1316</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D10" s="4">
         <v>46037</v>
@@ -32151,10 +32270,10 @@
         <v>40</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>1131</v>
+        <v>1134</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>139</v>
@@ -32166,13 +32285,13 @@
         <v>782</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>1129</v>
+        <v>1132</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>1128</v>
+        <v>1131</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>1127</v>
+        <v>1130</v>
       </c>
       <c r="O10" s="5">
         <v>300</v>
@@ -32205,7 +32324,7 @@
         <v>51</v>
       </c>
       <c r="Y10" s="2" t="s">
-        <v>1312</v>
+        <v>1315</v>
       </c>
       <c r="Z10" s="2" t="s">
         <v>0</v>
@@ -32243,13 +32362,13 @@
     </row>
     <row r="11" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>1311</v>
+        <v>1314</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>1311</v>
+        <v>1314</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D11" s="7">
         <v>46037</v>
@@ -32261,10 +32380,10 @@
         <v>40</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>1258</v>
+        <v>1261</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>1257</v>
+        <v>1260</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>43</v>
@@ -32276,13 +32395,13 @@
         <v>300</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>1310</v>
+        <v>1313</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>1309</v>
+        <v>1312</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>1308</v>
+        <v>1311</v>
       </c>
       <c r="O11" s="8">
         <v>25</v>
@@ -32315,7 +32434,7 @@
         <v>51</v>
       </c>
       <c r="Y11" s="3" t="s">
-        <v>1307</v>
+        <v>1310</v>
       </c>
       <c r="Z11" s="3" t="s">
         <v>0</v>
@@ -32353,13 +32472,13 @@
     </row>
     <row r="12" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>1306</v>
+        <v>1309</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>1306</v>
+        <v>1309</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D12" s="4">
         <v>46041</v>
@@ -32371,10 +32490,10 @@
         <v>212</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>1248</v>
+        <v>1251</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>139</v>
@@ -32383,7 +32502,7 @@
         <v>140</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>1157</v>
+        <v>1160</v>
       </c>
       <c r="L12" s="2" t="s">
         <v>0</v>
@@ -32425,7 +32544,7 @@
         <v>87</v>
       </c>
       <c r="Y12" s="2" t="s">
-        <v>1305</v>
+        <v>1308</v>
       </c>
       <c r="Z12" s="2" t="s">
         <v>0</v>
@@ -32440,10 +32559,10 @@
         <v>55</v>
       </c>
       <c r="AD12" s="2" t="s">
-        <v>1152</v>
+        <v>1155</v>
       </c>
       <c r="AE12" s="2" t="s">
-        <v>1151</v>
+        <v>1154</v>
       </c>
       <c r="AF12" s="2" t="s">
         <v>442</v>
@@ -32463,13 +32582,13 @@
     </row>
     <row r="13" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>1304</v>
+        <v>1307</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>1304</v>
+        <v>1307</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D13" s="7">
         <v>46042</v>
@@ -32487,22 +32606,22 @@
         <v>386</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>1215</v>
+        <v>1218</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>1214</v>
+        <v>1217</v>
       </c>
       <c r="K13" s="3" t="s">
         <v>446</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>1218</v>
+        <v>1221</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>1217</v>
+        <v>1220</v>
       </c>
       <c r="N13" s="3" t="s">
-        <v>1185</v>
+        <v>1188</v>
       </c>
       <c r="O13" s="8">
         <v>2000</v>
@@ -32535,7 +32654,7 @@
         <v>51</v>
       </c>
       <c r="Y13" s="3" t="s">
-        <v>1303</v>
+        <v>1306</v>
       </c>
       <c r="Z13" s="3" t="s">
         <v>0</v>
@@ -32573,13 +32692,13 @@
     </row>
     <row r="14" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>1302</v>
+        <v>1305</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>1302</v>
+        <v>1305</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D14" s="4">
         <v>46042</v>
@@ -32603,16 +32722,16 @@
         <v>294</v>
       </c>
       <c r="K14" s="2" t="s">
+        <v>1160</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>1276</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>1275</v>
+      </c>
+      <c r="N14" s="2" t="s">
         <v>1157</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>1273</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>1272</v>
-      </c>
-      <c r="N14" s="2" t="s">
-        <v>1154</v>
       </c>
       <c r="O14" s="5">
         <v>6000</v>
@@ -32636,16 +32755,16 @@
         <v>12873.6</v>
       </c>
       <c r="V14" s="2" t="s">
-        <v>1301</v>
+        <v>1304</v>
       </c>
       <c r="W14" s="2" t="s">
-        <v>1300</v>
+        <v>1303</v>
       </c>
       <c r="X14" s="2" t="s">
         <v>51</v>
       </c>
       <c r="Y14" s="2" t="s">
-        <v>1299</v>
+        <v>1302</v>
       </c>
       <c r="Z14" s="2" t="s">
         <v>0</v>
@@ -32660,10 +32779,10 @@
         <v>298</v>
       </c>
       <c r="AD14" s="2" t="s">
-        <v>1152</v>
+        <v>1155</v>
       </c>
       <c r="AE14" s="2" t="s">
-        <v>1151</v>
+        <v>1154</v>
       </c>
       <c r="AF14" s="2" t="s">
         <v>77</v>
@@ -32683,13 +32802,13 @@
     </row>
     <row r="15" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>1298</v>
+        <v>1301</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>1298</v>
+        <v>1301</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D15" s="7">
         <v>46042</v>
@@ -32701,10 +32820,10 @@
         <v>212</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>1248</v>
+        <v>1251</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>139</v>
@@ -32755,7 +32874,7 @@
         <v>87</v>
       </c>
       <c r="Y15" s="3" t="s">
-        <v>1297</v>
+        <v>1300</v>
       </c>
       <c r="Z15" s="3" t="s">
         <v>0</v>
@@ -32776,7 +32895,7 @@
         <v>518</v>
       </c>
       <c r="AF15" s="3" t="s">
-        <v>1268</v>
+        <v>1271</v>
       </c>
       <c r="AG15" s="9">
         <v>0</v>
@@ -32793,13 +32912,13 @@
     </row>
     <row r="16" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>1298</v>
+        <v>1301</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>1298</v>
+        <v>1301</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D16" s="4">
         <v>46042</v>
@@ -32811,10 +32930,10 @@
         <v>212</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>1248</v>
+        <v>1251</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>139</v>
@@ -32865,7 +32984,7 @@
         <v>87</v>
       </c>
       <c r="Y16" s="2" t="s">
-        <v>1297</v>
+        <v>1300</v>
       </c>
       <c r="Z16" s="2" t="s">
         <v>0</v>
@@ -32886,7 +33005,7 @@
         <v>518</v>
       </c>
       <c r="AF16" s="2" t="s">
-        <v>1268</v>
+        <v>1271</v>
       </c>
       <c r="AG16" s="6">
         <v>0</v>
@@ -32903,13 +33022,13 @@
     </row>
     <row r="17" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
-        <v>1296</v>
+        <v>1299</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>1296</v>
+        <v>1299</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D17" s="7">
         <v>46043</v>
@@ -32936,13 +33055,13 @@
         <v>417</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>1222</v>
+        <v>1225</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>1221</v>
+        <v>1224</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>1220</v>
+        <v>1223</v>
       </c>
       <c r="O17" s="8">
         <v>1000</v>
@@ -32975,7 +33094,7 @@
         <v>51</v>
       </c>
       <c r="Y17" s="3" t="s">
-        <v>1295</v>
+        <v>1298</v>
       </c>
       <c r="Z17" s="3" t="s">
         <v>0</v>
@@ -33013,28 +33132,28 @@
     </row>
     <row r="18" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>1283</v>
+        <v>1286</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>1283</v>
+        <v>1286</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D18" s="4">
         <v>46045</v>
       </c>
       <c r="E18" s="2" t="s">
+        <v>1119</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>1118</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>1117</v>
+      </c>
+      <c r="H18" s="2" t="s">
         <v>1116</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>1115</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>1114</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>1113</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>139</v>
@@ -33046,13 +33165,13 @@
         <v>628</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>1294</v>
+        <v>1297</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>1293</v>
+        <v>1296</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>1292</v>
+        <v>1295</v>
       </c>
       <c r="O18" s="5">
         <v>2000</v>
@@ -33076,16 +33195,16 @@
         <v>0</v>
       </c>
       <c r="V18" s="2" t="s">
-        <v>1109</v>
+        <v>1112</v>
       </c>
       <c r="W18" s="2" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="X18" s="2" t="s">
         <v>87</v>
       </c>
       <c r="Y18" s="2" t="s">
-        <v>1279</v>
+        <v>1282</v>
       </c>
       <c r="Z18" s="2" t="s">
         <v>0</v>
@@ -33123,28 +33242,28 @@
     </row>
     <row r="19" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
-        <v>1283</v>
+        <v>1286</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>1283</v>
+        <v>1286</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D19" s="7">
         <v>46045</v>
       </c>
       <c r="E19" s="3" t="s">
+        <v>1119</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>1118</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>1117</v>
+      </c>
+      <c r="H19" s="3" t="s">
         <v>1116</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>1115</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>1114</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>1113</v>
       </c>
       <c r="I19" s="3" t="s">
         <v>139</v>
@@ -33156,13 +33275,13 @@
         <v>631</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>1291</v>
+        <v>1294</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>1290</v>
+        <v>1293</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>1280</v>
+        <v>1283</v>
       </c>
       <c r="O19" s="8">
         <v>11725</v>
@@ -33186,16 +33305,16 @@
         <v>0</v>
       </c>
       <c r="V19" s="3" t="s">
-        <v>1109</v>
+        <v>1112</v>
       </c>
       <c r="W19" s="3" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="X19" s="3" t="s">
         <v>87</v>
       </c>
       <c r="Y19" s="3" t="s">
-        <v>1279</v>
+        <v>1282</v>
       </c>
       <c r="Z19" s="3" t="s">
         <v>0</v>
@@ -33233,28 +33352,28 @@
     </row>
     <row r="20" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>1283</v>
+        <v>1286</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>1283</v>
+        <v>1286</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D20" s="4">
         <v>46045</v>
       </c>
       <c r="E20" s="2" t="s">
+        <v>1119</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>1118</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>1117</v>
+      </c>
+      <c r="H20" s="2" t="s">
         <v>1116</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>1115</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>1114</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>1113</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>139</v>
@@ -33266,13 +33385,13 @@
         <v>632</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>1211</v>
+        <v>1214</v>
       </c>
       <c r="M20" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>1210</v>
+        <v>1213</v>
       </c>
       <c r="O20" s="5">
         <v>2925</v>
@@ -33296,16 +33415,16 @@
         <v>0</v>
       </c>
       <c r="V20" s="2" t="s">
-        <v>1109</v>
+        <v>1112</v>
       </c>
       <c r="W20" s="2" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="X20" s="2" t="s">
         <v>87</v>
       </c>
       <c r="Y20" s="2" t="s">
-        <v>1279</v>
+        <v>1282</v>
       </c>
       <c r="Z20" s="2" t="s">
         <v>0</v>
@@ -33343,28 +33462,28 @@
     </row>
     <row r="21" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
-        <v>1283</v>
+        <v>1286</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>1283</v>
+        <v>1286</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D21" s="7">
         <v>46045</v>
       </c>
       <c r="E21" s="3" t="s">
+        <v>1119</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>1118</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>1117</v>
+      </c>
+      <c r="H21" s="3" t="s">
         <v>1116</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>1115</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>1114</v>
-      </c>
-      <c r="H21" s="3" t="s">
-        <v>1113</v>
       </c>
       <c r="I21" s="3" t="s">
         <v>139</v>
@@ -33376,13 +33495,13 @@
         <v>633</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>1102</v>
+        <v>1105</v>
       </c>
       <c r="M21" s="3" t="s">
         <v>652</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>1101</v>
+        <v>1104</v>
       </c>
       <c r="O21" s="8">
         <v>2925</v>
@@ -33406,16 +33525,16 @@
         <v>0</v>
       </c>
       <c r="V21" s="3" t="s">
-        <v>1109</v>
+        <v>1112</v>
       </c>
       <c r="W21" s="3" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="X21" s="3" t="s">
         <v>87</v>
       </c>
       <c r="Y21" s="3" t="s">
-        <v>1279</v>
+        <v>1282</v>
       </c>
       <c r="Z21" s="3" t="s">
         <v>0</v>
@@ -33453,28 +33572,28 @@
     </row>
     <row r="22" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>1283</v>
+        <v>1286</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>1283</v>
+        <v>1286</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D22" s="4">
         <v>46045</v>
       </c>
       <c r="E22" s="2" t="s">
+        <v>1119</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>1118</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>1117</v>
+      </c>
+      <c r="H22" s="2" t="s">
         <v>1116</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>1115</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>1114</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>1113</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>139</v>
@@ -33486,13 +33605,13 @@
         <v>465</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>1289</v>
+        <v>1292</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>1288</v>
+        <v>1291</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>1287</v>
+        <v>1290</v>
       </c>
       <c r="O22" s="5">
         <v>2400</v>
@@ -33516,16 +33635,16 @@
         <v>0</v>
       </c>
       <c r="V22" s="2" t="s">
-        <v>1109</v>
+        <v>1112</v>
       </c>
       <c r="W22" s="2" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="X22" s="2" t="s">
         <v>87</v>
       </c>
       <c r="Y22" s="2" t="s">
-        <v>1279</v>
+        <v>1282</v>
       </c>
       <c r="Z22" s="2" t="s">
         <v>0</v>
@@ -33563,28 +33682,28 @@
     </row>
     <row r="23" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
-        <v>1283</v>
+        <v>1286</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>1283</v>
+        <v>1286</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D23" s="7">
         <v>46045</v>
       </c>
       <c r="E23" s="3" t="s">
+        <v>1119</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>1118</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>1117</v>
+      </c>
+      <c r="H23" s="3" t="s">
         <v>1116</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>1115</v>
-      </c>
-      <c r="G23" s="3" t="s">
-        <v>1114</v>
-      </c>
-      <c r="H23" s="3" t="s">
-        <v>1113</v>
       </c>
       <c r="I23" s="3" t="s">
         <v>139</v>
@@ -33596,13 +33715,13 @@
         <v>465</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>1286</v>
+        <v>1289</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>1285</v>
+        <v>1288</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>1284</v>
+        <v>1287</v>
       </c>
       <c r="O23" s="8">
         <v>1800</v>
@@ -33626,16 +33745,16 @@
         <v>0</v>
       </c>
       <c r="V23" s="3" t="s">
-        <v>1109</v>
+        <v>1112</v>
       </c>
       <c r="W23" s="3" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="X23" s="3" t="s">
         <v>87</v>
       </c>
       <c r="Y23" s="3" t="s">
-        <v>1279</v>
+        <v>1282</v>
       </c>
       <c r="Z23" s="3" t="s">
         <v>0</v>
@@ -33673,28 +33792,28 @@
     </row>
     <row r="24" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>1283</v>
+        <v>1286</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>1283</v>
+        <v>1286</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D24" s="4">
         <v>46045</v>
       </c>
       <c r="E24" s="2" t="s">
+        <v>1119</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>1118</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>1117</v>
+      </c>
+      <c r="H24" s="2" t="s">
         <v>1116</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>1115</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>1114</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>1113</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>139</v>
@@ -33706,13 +33825,13 @@
         <v>634</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>1282</v>
+        <v>1285</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>1281</v>
+        <v>1284</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>1280</v>
+        <v>1283</v>
       </c>
       <c r="O24" s="5">
         <v>1400</v>
@@ -33736,16 +33855,16 @@
         <v>0</v>
       </c>
       <c r="V24" s="2" t="s">
-        <v>1109</v>
+        <v>1112</v>
       </c>
       <c r="W24" s="2" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="X24" s="2" t="s">
         <v>87</v>
       </c>
       <c r="Y24" s="2" t="s">
-        <v>1279</v>
+        <v>1282</v>
       </c>
       <c r="Z24" s="2" t="s">
         <v>0</v>
@@ -33783,13 +33902,13 @@
     </row>
     <row r="25" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
-        <v>1278</v>
+        <v>1281</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>1278</v>
+        <v>1281</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D25" s="7">
         <v>46048</v>
@@ -33816,13 +33935,13 @@
         <v>417</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>1231</v>
+        <v>1234</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>1230</v>
+        <v>1233</v>
       </c>
       <c r="N25" s="3" t="s">
-        <v>1124</v>
+        <v>1127</v>
       </c>
       <c r="O25" s="8">
         <v>5000</v>
@@ -33846,16 +33965,16 @@
         <v>2354</v>
       </c>
       <c r="V25" s="3" t="s">
-        <v>1135</v>
+        <v>1138</v>
       </c>
       <c r="W25" s="3" t="s">
-        <v>1134</v>
+        <v>1137</v>
       </c>
       <c r="X25" s="3" t="s">
         <v>51</v>
       </c>
       <c r="Y25" s="3" t="s">
-        <v>1277</v>
+        <v>1280</v>
       </c>
       <c r="Z25" s="3" t="s">
         <v>0</v>
@@ -33893,13 +34012,13 @@
     </row>
     <row r="26" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>1276</v>
+        <v>1279</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>1276</v>
+        <v>1279</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D26" s="4">
         <v>46048</v>
@@ -33911,10 +34030,10 @@
         <v>40</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>1131</v>
+        <v>1134</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>139</v>
@@ -33926,13 +34045,13 @@
         <v>782</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>1129</v>
+        <v>1132</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>1128</v>
+        <v>1131</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>1127</v>
+        <v>1130</v>
       </c>
       <c r="O26" s="5">
         <v>300</v>
@@ -33965,7 +34084,7 @@
         <v>51</v>
       </c>
       <c r="Y26" s="2" t="s">
-        <v>1275</v>
+        <v>1278</v>
       </c>
       <c r="Z26" s="2" t="s">
         <v>0</v>
@@ -34003,13 +34122,13 @@
     </row>
     <row r="27" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
-        <v>1274</v>
+        <v>1277</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>1274</v>
+        <v>1277</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D27" s="7">
         <v>46048</v>
@@ -34021,10 +34140,10 @@
         <v>61</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>1104</v>
+        <v>1107</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>1103</v>
+        <v>1106</v>
       </c>
       <c r="I27" s="3" t="s">
         <v>163</v>
@@ -34036,13 +34155,13 @@
         <v>632</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>1211</v>
+        <v>1214</v>
       </c>
       <c r="M27" s="3" t="s">
         <v>648</v>
       </c>
       <c r="N27" s="3" t="s">
-        <v>1210</v>
+        <v>1213</v>
       </c>
       <c r="O27" s="8">
         <v>611</v>
@@ -34075,7 +34194,7 @@
         <v>51</v>
       </c>
       <c r="Y27" s="3" t="s">
-        <v>1271</v>
+        <v>1274</v>
       </c>
       <c r="Z27" s="3" t="s">
         <v>0</v>
@@ -34113,13 +34232,13 @@
     </row>
     <row r="28" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>1274</v>
+        <v>1277</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>1274</v>
+        <v>1277</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D28" s="4">
         <v>46048</v>
@@ -34131,10 +34250,10 @@
         <v>61</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>1104</v>
+        <v>1107</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>1103</v>
+        <v>1106</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>163</v>
@@ -34143,16 +34262,16 @@
         <v>164</v>
       </c>
       <c r="K28" s="2" t="s">
+        <v>1160</v>
+      </c>
+      <c r="L28" s="2" t="s">
+        <v>1276</v>
+      </c>
+      <c r="M28" s="2" t="s">
+        <v>1275</v>
+      </c>
+      <c r="N28" s="2" t="s">
         <v>1157</v>
-      </c>
-      <c r="L28" s="2" t="s">
-        <v>1273</v>
-      </c>
-      <c r="M28" s="2" t="s">
-        <v>1272</v>
-      </c>
-      <c r="N28" s="2" t="s">
-        <v>1154</v>
       </c>
       <c r="O28" s="5">
         <v>700</v>
@@ -34185,7 +34304,7 @@
         <v>51</v>
       </c>
       <c r="Y28" s="2" t="s">
-        <v>1271</v>
+        <v>1274</v>
       </c>
       <c r="Z28" s="2" t="s">
         <v>0</v>
@@ -34200,10 +34319,10 @@
         <v>55</v>
       </c>
       <c r="AD28" s="2" t="s">
-        <v>1152</v>
+        <v>1155</v>
       </c>
       <c r="AE28" s="2" t="s">
-        <v>1151</v>
+        <v>1154</v>
       </c>
       <c r="AF28" s="2" t="s">
         <v>77</v>
@@ -34223,13 +34342,13 @@
     </row>
     <row r="29" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
-        <v>1270</v>
+        <v>1273</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>1270</v>
+        <v>1273</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D29" s="7">
         <v>46048</v>
@@ -34241,10 +34360,10 @@
         <v>212</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>1248</v>
+        <v>1251</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="I29" s="3" t="s">
         <v>139</v>
@@ -34295,7 +34414,7 @@
         <v>87</v>
       </c>
       <c r="Y29" s="3" t="s">
-        <v>1269</v>
+        <v>1272</v>
       </c>
       <c r="Z29" s="3" t="s">
         <v>0</v>
@@ -34316,7 +34435,7 @@
         <v>57</v>
       </c>
       <c r="AF29" s="3" t="s">
-        <v>1268</v>
+        <v>1271</v>
       </c>
       <c r="AG29" s="9">
         <v>0</v>
@@ -34333,13 +34452,13 @@
     </row>
     <row r="30" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>1267</v>
+        <v>1270</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>1267</v>
+        <v>1270</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D30" s="4">
         <v>46049</v>
@@ -34351,10 +34470,10 @@
         <v>212</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>1248</v>
+        <v>1251</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>139</v>
@@ -34405,7 +34524,7 @@
         <v>87</v>
       </c>
       <c r="Y30" s="2" t="s">
-        <v>1266</v>
+        <v>1269</v>
       </c>
       <c r="Z30" s="2" t="s">
         <v>0</v>
@@ -34443,13 +34562,13 @@
     </row>
     <row r="31" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
-        <v>1267</v>
+        <v>1270</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>1267</v>
+        <v>1270</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D31" s="7">
         <v>46049</v>
@@ -34461,10 +34580,10 @@
         <v>212</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>1248</v>
+        <v>1251</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="I31" s="3" t="s">
         <v>139</v>
@@ -34515,7 +34634,7 @@
         <v>87</v>
       </c>
       <c r="Y31" s="3" t="s">
-        <v>1266</v>
+        <v>1269</v>
       </c>
       <c r="Z31" s="3" t="s">
         <v>0</v>
@@ -34553,13 +34672,13 @@
     </row>
     <row r="32" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>1263</v>
+        <v>1266</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>1263</v>
+        <v>1266</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D32" s="4">
         <v>46050</v>
@@ -34577,22 +34696,22 @@
         <v>386</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>1215</v>
+        <v>1218</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>1214</v>
+        <v>1217</v>
       </c>
       <c r="K32" s="2" t="s">
         <v>446</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>1265</v>
+        <v>1268</v>
       </c>
       <c r="M32" s="2" t="s">
         <v>448</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>1264</v>
+        <v>1267</v>
       </c>
       <c r="O32" s="5">
         <v>1000</v>
@@ -34625,7 +34744,7 @@
         <v>51</v>
       </c>
       <c r="Y32" s="2" t="s">
-        <v>1262</v>
+        <v>1265</v>
       </c>
       <c r="Z32" s="2" t="s">
         <v>0</v>
@@ -34663,13 +34782,13 @@
     </row>
     <row r="33" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
-        <v>1263</v>
+        <v>1266</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>1263</v>
+        <v>1266</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D33" s="7">
         <v>46050</v>
@@ -34687,22 +34806,22 @@
         <v>386</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>1215</v>
+        <v>1218</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>1214</v>
+        <v>1217</v>
       </c>
       <c r="K33" s="3" t="s">
         <v>446</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>1218</v>
+        <v>1221</v>
       </c>
       <c r="M33" s="3" t="s">
-        <v>1217</v>
+        <v>1220</v>
       </c>
       <c r="N33" s="3" t="s">
-        <v>1185</v>
+        <v>1188</v>
       </c>
       <c r="O33" s="8">
         <v>1000</v>
@@ -34735,7 +34854,7 @@
         <v>51</v>
       </c>
       <c r="Y33" s="3" t="s">
-        <v>1262</v>
+        <v>1265</v>
       </c>
       <c r="Z33" s="3" t="s">
         <v>0</v>
@@ -34773,13 +34892,13 @@
     </row>
     <row r="34" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>1261</v>
+        <v>1264</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>1261</v>
+        <v>1264</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D34" s="4">
         <v>46050</v>
@@ -34791,10 +34910,10 @@
         <v>212</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>1248</v>
+        <v>1251</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="I34" s="2" t="s">
         <v>139</v>
@@ -34845,7 +34964,7 @@
         <v>87</v>
       </c>
       <c r="Y34" s="2" t="s">
-        <v>1260</v>
+        <v>1263</v>
       </c>
       <c r="Z34" s="2" t="s">
         <v>0</v>
@@ -34883,13 +35002,13 @@
     </row>
     <row r="35" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
-        <v>1259</v>
+        <v>1262</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>1259</v>
+        <v>1262</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D35" s="7">
         <v>46051</v>
@@ -34901,10 +35020,10 @@
         <v>40</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>1258</v>
+        <v>1261</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>1257</v>
+        <v>1260</v>
       </c>
       <c r="I35" s="3" t="s">
         <v>43</v>
@@ -34916,13 +35035,13 @@
         <v>632</v>
       </c>
       <c r="L35" s="3" t="s">
-        <v>1211</v>
+        <v>1214</v>
       </c>
       <c r="M35" s="3" t="s">
         <v>648</v>
       </c>
       <c r="N35" s="3" t="s">
-        <v>1210</v>
+        <v>1213</v>
       </c>
       <c r="O35" s="8">
         <v>26</v>
@@ -34955,7 +35074,7 @@
         <v>51</v>
       </c>
       <c r="Y35" s="3" t="s">
-        <v>1256</v>
+        <v>1259</v>
       </c>
       <c r="Z35" s="3" t="s">
         <v>0</v>
@@ -34993,13 +35112,13 @@
     </row>
     <row r="36" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>1255</v>
+        <v>1258</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>1255</v>
+        <v>1258</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D36" s="4">
         <v>46052</v>
@@ -35011,10 +35130,10 @@
         <v>61</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>1104</v>
+        <v>1107</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>1103</v>
+        <v>1106</v>
       </c>
       <c r="I36" s="2" t="s">
         <v>163</v>
@@ -35026,13 +35145,13 @@
         <v>632</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>1211</v>
+        <v>1214</v>
       </c>
       <c r="M36" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>1210</v>
+        <v>1213</v>
       </c>
       <c r="O36" s="5">
         <v>507</v>
@@ -35065,7 +35184,7 @@
         <v>51</v>
       </c>
       <c r="Y36" s="2" t="s">
-        <v>1254</v>
+        <v>1257</v>
       </c>
       <c r="Z36" s="2" t="s">
         <v>0</v>
@@ -35103,13 +35222,13 @@
     </row>
     <row r="37" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
-        <v>1253</v>
+        <v>1256</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>1253</v>
+        <v>1256</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D37" s="7">
         <v>46052</v>
@@ -35133,16 +35252,16 @@
         <v>164</v>
       </c>
       <c r="K37" s="3" t="s">
+        <v>1165</v>
+      </c>
+      <c r="L37" s="3" t="s">
+        <v>1182</v>
+      </c>
+      <c r="M37" s="3" t="s">
+        <v>1181</v>
+      </c>
+      <c r="N37" s="3" t="s">
         <v>1162</v>
-      </c>
-      <c r="L37" s="3" t="s">
-        <v>1179</v>
-      </c>
-      <c r="M37" s="3" t="s">
-        <v>1178</v>
-      </c>
-      <c r="N37" s="3" t="s">
-        <v>1159</v>
       </c>
       <c r="O37" s="8">
         <v>500</v>
@@ -35175,7 +35294,7 @@
         <v>51</v>
       </c>
       <c r="Y37" s="3" t="s">
-        <v>1252</v>
+        <v>1255</v>
       </c>
       <c r="Z37" s="3" t="s">
         <v>0</v>
@@ -35213,13 +35332,13 @@
     </row>
     <row r="38" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>1251</v>
+        <v>1254</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>1251</v>
+        <v>1254</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D38" s="4">
         <v>46052</v>
@@ -35231,10 +35350,10 @@
         <v>40</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>1131</v>
+        <v>1134</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="I38" s="2" t="s">
         <v>139</v>
@@ -35246,13 +35365,13 @@
         <v>782</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>1129</v>
+        <v>1132</v>
       </c>
       <c r="M38" s="2" t="s">
-        <v>1128</v>
+        <v>1131</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>1127</v>
+        <v>1130</v>
       </c>
       <c r="O38" s="5">
         <v>300</v>
@@ -35285,7 +35404,7 @@
         <v>51</v>
       </c>
       <c r="Y38" s="2" t="s">
-        <v>1250</v>
+        <v>1253</v>
       </c>
       <c r="Z38" s="2" t="s">
         <v>0</v>
@@ -35323,13 +35442,13 @@
     </row>
     <row r="39" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
-        <v>1249</v>
+        <v>1252</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>1249</v>
+        <v>1252</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D39" s="7">
         <v>46055</v>
@@ -35341,10 +35460,10 @@
         <v>212</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>1248</v>
+        <v>1251</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="I39" s="3" t="s">
         <v>139</v>
@@ -35353,7 +35472,7 @@
         <v>140</v>
       </c>
       <c r="K39" s="3" t="s">
-        <v>1247</v>
+        <v>1250</v>
       </c>
       <c r="L39" s="3" t="s">
         <v>0</v>
@@ -35395,7 +35514,7 @@
         <v>87</v>
       </c>
       <c r="Y39" s="3" t="s">
-        <v>1246</v>
+        <v>1249</v>
       </c>
       <c r="Z39" s="3" t="s">
         <v>0</v>
@@ -35433,13 +35552,13 @@
     </row>
     <row r="40" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>1245</v>
+        <v>1248</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>1245</v>
+        <v>1248</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D40" s="4">
         <v>46057</v>
@@ -35451,10 +35570,10 @@
         <v>61</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>1104</v>
+        <v>1107</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>1103</v>
+        <v>1106</v>
       </c>
       <c r="I40" s="2" t="s">
         <v>163</v>
@@ -35466,13 +35585,13 @@
         <v>632</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>1211</v>
+        <v>1214</v>
       </c>
       <c r="M40" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>1210</v>
+        <v>1213</v>
       </c>
       <c r="O40" s="5">
         <v>507</v>
@@ -35505,7 +35624,7 @@
         <v>51</v>
       </c>
       <c r="Y40" s="2" t="s">
-        <v>1244</v>
+        <v>1247</v>
       </c>
       <c r="Z40" s="2" t="s">
         <v>0</v>
@@ -35543,13 +35662,13 @@
     </row>
     <row r="41" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
-        <v>1243</v>
+        <v>1246</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>1243</v>
+        <v>1246</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D41" s="7">
         <v>46057</v>
@@ -35567,22 +35686,22 @@
         <v>386</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>1215</v>
+        <v>1218</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>1214</v>
+        <v>1217</v>
       </c>
       <c r="K41" s="3" t="s">
         <v>446</v>
       </c>
       <c r="L41" s="3" t="s">
-        <v>1218</v>
+        <v>1221</v>
       </c>
       <c r="M41" s="3" t="s">
-        <v>1217</v>
+        <v>1220</v>
       </c>
       <c r="N41" s="3" t="s">
-        <v>1185</v>
+        <v>1188</v>
       </c>
       <c r="O41" s="8">
         <v>2000</v>
@@ -35615,7 +35734,7 @@
         <v>51</v>
       </c>
       <c r="Y41" s="3" t="s">
-        <v>1213</v>
+        <v>1216</v>
       </c>
       <c r="Z41" s="3" t="s">
         <v>0</v>
@@ -35653,13 +35772,13 @@
     </row>
     <row r="42" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>1242</v>
+        <v>1245</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>1242</v>
+        <v>1245</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D42" s="4">
         <v>46058</v>
@@ -35671,10 +35790,10 @@
         <v>61</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>1104</v>
+        <v>1107</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>1103</v>
+        <v>1106</v>
       </c>
       <c r="I42" s="2" t="s">
         <v>163</v>
@@ -35686,13 +35805,13 @@
         <v>632</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>1211</v>
+        <v>1214</v>
       </c>
       <c r="M42" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>1210</v>
+        <v>1213</v>
       </c>
       <c r="O42" s="5">
         <v>507</v>
@@ -35725,7 +35844,7 @@
         <v>51</v>
       </c>
       <c r="Y42" s="2" t="s">
-        <v>1241</v>
+        <v>1244</v>
       </c>
       <c r="Z42" s="2" t="s">
         <v>0</v>
@@ -35763,13 +35882,13 @@
     </row>
     <row r="43" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
-        <v>1240</v>
+        <v>1243</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>1240</v>
+        <v>1243</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D43" s="7">
         <v>46058</v>
@@ -35781,10 +35900,10 @@
         <v>61</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>1182</v>
+        <v>1185</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>1181</v>
+        <v>1184</v>
       </c>
       <c r="I43" s="3" t="s">
         <v>163</v>
@@ -35796,13 +35915,13 @@
         <v>417</v>
       </c>
       <c r="L43" s="3" t="s">
-        <v>1231</v>
+        <v>1234</v>
       </c>
       <c r="M43" s="3" t="s">
-        <v>1230</v>
+        <v>1233</v>
       </c>
       <c r="N43" s="3" t="s">
-        <v>1124</v>
+        <v>1127</v>
       </c>
       <c r="O43" s="8">
         <v>1800</v>
@@ -35835,7 +35954,7 @@
         <v>51</v>
       </c>
       <c r="Y43" s="3" t="s">
-        <v>1239</v>
+        <v>1242</v>
       </c>
       <c r="Z43" s="3" t="s">
         <v>0</v>
@@ -35873,13 +35992,13 @@
     </row>
     <row r="44" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>1238</v>
+        <v>1241</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>1238</v>
+        <v>1241</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D44" s="4">
         <v>46059</v>
@@ -35891,10 +36010,10 @@
         <v>40</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>1237</v>
+        <v>1240</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>1236</v>
+        <v>1239</v>
       </c>
       <c r="I44" s="2" t="s">
         <v>43</v>
@@ -35906,13 +36025,13 @@
         <v>782</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>1129</v>
+        <v>1132</v>
       </c>
       <c r="M44" s="2" t="s">
-        <v>1128</v>
+        <v>1131</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>1127</v>
+        <v>1130</v>
       </c>
       <c r="O44" s="5">
         <v>500</v>
@@ -35945,7 +36064,7 @@
         <v>51</v>
       </c>
       <c r="Y44" s="2" t="s">
-        <v>1235</v>
+        <v>1238</v>
       </c>
       <c r="Z44" s="2" t="s">
         <v>0</v>
@@ -35983,13 +36102,13 @@
     </row>
     <row r="45" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="3" t="s">
-        <v>1234</v>
+        <v>1237</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>1234</v>
+        <v>1237</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D45" s="7">
         <v>46059</v>
@@ -36001,10 +36120,10 @@
         <v>40</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>1233</v>
+        <v>1236</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>1232</v>
+        <v>1235</v>
       </c>
       <c r="I45" s="3" t="s">
         <v>43</v>
@@ -36016,13 +36135,13 @@
         <v>417</v>
       </c>
       <c r="L45" s="3" t="s">
-        <v>1231</v>
+        <v>1234</v>
       </c>
       <c r="M45" s="3" t="s">
-        <v>1230</v>
+        <v>1233</v>
       </c>
       <c r="N45" s="3" t="s">
-        <v>1124</v>
+        <v>1127</v>
       </c>
       <c r="O45" s="8">
         <v>200</v>
@@ -36055,7 +36174,7 @@
         <v>51</v>
       </c>
       <c r="Y45" s="3" t="s">
-        <v>1229</v>
+        <v>1232</v>
       </c>
       <c r="Z45" s="3" t="s">
         <v>0</v>
@@ -36093,28 +36212,28 @@
     </row>
     <row r="46" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
-        <v>1228</v>
+        <v>1231</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>1228</v>
+        <v>1231</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D46" s="4">
         <v>46063</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>1227</v>
+        <v>1230</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>267</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>1114</v>
+        <v>1117</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>1113</v>
+        <v>1116</v>
       </c>
       <c r="I46" s="2" t="s">
         <v>139</v>
@@ -36123,7 +36242,7 @@
         <v>140</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>1140</v>
+        <v>1143</v>
       </c>
       <c r="L46" s="2" t="s">
         <v>0</v>
@@ -36165,7 +36284,7 @@
         <v>0</v>
       </c>
       <c r="Y46" s="2" t="s">
-        <v>1226</v>
+        <v>1229</v>
       </c>
       <c r="Z46" s="2" t="s">
         <v>0</v>
@@ -36180,10 +36299,10 @@
         <v>74</v>
       </c>
       <c r="AD46" s="2" t="s">
-        <v>1138</v>
+        <v>1141</v>
       </c>
       <c r="AE46" s="2" t="s">
-        <v>1137</v>
+        <v>1140</v>
       </c>
       <c r="AF46" s="2" t="s">
         <v>0</v>
@@ -36203,13 +36322,13 @@
     </row>
     <row r="47" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
-        <v>1225</v>
+        <v>1228</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>1225</v>
+        <v>1228</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D47" s="7">
         <v>46064</v>
@@ -36221,10 +36340,10 @@
         <v>61</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>1224</v>
+        <v>1227</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>1223</v>
+        <v>1226</v>
       </c>
       <c r="I47" s="3" t="s">
         <v>139</v>
@@ -36236,13 +36355,13 @@
         <v>417</v>
       </c>
       <c r="L47" s="3" t="s">
-        <v>1222</v>
+        <v>1225</v>
       </c>
       <c r="M47" s="3" t="s">
-        <v>1221</v>
+        <v>1224</v>
       </c>
       <c r="N47" s="3" t="s">
-        <v>1220</v>
+        <v>1223</v>
       </c>
       <c r="O47" s="8">
         <v>1000</v>
@@ -36275,7 +36394,7 @@
         <v>51</v>
       </c>
       <c r="Y47" s="3" t="s">
-        <v>1219</v>
+        <v>1222</v>
       </c>
       <c r="Z47" s="3" t="s">
         <v>0</v>
@@ -36313,13 +36432,13 @@
     </row>
     <row r="48" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
-        <v>1216</v>
+        <v>1219</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>1216</v>
+        <v>1219</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D48" s="4">
         <v>46064</v>
@@ -36337,22 +36456,22 @@
         <v>386</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>1215</v>
+        <v>1218</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>1214</v>
+        <v>1217</v>
       </c>
       <c r="K48" s="2" t="s">
         <v>446</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>1218</v>
+        <v>1221</v>
       </c>
       <c r="M48" s="2" t="s">
-        <v>1217</v>
+        <v>1220</v>
       </c>
       <c r="N48" s="2" t="s">
-        <v>1185</v>
+        <v>1188</v>
       </c>
       <c r="O48" s="5">
         <v>1000</v>
@@ -36385,7 +36504,7 @@
         <v>51</v>
       </c>
       <c r="Y48" s="2" t="s">
-        <v>1213</v>
+        <v>1216</v>
       </c>
       <c r="Z48" s="2" t="s">
         <v>0</v>
@@ -36423,13 +36542,13 @@
     </row>
     <row r="49" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
-        <v>1216</v>
+        <v>1219</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>1216</v>
+        <v>1219</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D49" s="7">
         <v>46064</v>
@@ -36447,22 +36566,22 @@
         <v>386</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>1215</v>
+        <v>1218</v>
       </c>
       <c r="J49" s="3" t="s">
-        <v>1214</v>
+        <v>1217</v>
       </c>
       <c r="K49" s="3" t="s">
         <v>446</v>
       </c>
       <c r="L49" s="3" t="s">
-        <v>1187</v>
+        <v>1190</v>
       </c>
       <c r="M49" s="3" t="s">
-        <v>1186</v>
+        <v>1189</v>
       </c>
       <c r="N49" s="3" t="s">
-        <v>1185</v>
+        <v>1188</v>
       </c>
       <c r="O49" s="8">
         <v>1000</v>
@@ -36495,7 +36614,7 @@
         <v>51</v>
       </c>
       <c r="Y49" s="3" t="s">
-        <v>1213</v>
+        <v>1216</v>
       </c>
       <c r="Z49" s="3" t="s">
         <v>0</v>
@@ -36533,13 +36652,13 @@
     </row>
     <row r="50" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
-        <v>1212</v>
+        <v>1215</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>1212</v>
+        <v>1215</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D50" s="4">
         <v>46066</v>
@@ -36551,10 +36670,10 @@
         <v>61</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>1104</v>
+        <v>1107</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>1103</v>
+        <v>1106</v>
       </c>
       <c r="I50" s="2" t="s">
         <v>163</v>
@@ -36566,13 +36685,13 @@
         <v>632</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>1211</v>
+        <v>1214</v>
       </c>
       <c r="M50" s="2" t="s">
         <v>648</v>
       </c>
       <c r="N50" s="2" t="s">
-        <v>1210</v>
+        <v>1213</v>
       </c>
       <c r="O50" s="5">
         <v>507</v>
@@ -36605,7 +36724,7 @@
         <v>51</v>
       </c>
       <c r="Y50" s="2" t="s">
-        <v>1209</v>
+        <v>1212</v>
       </c>
       <c r="Z50" s="2" t="s">
         <v>0</v>
@@ -36643,13 +36762,13 @@
     </row>
     <row r="51" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
-        <v>1208</v>
+        <v>1211</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>1208</v>
+        <v>1211</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D51" s="7">
         <v>46071</v>
@@ -36673,16 +36792,16 @@
         <v>164</v>
       </c>
       <c r="K51" s="3" t="s">
-        <v>1157</v>
+        <v>1160</v>
       </c>
       <c r="L51" s="3" t="s">
-        <v>1207</v>
+        <v>1210</v>
       </c>
       <c r="M51" s="3" t="s">
-        <v>1206</v>
+        <v>1209</v>
       </c>
       <c r="N51" s="3" t="s">
-        <v>1205</v>
+        <v>1208</v>
       </c>
       <c r="O51" s="8">
         <v>500</v>
@@ -36715,7 +36834,7 @@
         <v>51</v>
       </c>
       <c r="Y51" s="3" t="s">
-        <v>1204</v>
+        <v>1207</v>
       </c>
       <c r="Z51" s="3" t="s">
         <v>0</v>
@@ -36730,10 +36849,10 @@
         <v>111</v>
       </c>
       <c r="AD51" s="3" t="s">
-        <v>1152</v>
+        <v>1155</v>
       </c>
       <c r="AE51" s="3" t="s">
-        <v>1151</v>
+        <v>1154</v>
       </c>
       <c r="AF51" s="3" t="s">
         <v>77</v>
@@ -36753,13 +36872,13 @@
     </row>
     <row r="52" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>1203</v>
+        <v>1206</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>1203</v>
+        <v>1206</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D52" s="4">
         <v>46071</v>
@@ -36771,10 +36890,10 @@
         <v>61</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>1202</v>
+        <v>1205</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>1201</v>
+        <v>1204</v>
       </c>
       <c r="I52" s="2" t="s">
         <v>139</v>
@@ -36786,13 +36905,13 @@
         <v>446</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>1187</v>
+        <v>1190</v>
       </c>
       <c r="M52" s="2" t="s">
-        <v>1186</v>
+        <v>1189</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>1185</v>
+        <v>1188</v>
       </c>
       <c r="O52" s="5">
         <v>200</v>
@@ -36825,7 +36944,7 @@
         <v>51</v>
       </c>
       <c r="Y52" s="2" t="s">
-        <v>1200</v>
+        <v>1203</v>
       </c>
       <c r="Z52" s="2" t="s">
         <v>0</v>
@@ -36863,13 +36982,13 @@
     </row>
     <row r="53" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
-        <v>1199</v>
+        <v>1202</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>1199</v>
+        <v>1202</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D53" s="7">
         <v>46072</v>
@@ -36881,10 +37000,10 @@
         <v>40</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>1142</v>
+        <v>1145</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>1141</v>
+        <v>1144</v>
       </c>
       <c r="I53" s="3" t="s">
         <v>43</v>
@@ -36896,13 +37015,13 @@
         <v>440</v>
       </c>
       <c r="L53" s="3" t="s">
-        <v>1198</v>
+        <v>1201</v>
       </c>
       <c r="M53" s="3" t="s">
-        <v>1197</v>
+        <v>1200</v>
       </c>
       <c r="N53" s="3" t="s">
-        <v>1196</v>
+        <v>1199</v>
       </c>
       <c r="O53" s="8">
         <v>50</v>
@@ -36926,16 +37045,16 @@
         <v>0</v>
       </c>
       <c r="V53" s="3" t="s">
-        <v>1195</v>
+        <v>1198</v>
       </c>
       <c r="W53" s="3" t="s">
-        <v>1194</v>
+        <v>1197</v>
       </c>
       <c r="X53" s="3" t="s">
         <v>51</v>
       </c>
       <c r="Y53" s="3" t="s">
-        <v>1193</v>
+        <v>1196</v>
       </c>
       <c r="Z53" s="3" t="s">
         <v>0</v>
@@ -36973,13 +37092,13 @@
     </row>
     <row r="54" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>1192</v>
+        <v>1195</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>1192</v>
+        <v>1195</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D54" s="4">
         <v>46072</v>
@@ -36991,10 +37110,10 @@
         <v>61</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>1182</v>
+        <v>1185</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>1181</v>
+        <v>1184</v>
       </c>
       <c r="I54" s="2" t="s">
         <v>163</v>
@@ -37006,13 +37125,13 @@
         <v>417</v>
       </c>
       <c r="L54" s="2" t="s">
-        <v>1172</v>
+        <v>1175</v>
       </c>
       <c r="M54" s="2" t="s">
-        <v>1171</v>
+        <v>1174</v>
       </c>
       <c r="N54" s="2" t="s">
-        <v>1121</v>
+        <v>1124</v>
       </c>
       <c r="O54" s="5">
         <v>1600</v>
@@ -37045,7 +37164,7 @@
         <v>51</v>
       </c>
       <c r="Y54" s="2" t="s">
-        <v>1191</v>
+        <v>1194</v>
       </c>
       <c r="Z54" s="2" t="s">
         <v>0</v>
@@ -37083,13 +37202,13 @@
     </row>
     <row r="55" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
-        <v>1190</v>
+        <v>1193</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>1190</v>
+        <v>1193</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D55" s="7">
         <v>46072</v>
@@ -37101,10 +37220,10 @@
         <v>40</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>1189</v>
+        <v>1192</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>1188</v>
+        <v>1191</v>
       </c>
       <c r="I55" s="3" t="s">
         <v>43</v>
@@ -37116,13 +37235,13 @@
         <v>446</v>
       </c>
       <c r="L55" s="3" t="s">
-        <v>1187</v>
+        <v>1190</v>
       </c>
       <c r="M55" s="3" t="s">
-        <v>1186</v>
+        <v>1189</v>
       </c>
       <c r="N55" s="3" t="s">
-        <v>1185</v>
+        <v>1188</v>
       </c>
       <c r="O55" s="8">
         <v>500</v>
@@ -37155,7 +37274,7 @@
         <v>51</v>
       </c>
       <c r="Y55" s="3" t="s">
-        <v>1184</v>
+        <v>1187</v>
       </c>
       <c r="Z55" s="3" t="s">
         <v>0</v>
@@ -37193,13 +37312,13 @@
     </row>
     <row r="56" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
-        <v>1183</v>
+        <v>1186</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>1183</v>
+        <v>1186</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D56" s="4">
         <v>46076</v>
@@ -37211,10 +37330,10 @@
         <v>61</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>1182</v>
+        <v>1185</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>1181</v>
+        <v>1184</v>
       </c>
       <c r="I56" s="2" t="s">
         <v>163</v>
@@ -37226,13 +37345,13 @@
         <v>417</v>
       </c>
       <c r="L56" s="2" t="s">
-        <v>1172</v>
+        <v>1175</v>
       </c>
       <c r="M56" s="2" t="s">
-        <v>1171</v>
+        <v>1174</v>
       </c>
       <c r="N56" s="2" t="s">
-        <v>1121</v>
+        <v>1124</v>
       </c>
       <c r="O56" s="5">
         <v>1700</v>
@@ -37265,7 +37384,7 @@
         <v>51</v>
       </c>
       <c r="Y56" s="2" t="s">
-        <v>1180</v>
+        <v>1183</v>
       </c>
       <c r="Z56" s="2" t="s">
         <v>0</v>
@@ -37303,13 +37422,13 @@
     </row>
     <row r="57" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
-        <v>1177</v>
+        <v>1180</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>1177</v>
+        <v>1180</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D57" s="7">
         <v>46077</v>
@@ -37333,16 +37452,16 @@
         <v>164</v>
       </c>
       <c r="K57" s="3" t="s">
+        <v>1165</v>
+      </c>
+      <c r="L57" s="3" t="s">
+        <v>1182</v>
+      </c>
+      <c r="M57" s="3" t="s">
+        <v>1181</v>
+      </c>
+      <c r="N57" s="3" t="s">
         <v>1162</v>
-      </c>
-      <c r="L57" s="3" t="s">
-        <v>1179</v>
-      </c>
-      <c r="M57" s="3" t="s">
-        <v>1178</v>
-      </c>
-      <c r="N57" s="3" t="s">
-        <v>1159</v>
       </c>
       <c r="O57" s="8">
         <v>500</v>
@@ -37375,7 +37494,7 @@
         <v>51</v>
       </c>
       <c r="Y57" s="3" t="s">
-        <v>1176</v>
+        <v>1179</v>
       </c>
       <c r="Z57" s="3" t="s">
         <v>0</v>
@@ -37413,13 +37532,13 @@
     </row>
     <row r="58" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
-        <v>1177</v>
+        <v>1180</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>1177</v>
+        <v>1180</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D58" s="4">
         <v>46077</v>
@@ -37443,16 +37562,16 @@
         <v>164</v>
       </c>
       <c r="K58" s="2" t="s">
+        <v>1160</v>
+      </c>
+      <c r="L58" s="2" t="s">
+        <v>1159</v>
+      </c>
+      <c r="M58" s="2" t="s">
+        <v>1158</v>
+      </c>
+      <c r="N58" s="2" t="s">
         <v>1157</v>
-      </c>
-      <c r="L58" s="2" t="s">
-        <v>1156</v>
-      </c>
-      <c r="M58" s="2" t="s">
-        <v>1155</v>
-      </c>
-      <c r="N58" s="2" t="s">
-        <v>1154</v>
       </c>
       <c r="O58" s="5">
         <v>500</v>
@@ -37485,7 +37604,7 @@
         <v>51</v>
       </c>
       <c r="Y58" s="2" t="s">
-        <v>1176</v>
+        <v>1179</v>
       </c>
       <c r="Z58" s="2" t="s">
         <v>0</v>
@@ -37500,10 +37619,10 @@
         <v>111</v>
       </c>
       <c r="AD58" s="2" t="s">
-        <v>1152</v>
+        <v>1155</v>
       </c>
       <c r="AE58" s="2" t="s">
-        <v>1151</v>
+        <v>1154</v>
       </c>
       <c r="AF58" s="2" t="s">
         <v>77</v>
@@ -37523,13 +37642,13 @@
     </row>
     <row r="59" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
-        <v>1175</v>
+        <v>1178</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>1175</v>
+        <v>1178</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D59" s="7">
         <v>46078</v>
@@ -37541,10 +37660,10 @@
         <v>40</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>1131</v>
+        <v>1134</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="I59" s="3" t="s">
         <v>139</v>
@@ -37556,13 +37675,13 @@
         <v>782</v>
       </c>
       <c r="L59" s="3" t="s">
-        <v>1129</v>
+        <v>1132</v>
       </c>
       <c r="M59" s="3" t="s">
-        <v>1128</v>
+        <v>1131</v>
       </c>
       <c r="N59" s="3" t="s">
-        <v>1127</v>
+        <v>1130</v>
       </c>
       <c r="O59" s="8">
         <v>225</v>
@@ -37595,7 +37714,7 @@
         <v>51</v>
       </c>
       <c r="Y59" s="3" t="s">
-        <v>1174</v>
+        <v>1177</v>
       </c>
       <c r="Z59" s="3" t="s">
         <v>0</v>
@@ -37633,13 +37752,13 @@
     </row>
     <row r="60" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
-        <v>1173</v>
+        <v>1176</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>1173</v>
+        <v>1176</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D60" s="4">
         <v>46079</v>
@@ -37666,13 +37785,13 @@
         <v>417</v>
       </c>
       <c r="L60" s="2" t="s">
-        <v>1172</v>
+        <v>1175</v>
       </c>
       <c r="M60" s="2" t="s">
-        <v>1171</v>
+        <v>1174</v>
       </c>
       <c r="N60" s="2" t="s">
-        <v>1121</v>
+        <v>1124</v>
       </c>
       <c r="O60" s="5">
         <v>5000</v>
@@ -37696,16 +37815,16 @@
         <v>2354</v>
       </c>
       <c r="V60" s="2" t="s">
-        <v>1135</v>
+        <v>1138</v>
       </c>
       <c r="W60" s="2" t="s">
-        <v>1134</v>
+        <v>1137</v>
       </c>
       <c r="X60" s="2" t="s">
         <v>51</v>
       </c>
       <c r="Y60" s="2" t="s">
-        <v>1170</v>
+        <v>1173</v>
       </c>
       <c r="Z60" s="2" t="s">
         <v>0</v>
@@ -37743,13 +37862,13 @@
     </row>
     <row r="61" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
-        <v>1169</v>
+        <v>1172</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>1169</v>
+        <v>1172</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D61" s="7">
         <v>46079</v>
@@ -37776,13 +37895,13 @@
         <v>1058</v>
       </c>
       <c r="L61" s="3" t="s">
-        <v>1168</v>
+        <v>1171</v>
       </c>
       <c r="M61" s="3" t="s">
-        <v>1167</v>
+        <v>1170</v>
       </c>
       <c r="N61" s="3" t="s">
-        <v>1166</v>
+        <v>1169</v>
       </c>
       <c r="O61" s="8">
         <v>12000</v>
@@ -37815,7 +37934,7 @@
         <v>51</v>
       </c>
       <c r="Y61" s="3" t="s">
-        <v>1165</v>
+        <v>1168</v>
       </c>
       <c r="Z61" s="3" t="s">
         <v>0</v>
@@ -37853,13 +37972,13 @@
     </row>
     <row r="62" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
-        <v>1164</v>
+        <v>1167</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>1164</v>
+        <v>1167</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D62" s="4">
         <v>46085</v>
@@ -37886,13 +38005,13 @@
         <v>633</v>
       </c>
       <c r="L62" s="2" t="s">
-        <v>1102</v>
+        <v>1105</v>
       </c>
       <c r="M62" s="2" t="s">
         <v>652</v>
       </c>
       <c r="N62" s="2" t="s">
-        <v>1101</v>
+        <v>1104</v>
       </c>
       <c r="O62" s="5">
         <v>5005</v>
@@ -37925,7 +38044,7 @@
         <v>51</v>
       </c>
       <c r="Y62" s="2" t="s">
-        <v>1163</v>
+        <v>1166</v>
       </c>
       <c r="Z62" s="2" t="s">
         <v>0</v>
@@ -37963,13 +38082,13 @@
     </row>
     <row r="63" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
-        <v>1158</v>
+        <v>1161</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>1158</v>
+        <v>1161</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D63" s="7">
         <v>46085</v>
@@ -37993,16 +38112,16 @@
         <v>164</v>
       </c>
       <c r="K63" s="3" t="s">
+        <v>1165</v>
+      </c>
+      <c r="L63" s="3" t="s">
+        <v>1164</v>
+      </c>
+      <c r="M63" s="3" t="s">
+        <v>1163</v>
+      </c>
+      <c r="N63" s="3" t="s">
         <v>1162</v>
-      </c>
-      <c r="L63" s="3" t="s">
-        <v>1161</v>
-      </c>
-      <c r="M63" s="3" t="s">
-        <v>1160</v>
-      </c>
-      <c r="N63" s="3" t="s">
-        <v>1159</v>
       </c>
       <c r="O63" s="8">
         <v>500</v>
@@ -38035,7 +38154,7 @@
         <v>51</v>
       </c>
       <c r="Y63" s="3" t="s">
-        <v>1153</v>
+        <v>1156</v>
       </c>
       <c r="Z63" s="3" t="s">
         <v>0</v>
@@ -38073,13 +38192,13 @@
     </row>
     <row r="64" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
-        <v>1158</v>
+        <v>1161</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>1158</v>
+        <v>1161</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D64" s="4">
         <v>46085</v>
@@ -38103,16 +38222,16 @@
         <v>164</v>
       </c>
       <c r="K64" s="2" t="s">
+        <v>1160</v>
+      </c>
+      <c r="L64" s="2" t="s">
+        <v>1159</v>
+      </c>
+      <c r="M64" s="2" t="s">
+        <v>1158</v>
+      </c>
+      <c r="N64" s="2" t="s">
         <v>1157</v>
-      </c>
-      <c r="L64" s="2" t="s">
-        <v>1156</v>
-      </c>
-      <c r="M64" s="2" t="s">
-        <v>1155</v>
-      </c>
-      <c r="N64" s="2" t="s">
-        <v>1154</v>
       </c>
       <c r="O64" s="5">
         <v>500</v>
@@ -38145,7 +38264,7 @@
         <v>51</v>
       </c>
       <c r="Y64" s="2" t="s">
-        <v>1153</v>
+        <v>1156</v>
       </c>
       <c r="Z64" s="2" t="s">
         <v>0</v>
@@ -38160,10 +38279,10 @@
         <v>111</v>
       </c>
       <c r="AD64" s="2" t="s">
-        <v>1152</v>
+        <v>1155</v>
       </c>
       <c r="AE64" s="2" t="s">
-        <v>1151</v>
+        <v>1154</v>
       </c>
       <c r="AF64" s="2" t="s">
         <v>77</v>
@@ -38183,13 +38302,13 @@
     </row>
     <row r="65" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
-        <v>1150</v>
+        <v>1153</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>1150</v>
+        <v>1153</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D65" s="7">
         <v>46085</v>
@@ -38201,10 +38320,10 @@
         <v>40</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>1149</v>
+        <v>1152</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>1148</v>
+        <v>1151</v>
       </c>
       <c r="I65" s="3" t="s">
         <v>163</v>
@@ -38216,13 +38335,13 @@
         <v>154</v>
       </c>
       <c r="L65" s="3" t="s">
-        <v>1147</v>
+        <v>1150</v>
       </c>
       <c r="M65" s="3" t="s">
-        <v>1146</v>
+        <v>1149</v>
       </c>
       <c r="N65" s="3" t="s">
-        <v>1145</v>
+        <v>1148</v>
       </c>
       <c r="O65" s="8">
         <v>3700</v>
@@ -38255,7 +38374,7 @@
         <v>51</v>
       </c>
       <c r="Y65" s="3" t="s">
-        <v>1144</v>
+        <v>1147</v>
       </c>
       <c r="Z65" s="3" t="s">
         <v>0</v>
@@ -38293,13 +38412,13 @@
     </row>
     <row r="66" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
-        <v>1143</v>
+        <v>1146</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>1143</v>
+        <v>1146</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D66" s="4">
         <v>46085</v>
@@ -38311,10 +38430,10 @@
         <v>40</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>1142</v>
+        <v>1145</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>1141</v>
+        <v>1144</v>
       </c>
       <c r="I66" s="2" t="s">
         <v>139</v>
@@ -38323,7 +38442,7 @@
         <v>140</v>
       </c>
       <c r="K66" s="2" t="s">
-        <v>1140</v>
+        <v>1143</v>
       </c>
       <c r="L66" s="2" t="s">
         <v>0</v>
@@ -38365,7 +38484,7 @@
         <v>0</v>
       </c>
       <c r="Y66" s="2" t="s">
-        <v>1139</v>
+        <v>1142</v>
       </c>
       <c r="Z66" s="2" t="s">
         <v>0</v>
@@ -38380,10 +38499,10 @@
         <v>298</v>
       </c>
       <c r="AD66" s="2" t="s">
-        <v>1138</v>
+        <v>1141</v>
       </c>
       <c r="AE66" s="2" t="s">
-        <v>1137</v>
+        <v>1140</v>
       </c>
       <c r="AF66" s="2" t="s">
         <v>0</v>
@@ -38403,13 +38522,13 @@
     </row>
     <row r="67" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
-        <v>1136</v>
+        <v>1139</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>1136</v>
+        <v>1139</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D67" s="7">
         <v>46091</v>
@@ -38436,13 +38555,13 @@
         <v>417</v>
       </c>
       <c r="L67" s="3" t="s">
-        <v>1123</v>
+        <v>1126</v>
       </c>
       <c r="M67" s="3" t="s">
-        <v>1122</v>
+        <v>1125</v>
       </c>
       <c r="N67" s="3" t="s">
-        <v>1121</v>
+        <v>1124</v>
       </c>
       <c r="O67" s="8">
         <v>5000</v>
@@ -38466,16 +38585,16 @@
         <v>2354</v>
       </c>
       <c r="V67" s="3" t="s">
-        <v>1135</v>
+        <v>1138</v>
       </c>
       <c r="W67" s="3" t="s">
-        <v>1134</v>
+        <v>1137</v>
       </c>
       <c r="X67" s="3" t="s">
         <v>51</v>
       </c>
       <c r="Y67" s="3" t="s">
-        <v>1133</v>
+        <v>1136</v>
       </c>
       <c r="Z67" s="3" t="s">
         <v>0</v>
@@ -38513,13 +38632,13 @@
     </row>
     <row r="68" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
-        <v>1132</v>
+        <v>1135</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>1132</v>
+        <v>1135</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D68" s="4">
         <v>46091</v>
@@ -38531,10 +38650,10 @@
         <v>40</v>
       </c>
       <c r="G68" s="2" t="s">
-        <v>1131</v>
+        <v>1134</v>
       </c>
       <c r="H68" s="2" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="I68" s="2" t="s">
         <v>139</v>
@@ -38546,13 +38665,13 @@
         <v>782</v>
       </c>
       <c r="L68" s="2" t="s">
-        <v>1129</v>
+        <v>1132</v>
       </c>
       <c r="M68" s="2" t="s">
-        <v>1128</v>
+        <v>1131</v>
       </c>
       <c r="N68" s="2" t="s">
-        <v>1127</v>
+        <v>1130</v>
       </c>
       <c r="O68" s="5">
         <v>225</v>
@@ -38585,7 +38704,7 @@
         <v>51</v>
       </c>
       <c r="Y68" s="2" t="s">
-        <v>1126</v>
+        <v>1129</v>
       </c>
       <c r="Z68" s="2" t="s">
         <v>0</v>
@@ -38623,28 +38742,28 @@
     </row>
     <row r="69" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="3" t="s">
-        <v>1117</v>
+        <v>1120</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>1117</v>
+        <v>1120</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D69" s="7">
         <v>46092</v>
       </c>
       <c r="E69" s="3" t="s">
+        <v>1119</v>
+      </c>
+      <c r="F69" s="3" t="s">
+        <v>1118</v>
+      </c>
+      <c r="G69" s="3" t="s">
+        <v>1117</v>
+      </c>
+      <c r="H69" s="3" t="s">
         <v>1116</v>
-      </c>
-      <c r="F69" s="3" t="s">
-        <v>1115</v>
-      </c>
-      <c r="G69" s="3" t="s">
-        <v>1114</v>
-      </c>
-      <c r="H69" s="3" t="s">
-        <v>1113</v>
       </c>
       <c r="I69" s="3" t="s">
         <v>139</v>
@@ -38656,13 +38775,13 @@
         <v>272</v>
       </c>
       <c r="L69" s="3" t="s">
-        <v>1125</v>
+        <v>1128</v>
       </c>
       <c r="M69" s="3" t="s">
         <v>274</v>
       </c>
       <c r="N69" s="3" t="s">
-        <v>1124</v>
+        <v>1127</v>
       </c>
       <c r="O69" s="8">
         <v>10000</v>
@@ -38686,16 +38805,16 @@
         <v>3312.29</v>
       </c>
       <c r="V69" s="3" t="s">
-        <v>1109</v>
+        <v>1112</v>
       </c>
       <c r="W69" s="3" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="X69" s="3" t="s">
         <v>87</v>
       </c>
       <c r="Y69" s="3" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="Z69" s="3" t="s">
         <v>0</v>
@@ -38733,28 +38852,28 @@
     </row>
     <row r="70" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
-        <v>1117</v>
+        <v>1120</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>1117</v>
+        <v>1120</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D70" s="4">
         <v>46092</v>
       </c>
       <c r="E70" s="2" t="s">
+        <v>1119</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>1118</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>1117</v>
+      </c>
+      <c r="H70" s="2" t="s">
         <v>1116</v>
-      </c>
-      <c r="F70" s="2" t="s">
-        <v>1115</v>
-      </c>
-      <c r="G70" s="2" t="s">
-        <v>1114</v>
-      </c>
-      <c r="H70" s="2" t="s">
-        <v>1113</v>
       </c>
       <c r="I70" s="2" t="s">
         <v>139</v>
@@ -38766,13 +38885,13 @@
         <v>417</v>
       </c>
       <c r="L70" s="2" t="s">
-        <v>1123</v>
+        <v>1126</v>
       </c>
       <c r="M70" s="2" t="s">
-        <v>1122</v>
+        <v>1125</v>
       </c>
       <c r="N70" s="2" t="s">
-        <v>1121</v>
+        <v>1124</v>
       </c>
       <c r="O70" s="5">
         <v>5000</v>
@@ -38796,16 +38915,16 @@
         <v>1559.15</v>
       </c>
       <c r="V70" s="2" t="s">
-        <v>1109</v>
+        <v>1112</v>
       </c>
       <c r="W70" s="2" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="X70" s="2" t="s">
         <v>87</v>
       </c>
       <c r="Y70" s="2" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="Z70" s="2" t="s">
         <v>0</v>
@@ -38843,28 +38962,28 @@
     </row>
     <row r="71" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="3" t="s">
-        <v>1117</v>
+        <v>1120</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>1117</v>
+        <v>1120</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D71" s="7">
         <v>46092</v>
       </c>
       <c r="E71" s="3" t="s">
+        <v>1119</v>
+      </c>
+      <c r="F71" s="3" t="s">
+        <v>1118</v>
+      </c>
+      <c r="G71" s="3" t="s">
+        <v>1117</v>
+      </c>
+      <c r="H71" s="3" t="s">
         <v>1116</v>
-      </c>
-      <c r="F71" s="3" t="s">
-        <v>1115</v>
-      </c>
-      <c r="G71" s="3" t="s">
-        <v>1114</v>
-      </c>
-      <c r="H71" s="3" t="s">
-        <v>1113</v>
       </c>
       <c r="I71" s="3" t="s">
         <v>139</v>
@@ -38876,13 +38995,13 @@
         <v>342</v>
       </c>
       <c r="L71" s="3" t="s">
-        <v>1120</v>
+        <v>1123</v>
       </c>
       <c r="M71" s="3" t="s">
-        <v>1119</v>
+        <v>1122</v>
       </c>
       <c r="N71" s="3" t="s">
-        <v>1118</v>
+        <v>1121</v>
       </c>
       <c r="O71" s="8">
         <v>8400</v>
@@ -38906,16 +39025,16 @@
         <v>2580.5300000000002</v>
       </c>
       <c r="V71" s="3" t="s">
-        <v>1109</v>
+        <v>1112</v>
       </c>
       <c r="W71" s="3" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="X71" s="3" t="s">
         <v>87</v>
       </c>
       <c r="Y71" s="3" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="Z71" s="3" t="s">
         <v>0</v>
@@ -38953,28 +39072,28 @@
     </row>
     <row r="72" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
-        <v>1117</v>
+        <v>1120</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>1117</v>
+        <v>1120</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D72" s="4">
         <v>46092</v>
       </c>
       <c r="E72" s="2" t="s">
+        <v>1119</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>1118</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>1117</v>
+      </c>
+      <c r="H72" s="2" t="s">
         <v>1116</v>
-      </c>
-      <c r="F72" s="2" t="s">
-        <v>1115</v>
-      </c>
-      <c r="G72" s="2" t="s">
-        <v>1114</v>
-      </c>
-      <c r="H72" s="2" t="s">
-        <v>1113</v>
       </c>
       <c r="I72" s="2" t="s">
         <v>139</v>
@@ -38986,13 +39105,13 @@
         <v>782</v>
       </c>
       <c r="L72" s="2" t="s">
-        <v>1112</v>
+        <v>1115</v>
       </c>
       <c r="M72" s="2" t="s">
-        <v>1111</v>
+        <v>1114</v>
       </c>
       <c r="N72" s="2" t="s">
-        <v>1110</v>
+        <v>1113</v>
       </c>
       <c r="O72" s="5">
         <v>2400</v>
@@ -39016,16 +39135,16 @@
         <v>775.1</v>
       </c>
       <c r="V72" s="2" t="s">
-        <v>1109</v>
+        <v>1112</v>
       </c>
       <c r="W72" s="2" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="X72" s="2" t="s">
         <v>87</v>
       </c>
       <c r="Y72" s="2" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="Z72" s="2" t="s">
         <v>0</v>
@@ -39063,13 +39182,13 @@
     </row>
     <row r="73" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="3" t="s">
-        <v>1106</v>
+        <v>1109</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>1106</v>
+        <v>1109</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="D73" s="7">
         <v>46093</v>
@@ -39081,10 +39200,10 @@
         <v>61</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>1104</v>
+        <v>1107</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>1103</v>
+        <v>1106</v>
       </c>
       <c r="I73" s="3" t="s">
         <v>163</v>
@@ -39096,13 +39215,13 @@
         <v>633</v>
       </c>
       <c r="L73" s="3" t="s">
-        <v>1102</v>
+        <v>1105</v>
       </c>
       <c r="M73" s="3" t="s">
         <v>652</v>
       </c>
       <c r="N73" s="3" t="s">
-        <v>1101</v>
+        <v>1104</v>
       </c>
       <c r="O73" s="8">
         <v>507</v>
@@ -39135,7 +39254,7 @@
         <v>51</v>
       </c>
       <c r="Y73" s="3" t="s">
-        <v>1100</v>
+        <v>1103</v>
       </c>
       <c r="Z73" s="3" t="s">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização da base de dados 17.03.2026
</commit_message>
<xml_diff>
--- a/BASE_KEMPARTS.xlsx
+++ b/BASE_KEMPARTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dash_kp_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EA8A3F2C-866D-42B3-8A3C-2D6D932EF647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{37747EB9-AC77-457C-916A-EFE6DAB95DC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{923D3E5D-1ACF-4B7D-A9DE-3134991C402F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{EF136881-73C8-429C-8DA8-74B3A074961C}"/>
   </bookViews>
   <sheets>
     <sheet name="FSP" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5497" uniqueCount="1076">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5597" uniqueCount="1084">
   <si>
     <t>Numero</t>
   </si>
@@ -2649,6 +2649,18 @@
     <t>2025.103.08.</t>
   </si>
   <si>
+    <t>000015572</t>
+  </si>
+  <si>
+    <t>C00084</t>
+  </si>
+  <si>
+    <t>COLORART INDUSTRIA E COMERCIO DE TINTAS</t>
+  </si>
+  <si>
+    <t>173896</t>
+  </si>
+  <si>
     <t>000002433</t>
   </si>
   <si>
@@ -3265,6 +3277,18 @@
   </si>
   <si>
     <t>003281</t>
+  </si>
+  <si>
+    <t>000002514</t>
+  </si>
+  <si>
+    <t>003303</t>
+  </si>
+  <si>
+    <t>000002515</t>
+  </si>
+  <si>
+    <t>003320</t>
   </si>
 </sst>
 </file>
@@ -3723,7 +3747,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2E0A97F-906F-4148-9006-57F27B41FC68}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6464A559-2DDB-4F7B-AC86-4AB84A7663F7}">
   <dimension ref="A1:AJ175"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -22023,8 +22047,226 @@
         <v>46573.902600000001</v>
       </c>
     </row>
-    <row r="167" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="168" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="167" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A167" s="2" t="s">
+        <v>870</v>
+      </c>
+      <c r="B167" s="2" t="s">
+        <v>870</v>
+      </c>
+      <c r="C167" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D167" s="3">
+        <v>46098</v>
+      </c>
+      <c r="E167" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F167" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G167" s="2" t="s">
+        <v>871</v>
+      </c>
+      <c r="H167" s="2" t="s">
+        <v>872</v>
+      </c>
+      <c r="I167" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="J167" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="K167" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="L167" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="M167" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="N167" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="O167" s="4">
+        <v>200</v>
+      </c>
+      <c r="P167" s="4">
+        <v>13.99</v>
+      </c>
+      <c r="Q167" s="5">
+        <v>2798</v>
+      </c>
+      <c r="R167" s="5">
+        <v>90.94</v>
+      </c>
+      <c r="S167" s="5">
+        <v>2888.94</v>
+      </c>
+      <c r="T167" s="5">
+        <v>13990</v>
+      </c>
+      <c r="U167" s="5">
+        <v>503.64</v>
+      </c>
+      <c r="V167" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="W167" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="X167" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y167" s="2" t="s">
+        <v>873</v>
+      </c>
+      <c r="Z167" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA167" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB167" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="AC167" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD167" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="AE167" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="AF167" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AG167" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH167" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="AI167" s="5">
+        <v>18</v>
+      </c>
+      <c r="AJ167" s="4">
+        <v>1966.3</v>
+      </c>
+    </row>
+    <row r="168" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A168" s="6" t="s">
+        <v>870</v>
+      </c>
+      <c r="B168" s="6" t="s">
+        <v>870</v>
+      </c>
+      <c r="C168" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D168" s="7">
+        <v>46098</v>
+      </c>
+      <c r="E168" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F168" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="G168" s="6" t="s">
+        <v>871</v>
+      </c>
+      <c r="H168" s="6" t="s">
+        <v>872</v>
+      </c>
+      <c r="I168" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="J168" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="K168" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="L168" s="6" t="s">
+        <v>815</v>
+      </c>
+      <c r="M168" s="6" t="s">
+        <v>816</v>
+      </c>
+      <c r="N168" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="O168" s="8">
+        <v>800</v>
+      </c>
+      <c r="P168" s="8">
+        <v>13.99</v>
+      </c>
+      <c r="Q168" s="9">
+        <v>11192</v>
+      </c>
+      <c r="R168" s="9">
+        <v>363.74</v>
+      </c>
+      <c r="S168" s="9">
+        <v>11555.74</v>
+      </c>
+      <c r="T168" s="9">
+        <v>13990</v>
+      </c>
+      <c r="U168" s="9">
+        <v>2014.56</v>
+      </c>
+      <c r="V168" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="W168" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="X168" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y168" s="6" t="s">
+        <v>873</v>
+      </c>
+      <c r="Z168" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA168" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB168" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="AC168" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="AD168" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="AE168" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="AF168" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="AG168" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH168" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="AI168" s="9">
+        <v>18</v>
+      </c>
+      <c r="AJ168" s="8">
+        <v>7865.2</v>
+      </c>
+    </row>
     <row r="169" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="170" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="171" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -22038,7 +22280,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA6E2153-9182-4875-A12C-C48238189A2F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91012DBE-85F6-4275-8A99-FD2D47C0B73C}">
   <dimension ref="A1:AJ63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -22189,13 +22431,13 @@
     </row>
     <row r="2" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>870</v>
+        <v>874</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>870</v>
+        <v>874</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D2" s="3">
         <v>46024</v>
@@ -22207,10 +22449,10 @@
         <v>39</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>872</v>
+        <v>876</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>873</v>
+        <v>877</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>42</v>
@@ -22219,16 +22461,16 @@
         <v>43</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>874</v>
+        <v>878</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>875</v>
+        <v>879</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>876</v>
+        <v>880</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>877</v>
+        <v>881</v>
       </c>
       <c r="O2" s="4">
         <v>50</v>
@@ -22252,16 +22494,16 @@
         <v>39.06</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>878</v>
+        <v>882</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>879</v>
+        <v>883</v>
       </c>
       <c r="X2" s="2" t="s">
         <v>50</v>
       </c>
       <c r="Y2" s="2" t="s">
-        <v>880</v>
+        <v>884</v>
       </c>
       <c r="Z2" s="2" t="s">
         <v>52</v>
@@ -22299,13 +22541,13 @@
     </row>
     <row r="3" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>881</v>
+        <v>885</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>881</v>
+        <v>885</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D3" s="7">
         <v>46027</v>
@@ -22317,10 +22559,10 @@
         <v>61</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>882</v>
+        <v>886</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="I3" s="6" t="s">
         <v>148</v>
@@ -22329,16 +22571,16 @@
         <v>149</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>884</v>
+        <v>888</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>885</v>
+        <v>889</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>886</v>
+        <v>890</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="O3" s="8">
         <v>1001</v>
@@ -22371,7 +22613,7 @@
         <v>50</v>
       </c>
       <c r="Y3" s="6" t="s">
-        <v>888</v>
+        <v>892</v>
       </c>
       <c r="Z3" s="6" t="s">
         <v>52</v>
@@ -22409,13 +22651,13 @@
     </row>
     <row r="4" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>889</v>
+        <v>893</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>889</v>
+        <v>893</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D4" s="3">
         <v>46027</v>
@@ -22427,10 +22669,10 @@
         <v>61</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>890</v>
+        <v>894</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>891</v>
+        <v>895</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>137</v>
@@ -22442,13 +22684,13 @@
         <v>441</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>892</v>
+        <v>896</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>893</v>
+        <v>897</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>894</v>
+        <v>898</v>
       </c>
       <c r="O4" s="4">
         <v>600</v>
@@ -22472,16 +22714,16 @@
         <v>355.68</v>
       </c>
       <c r="V4" s="2" t="s">
-        <v>895</v>
+        <v>899</v>
       </c>
       <c r="W4" s="2" t="s">
-        <v>896</v>
+        <v>900</v>
       </c>
       <c r="X4" s="2" t="s">
         <v>50</v>
       </c>
       <c r="Y4" s="2" t="s">
-        <v>897</v>
+        <v>901</v>
       </c>
       <c r="Z4" s="2" t="s">
         <v>52</v>
@@ -22519,13 +22761,13 @@
     </row>
     <row r="5" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>898</v>
+        <v>902</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>898</v>
+        <v>902</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D5" s="7">
         <v>46029</v>
@@ -22543,22 +22785,22 @@
         <v>330</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>899</v>
+        <v>903</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>900</v>
+        <v>904</v>
       </c>
       <c r="K5" s="6" t="s">
         <v>852</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>901</v>
+        <v>905</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>902</v>
+        <v>906</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>903</v>
+        <v>907</v>
       </c>
       <c r="O5" s="8">
         <v>1000</v>
@@ -22591,7 +22833,7 @@
         <v>50</v>
       </c>
       <c r="Y5" s="6" t="s">
-        <v>904</v>
+        <v>908</v>
       </c>
       <c r="Z5" s="6" t="s">
         <v>52</v>
@@ -22629,13 +22871,13 @@
     </row>
     <row r="6" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>905</v>
+        <v>909</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>905</v>
+        <v>909</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D6" s="3">
         <v>46036</v>
@@ -22647,10 +22889,10 @@
         <v>61</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>882</v>
+        <v>886</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>148</v>
@@ -22659,16 +22901,16 @@
         <v>149</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>884</v>
+        <v>888</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>885</v>
+        <v>889</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>886</v>
+        <v>890</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="O6" s="4">
         <v>1001</v>
@@ -22701,7 +22943,7 @@
         <v>50</v>
       </c>
       <c r="Y6" s="2" t="s">
-        <v>906</v>
+        <v>910</v>
       </c>
       <c r="Z6" s="2" t="s">
         <v>52</v>
@@ -22739,13 +22981,13 @@
     </row>
     <row r="7" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>907</v>
+        <v>911</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>907</v>
+        <v>911</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D7" s="7">
         <v>46037</v>
@@ -22757,10 +22999,10 @@
         <v>61</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>908</v>
+        <v>912</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>909</v>
+        <v>913</v>
       </c>
       <c r="I7" s="6" t="s">
         <v>148</v>
@@ -22772,13 +23014,13 @@
         <v>361</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>910</v>
+        <v>914</v>
       </c>
       <c r="M7" s="6" t="s">
         <v>816</v>
       </c>
       <c r="N7" s="6" t="s">
-        <v>911</v>
+        <v>915</v>
       </c>
       <c r="O7" s="8">
         <v>1000</v>
@@ -22811,7 +23053,7 @@
         <v>50</v>
       </c>
       <c r="Y7" s="6" t="s">
-        <v>912</v>
+        <v>916</v>
       </c>
       <c r="Z7" s="6" t="s">
         <v>52</v>
@@ -22849,13 +23091,13 @@
     </row>
     <row r="8" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>913</v>
+        <v>917</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>913</v>
+        <v>917</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D8" s="3">
         <v>46037</v>
@@ -22867,10 +23109,10 @@
         <v>39</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>914</v>
+        <v>918</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>915</v>
+        <v>919</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>174</v>
@@ -22879,16 +23121,16 @@
         <v>175</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>916</v>
+        <v>920</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>917</v>
+        <v>921</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>918</v>
+        <v>922</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>919</v>
+        <v>923</v>
       </c>
       <c r="O8" s="4">
         <v>300</v>
@@ -22921,7 +23163,7 @@
         <v>50</v>
       </c>
       <c r="Y8" s="2" t="s">
-        <v>920</v>
+        <v>924</v>
       </c>
       <c r="Z8" s="2" t="s">
         <v>52</v>
@@ -22959,13 +23201,13 @@
     </row>
     <row r="9" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>921</v>
+        <v>925</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>921</v>
+        <v>925</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D9" s="7">
         <v>46037</v>
@@ -22977,10 +23219,10 @@
         <v>39</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>922</v>
+        <v>926</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>923</v>
+        <v>927</v>
       </c>
       <c r="I9" s="6" t="s">
         <v>42</v>
@@ -22992,13 +23234,13 @@
         <v>494</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>924</v>
+        <v>928</v>
       </c>
       <c r="M9" s="6" t="s">
-        <v>925</v>
+        <v>929</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>926</v>
+        <v>930</v>
       </c>
       <c r="O9" s="8">
         <v>25</v>
@@ -23031,7 +23273,7 @@
         <v>50</v>
       </c>
       <c r="Y9" s="6" t="s">
-        <v>927</v>
+        <v>931</v>
       </c>
       <c r="Z9" s="6" t="s">
         <v>52</v>
@@ -23069,13 +23311,13 @@
     </row>
     <row r="10" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>928</v>
+        <v>932</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>928</v>
+        <v>932</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D10" s="7">
         <v>46042</v>
@@ -23093,22 +23335,22 @@
         <v>330</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>899</v>
+        <v>903</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>900</v>
+        <v>904</v>
       </c>
       <c r="K10" s="6" t="s">
         <v>382</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>929</v>
+        <v>933</v>
       </c>
       <c r="M10" s="6" t="s">
-        <v>930</v>
+        <v>934</v>
       </c>
       <c r="N10" s="6" t="s">
-        <v>931</v>
+        <v>935</v>
       </c>
       <c r="O10" s="8">
         <v>2000</v>
@@ -23141,7 +23383,7 @@
         <v>50</v>
       </c>
       <c r="Y10" s="6" t="s">
-        <v>932</v>
+        <v>936</v>
       </c>
       <c r="Z10" s="6" t="s">
         <v>52</v>
@@ -23179,13 +23421,13 @@
     </row>
     <row r="11" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>933</v>
+        <v>937</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>933</v>
+        <v>937</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D11" s="3">
         <v>46042</v>
@@ -23209,16 +23451,16 @@
         <v>276</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>934</v>
+        <v>938</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>935</v>
+        <v>939</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>936</v>
+        <v>940</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>937</v>
+        <v>941</v>
       </c>
       <c r="O11" s="4">
         <v>6000</v>
@@ -23242,16 +23484,16 @@
         <v>12873.6</v>
       </c>
       <c r="V11" s="2" t="s">
-        <v>938</v>
+        <v>942</v>
       </c>
       <c r="W11" s="2" t="s">
-        <v>939</v>
+        <v>943</v>
       </c>
       <c r="X11" s="2" t="s">
         <v>50</v>
       </c>
       <c r="Y11" s="2" t="s">
-        <v>940</v>
+        <v>944</v>
       </c>
       <c r="Z11" s="2" t="s">
         <v>52</v>
@@ -23266,10 +23508,10 @@
         <v>280</v>
       </c>
       <c r="AD11" s="2" t="s">
-        <v>941</v>
+        <v>945</v>
       </c>
       <c r="AE11" s="2" t="s">
-        <v>942</v>
+        <v>946</v>
       </c>
       <c r="AF11" s="2" t="s">
         <v>77</v>
@@ -23289,13 +23531,13 @@
     </row>
     <row r="12" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>943</v>
+        <v>947</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>943</v>
+        <v>947</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D12" s="7">
         <v>46043</v>
@@ -23307,10 +23549,10 @@
         <v>61</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>944</v>
+        <v>948</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>945</v>
+        <v>949</v>
       </c>
       <c r="I12" s="6" t="s">
         <v>42</v>
@@ -23322,13 +23564,13 @@
         <v>361</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>946</v>
+        <v>950</v>
       </c>
       <c r="M12" s="6" t="s">
-        <v>947</v>
+        <v>951</v>
       </c>
       <c r="N12" s="6" t="s">
-        <v>911</v>
+        <v>915</v>
       </c>
       <c r="O12" s="8">
         <v>1000</v>
@@ -23361,7 +23603,7 @@
         <v>50</v>
       </c>
       <c r="Y12" s="6" t="s">
-        <v>948</v>
+        <v>952</v>
       </c>
       <c r="Z12" s="6" t="s">
         <v>52</v>
@@ -23399,13 +23641,13 @@
     </row>
     <row r="13" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>949</v>
+        <v>953</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>949</v>
+        <v>953</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D13" s="7">
         <v>46048</v>
@@ -23417,10 +23659,10 @@
         <v>39</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>950</v>
+        <v>954</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>951</v>
+        <v>955</v>
       </c>
       <c r="I13" s="6" t="s">
         <v>137</v>
@@ -23432,13 +23674,13 @@
         <v>361</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>952</v>
+        <v>956</v>
       </c>
       <c r="M13" s="6" t="s">
-        <v>953</v>
+        <v>957</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>954</v>
+        <v>958</v>
       </c>
       <c r="O13" s="8">
         <v>5000</v>
@@ -23462,16 +23704,16 @@
         <v>2354</v>
       </c>
       <c r="V13" s="6" t="s">
-        <v>955</v>
+        <v>959</v>
       </c>
       <c r="W13" s="6" t="s">
-        <v>956</v>
+        <v>960</v>
       </c>
       <c r="X13" s="6" t="s">
         <v>50</v>
       </c>
       <c r="Y13" s="6" t="s">
-        <v>957</v>
+        <v>961</v>
       </c>
       <c r="Z13" s="6" t="s">
         <v>52</v>
@@ -23509,13 +23751,13 @@
     </row>
     <row r="14" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>958</v>
+        <v>962</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>958</v>
+        <v>962</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D14" s="3">
         <v>46048</v>
@@ -23527,10 +23769,10 @@
         <v>39</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>914</v>
+        <v>918</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>915</v>
+        <v>919</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>174</v>
@@ -23539,16 +23781,16 @@
         <v>175</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>916</v>
+        <v>920</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>917</v>
+        <v>921</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>918</v>
+        <v>922</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>919</v>
+        <v>923</v>
       </c>
       <c r="O14" s="4">
         <v>300</v>
@@ -23581,7 +23823,7 @@
         <v>50</v>
       </c>
       <c r="Y14" s="2" t="s">
-        <v>959</v>
+        <v>963</v>
       </c>
       <c r="Z14" s="2" t="s">
         <v>52</v>
@@ -23619,13 +23861,13 @@
     </row>
     <row r="15" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>960</v>
+        <v>964</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>960</v>
+        <v>964</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D15" s="7">
         <v>46048</v>
@@ -23637,10 +23879,10 @@
         <v>61</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>882</v>
+        <v>886</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="I15" s="6" t="s">
         <v>148</v>
@@ -23649,16 +23891,16 @@
         <v>149</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>884</v>
+        <v>888</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>885</v>
+        <v>889</v>
       </c>
       <c r="M15" s="6" t="s">
-        <v>886</v>
+        <v>890</v>
       </c>
       <c r="N15" s="6" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="O15" s="8">
         <v>611</v>
@@ -23691,7 +23933,7 @@
         <v>50</v>
       </c>
       <c r="Y15" s="6" t="s">
-        <v>961</v>
+        <v>965</v>
       </c>
       <c r="Z15" s="6" t="s">
         <v>52</v>
@@ -23729,13 +23971,13 @@
     </row>
     <row r="16" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>960</v>
+        <v>964</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>960</v>
+        <v>964</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D16" s="3">
         <v>46048</v>
@@ -23747,10 +23989,10 @@
         <v>61</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>882</v>
+        <v>886</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>148</v>
@@ -23759,16 +24001,16 @@
         <v>149</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>934</v>
+        <v>938</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>935</v>
+        <v>939</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>936</v>
+        <v>940</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>937</v>
+        <v>941</v>
       </c>
       <c r="O16" s="4">
         <v>700</v>
@@ -23801,7 +24043,7 @@
         <v>50</v>
       </c>
       <c r="Y16" s="2" t="s">
-        <v>961</v>
+        <v>965</v>
       </c>
       <c r="Z16" s="2" t="s">
         <v>52</v>
@@ -23816,10 +24058,10 @@
         <v>55</v>
       </c>
       <c r="AD16" s="2" t="s">
-        <v>941</v>
+        <v>945</v>
       </c>
       <c r="AE16" s="2" t="s">
-        <v>942</v>
+        <v>946</v>
       </c>
       <c r="AF16" s="2" t="s">
         <v>77</v>
@@ -23839,13 +24081,13 @@
     </row>
     <row r="17" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>962</v>
+        <v>966</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>962</v>
+        <v>966</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D17" s="3">
         <v>46050</v>
@@ -23863,22 +24105,22 @@
         <v>330</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>899</v>
+        <v>903</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>900</v>
+        <v>904</v>
       </c>
       <c r="K17" s="2" t="s">
         <v>382</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>963</v>
+        <v>967</v>
       </c>
       <c r="M17" s="2" t="s">
         <v>384</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>964</v>
+        <v>968</v>
       </c>
       <c r="O17" s="4">
         <v>1000</v>
@@ -23911,7 +24153,7 @@
         <v>50</v>
       </c>
       <c r="Y17" s="2" t="s">
-        <v>965</v>
+        <v>969</v>
       </c>
       <c r="Z17" s="2" t="s">
         <v>52</v>
@@ -23949,13 +24191,13 @@
     </row>
     <row r="18" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>962</v>
+        <v>966</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>962</v>
+        <v>966</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D18" s="7">
         <v>46050</v>
@@ -23973,22 +24215,22 @@
         <v>330</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>899</v>
+        <v>903</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>900</v>
+        <v>904</v>
       </c>
       <c r="K18" s="6" t="s">
         <v>382</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>929</v>
+        <v>933</v>
       </c>
       <c r="M18" s="6" t="s">
-        <v>930</v>
+        <v>934</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>931</v>
+        <v>935</v>
       </c>
       <c r="O18" s="8">
         <v>1000</v>
@@ -24021,7 +24263,7 @@
         <v>50</v>
       </c>
       <c r="Y18" s="6" t="s">
-        <v>965</v>
+        <v>969</v>
       </c>
       <c r="Z18" s="6" t="s">
         <v>52</v>
@@ -24059,13 +24301,13 @@
     </row>
     <row r="19" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>966</v>
+        <v>970</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>966</v>
+        <v>970</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D19" s="7">
         <v>46051</v>
@@ -24077,10 +24319,10 @@
         <v>39</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>922</v>
+        <v>926</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>923</v>
+        <v>927</v>
       </c>
       <c r="I19" s="6" t="s">
         <v>42</v>
@@ -24089,16 +24331,16 @@
         <v>43</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>884</v>
+        <v>888</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>885</v>
+        <v>889</v>
       </c>
       <c r="M19" s="6" t="s">
-        <v>886</v>
+        <v>890</v>
       </c>
       <c r="N19" s="6" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="O19" s="8">
         <v>26</v>
@@ -24131,7 +24373,7 @@
         <v>50</v>
       </c>
       <c r="Y19" s="6" t="s">
-        <v>967</v>
+        <v>971</v>
       </c>
       <c r="Z19" s="6" t="s">
         <v>52</v>
@@ -24169,13 +24411,13 @@
     </row>
     <row r="20" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>968</v>
+        <v>972</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>968</v>
+        <v>972</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D20" s="3">
         <v>46052</v>
@@ -24187,10 +24429,10 @@
         <v>61</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>882</v>
+        <v>886</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>148</v>
@@ -24199,16 +24441,16 @@
         <v>149</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>884</v>
+        <v>888</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>885</v>
+        <v>889</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>886</v>
+        <v>890</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="O20" s="4">
         <v>507</v>
@@ -24241,7 +24483,7 @@
         <v>50</v>
       </c>
       <c r="Y20" s="2" t="s">
-        <v>969</v>
+        <v>973</v>
       </c>
       <c r="Z20" s="2" t="s">
         <v>52</v>
@@ -24279,13 +24521,13 @@
     </row>
     <row r="21" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>970</v>
+        <v>974</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>970</v>
+        <v>974</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D21" s="7">
         <v>46052</v>
@@ -24309,16 +24551,16 @@
         <v>149</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>971</v>
+        <v>975</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>972</v>
+        <v>976</v>
       </c>
       <c r="M21" s="6" t="s">
-        <v>973</v>
+        <v>977</v>
       </c>
       <c r="N21" s="6" t="s">
-        <v>974</v>
+        <v>978</v>
       </c>
       <c r="O21" s="8">
         <v>500</v>
@@ -24351,7 +24593,7 @@
         <v>50</v>
       </c>
       <c r="Y21" s="6" t="s">
-        <v>975</v>
+        <v>979</v>
       </c>
       <c r="Z21" s="6" t="s">
         <v>52</v>
@@ -24389,13 +24631,13 @@
     </row>
     <row r="22" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>976</v>
+        <v>980</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>976</v>
+        <v>980</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D22" s="3">
         <v>46052</v>
@@ -24407,10 +24649,10 @@
         <v>39</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>914</v>
+        <v>918</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>915</v>
+        <v>919</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>174</v>
@@ -24419,16 +24661,16 @@
         <v>175</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>916</v>
+        <v>920</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>917</v>
+        <v>921</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>918</v>
+        <v>922</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>919</v>
+        <v>923</v>
       </c>
       <c r="O22" s="4">
         <v>300</v>
@@ -24461,7 +24703,7 @@
         <v>50</v>
       </c>
       <c r="Y22" s="2" t="s">
-        <v>977</v>
+        <v>981</v>
       </c>
       <c r="Z22" s="2" t="s">
         <v>52</v>
@@ -24499,13 +24741,13 @@
     </row>
     <row r="23" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>978</v>
+        <v>982</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>978</v>
+        <v>982</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D23" s="3">
         <v>46057</v>
@@ -24517,10 +24759,10 @@
         <v>61</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>882</v>
+        <v>886</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>148</v>
@@ -24529,16 +24771,16 @@
         <v>149</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>884</v>
+        <v>888</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>885</v>
+        <v>889</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>886</v>
+        <v>890</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="O23" s="4">
         <v>507</v>
@@ -24571,7 +24813,7 @@
         <v>50</v>
       </c>
       <c r="Y23" s="2" t="s">
-        <v>979</v>
+        <v>983</v>
       </c>
       <c r="Z23" s="2" t="s">
         <v>52</v>
@@ -24609,13 +24851,13 @@
     </row>
     <row r="24" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>980</v>
+        <v>984</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>980</v>
+        <v>984</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D24" s="7">
         <v>46057</v>
@@ -24633,22 +24875,22 @@
         <v>330</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>899</v>
+        <v>903</v>
       </c>
       <c r="J24" s="6" t="s">
-        <v>900</v>
+        <v>904</v>
       </c>
       <c r="K24" s="6" t="s">
         <v>382</v>
       </c>
       <c r="L24" s="6" t="s">
-        <v>929</v>
+        <v>933</v>
       </c>
       <c r="M24" s="6" t="s">
-        <v>930</v>
+        <v>934</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>931</v>
+        <v>935</v>
       </c>
       <c r="O24" s="8">
         <v>2000</v>
@@ -24681,7 +24923,7 @@
         <v>50</v>
       </c>
       <c r="Y24" s="6" t="s">
-        <v>981</v>
+        <v>985</v>
       </c>
       <c r="Z24" s="6" t="s">
         <v>52</v>
@@ -24719,13 +24961,13 @@
     </row>
     <row r="25" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>982</v>
+        <v>986</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>982</v>
+        <v>986</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D25" s="3">
         <v>46058</v>
@@ -24737,10 +24979,10 @@
         <v>61</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>882</v>
+        <v>886</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>148</v>
@@ -24749,16 +24991,16 @@
         <v>149</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>884</v>
+        <v>888</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>885</v>
+        <v>889</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>886</v>
+        <v>890</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="O25" s="4">
         <v>507</v>
@@ -24791,7 +25033,7 @@
         <v>50</v>
       </c>
       <c r="Y25" s="2" t="s">
-        <v>983</v>
+        <v>987</v>
       </c>
       <c r="Z25" s="2" t="s">
         <v>52</v>
@@ -24829,13 +25071,13 @@
     </row>
     <row r="26" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>984</v>
+        <v>988</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>984</v>
+        <v>988</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D26" s="7">
         <v>46058</v>
@@ -24847,10 +25089,10 @@
         <v>61</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>985</v>
+        <v>989</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>986</v>
+        <v>990</v>
       </c>
       <c r="I26" s="6" t="s">
         <v>148</v>
@@ -24862,13 +25104,13 @@
         <v>361</v>
       </c>
       <c r="L26" s="6" t="s">
-        <v>952</v>
+        <v>956</v>
       </c>
       <c r="M26" s="6" t="s">
-        <v>953</v>
+        <v>957</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>954</v>
+        <v>958</v>
       </c>
       <c r="O26" s="8">
         <v>1800</v>
@@ -24901,7 +25143,7 @@
         <v>50</v>
       </c>
       <c r="Y26" s="6" t="s">
-        <v>987</v>
+        <v>991</v>
       </c>
       <c r="Z26" s="6" t="s">
         <v>52</v>
@@ -24939,13 +25181,13 @@
     </row>
     <row r="27" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>988</v>
+        <v>992</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>988</v>
+        <v>992</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D27" s="3">
         <v>46059</v>
@@ -24957,10 +25199,10 @@
         <v>39</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>989</v>
+        <v>993</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>990</v>
+        <v>994</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>42</v>
@@ -24969,16 +25211,16 @@
         <v>43</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>916</v>
+        <v>920</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>917</v>
+        <v>921</v>
       </c>
       <c r="M27" s="2" t="s">
-        <v>918</v>
+        <v>922</v>
       </c>
       <c r="N27" s="2" t="s">
-        <v>919</v>
+        <v>923</v>
       </c>
       <c r="O27" s="4">
         <v>500</v>
@@ -25011,7 +25253,7 @@
         <v>50</v>
       </c>
       <c r="Y27" s="2" t="s">
-        <v>991</v>
+        <v>995</v>
       </c>
       <c r="Z27" s="2" t="s">
         <v>52</v>
@@ -25049,13 +25291,13 @@
     </row>
     <row r="28" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>992</v>
+        <v>996</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>992</v>
+        <v>996</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D28" s="7">
         <v>46059</v>
@@ -25067,10 +25309,10 @@
         <v>39</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>993</v>
+        <v>997</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>994</v>
+        <v>998</v>
       </c>
       <c r="I28" s="6" t="s">
         <v>42</v>
@@ -25082,13 +25324,13 @@
         <v>361</v>
       </c>
       <c r="L28" s="6" t="s">
-        <v>952</v>
+        <v>956</v>
       </c>
       <c r="M28" s="6" t="s">
-        <v>953</v>
+        <v>957</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>954</v>
+        <v>958</v>
       </c>
       <c r="O28" s="8">
         <v>200</v>
@@ -25121,7 +25363,7 @@
         <v>50</v>
       </c>
       <c r="Y28" s="6" t="s">
-        <v>995</v>
+        <v>999</v>
       </c>
       <c r="Z28" s="6" t="s">
         <v>52</v>
@@ -25159,28 +25401,28 @@
     </row>
     <row r="29" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>996</v>
+        <v>1000</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>996</v>
+        <v>1000</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D29" s="3">
         <v>46063</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>997</v>
+        <v>1001</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>249</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>998</v>
+        <v>1002</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>999</v>
+        <v>1003</v>
       </c>
       <c r="I29" s="2" t="s">
         <v>174</v>
@@ -25189,7 +25431,7 @@
         <v>175</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>1000</v>
+        <v>1004</v>
       </c>
       <c r="L29" s="2" t="s">
         <v>52</v>
@@ -25231,7 +25473,7 @@
         <v>52</v>
       </c>
       <c r="Y29" s="2" t="s">
-        <v>1001</v>
+        <v>1005</v>
       </c>
       <c r="Z29" s="2" t="s">
         <v>52</v>
@@ -25240,16 +25482,16 @@
         <v>53</v>
       </c>
       <c r="AB29" s="2" t="s">
-        <v>1002</v>
+        <v>1006</v>
       </c>
       <c r="AC29" s="2" t="s">
         <v>74</v>
       </c>
       <c r="AD29" s="2" t="s">
-        <v>1003</v>
+        <v>1007</v>
       </c>
       <c r="AE29" s="2" t="s">
-        <v>1004</v>
+        <v>1008</v>
       </c>
       <c r="AF29" s="2" t="s">
         <v>52</v>
@@ -25269,13 +25511,13 @@
     </row>
     <row r="30" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>1005</v>
+        <v>1009</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>1005</v>
+        <v>1009</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D30" s="7">
         <v>46064</v>
@@ -25287,10 +25529,10 @@
         <v>61</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>908</v>
+        <v>912</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>909</v>
+        <v>913</v>
       </c>
       <c r="I30" s="6" t="s">
         <v>174</v>
@@ -25302,13 +25544,13 @@
         <v>361</v>
       </c>
       <c r="L30" s="6" t="s">
-        <v>946</v>
+        <v>950</v>
       </c>
       <c r="M30" s="6" t="s">
-        <v>947</v>
+        <v>951</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>911</v>
+        <v>915</v>
       </c>
       <c r="O30" s="8">
         <v>1000</v>
@@ -25341,7 +25583,7 @@
         <v>50</v>
       </c>
       <c r="Y30" s="6" t="s">
-        <v>1006</v>
+        <v>1010</v>
       </c>
       <c r="Z30" s="6" t="s">
         <v>52</v>
@@ -25379,13 +25621,13 @@
     </row>
     <row r="31" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>1007</v>
+        <v>1011</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>1007</v>
+        <v>1011</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D31" s="3">
         <v>46064</v>
@@ -25403,22 +25645,22 @@
         <v>330</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>899</v>
+        <v>903</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>900</v>
+        <v>904</v>
       </c>
       <c r="K31" s="2" t="s">
         <v>382</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>929</v>
+        <v>933</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>930</v>
+        <v>934</v>
       </c>
       <c r="N31" s="2" t="s">
-        <v>931</v>
+        <v>935</v>
       </c>
       <c r="O31" s="4">
         <v>1000</v>
@@ -25451,7 +25693,7 @@
         <v>50</v>
       </c>
       <c r="Y31" s="2" t="s">
-        <v>981</v>
+        <v>985</v>
       </c>
       <c r="Z31" s="2" t="s">
         <v>52</v>
@@ -25489,13 +25731,13 @@
     </row>
     <row r="32" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>1007</v>
+        <v>1011</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>1007</v>
+        <v>1011</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D32" s="7">
         <v>46064</v>
@@ -25513,22 +25755,22 @@
         <v>330</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>899</v>
+        <v>903</v>
       </c>
       <c r="J32" s="6" t="s">
-        <v>900</v>
+        <v>904</v>
       </c>
       <c r="K32" s="6" t="s">
         <v>382</v>
       </c>
       <c r="L32" s="6" t="s">
-        <v>1008</v>
+        <v>1012</v>
       </c>
       <c r="M32" s="6" t="s">
-        <v>1009</v>
+        <v>1013</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>931</v>
+        <v>935</v>
       </c>
       <c r="O32" s="8">
         <v>1000</v>
@@ -25561,7 +25803,7 @@
         <v>50</v>
       </c>
       <c r="Y32" s="6" t="s">
-        <v>981</v>
+        <v>985</v>
       </c>
       <c r="Z32" s="6" t="s">
         <v>52</v>
@@ -25599,13 +25841,13 @@
     </row>
     <row r="33" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>1010</v>
+        <v>1014</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>1010</v>
+        <v>1014</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D33" s="3">
         <v>46066</v>
@@ -25617,10 +25859,10 @@
         <v>61</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>882</v>
+        <v>886</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="I33" s="2" t="s">
         <v>148</v>
@@ -25629,16 +25871,16 @@
         <v>149</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>884</v>
+        <v>888</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>885</v>
+        <v>889</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>886</v>
+        <v>890</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="O33" s="4">
         <v>507</v>
@@ -25671,7 +25913,7 @@
         <v>50</v>
       </c>
       <c r="Y33" s="2" t="s">
-        <v>1011</v>
+        <v>1015</v>
       </c>
       <c r="Z33" s="2" t="s">
         <v>52</v>
@@ -25709,13 +25951,13 @@
     </row>
     <row r="34" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>1012</v>
+        <v>1016</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>1012</v>
+        <v>1016</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D34" s="7">
         <v>46071</v>
@@ -25739,16 +25981,16 @@
         <v>149</v>
       </c>
       <c r="K34" s="6" t="s">
-        <v>934</v>
+        <v>938</v>
       </c>
       <c r="L34" s="6" t="s">
-        <v>1013</v>
+        <v>1017</v>
       </c>
       <c r="M34" s="6" t="s">
-        <v>1014</v>
+        <v>1018</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>1015</v>
+        <v>1019</v>
       </c>
       <c r="O34" s="8">
         <v>500</v>
@@ -25781,7 +26023,7 @@
         <v>50</v>
       </c>
       <c r="Y34" s="6" t="s">
-        <v>1016</v>
+        <v>1020</v>
       </c>
       <c r="Z34" s="6" t="s">
         <v>52</v>
@@ -25796,10 +26038,10 @@
         <v>111</v>
       </c>
       <c r="AD34" s="6" t="s">
-        <v>941</v>
+        <v>945</v>
       </c>
       <c r="AE34" s="6" t="s">
-        <v>942</v>
+        <v>946</v>
       </c>
       <c r="AF34" s="6" t="s">
         <v>77</v>
@@ -25819,13 +26061,13 @@
     </row>
     <row r="35" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>1017</v>
+        <v>1021</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>1017</v>
+        <v>1021</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D35" s="3">
         <v>46071</v>
@@ -25837,10 +26079,10 @@
         <v>61</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>1018</v>
+        <v>1022</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>1019</v>
+        <v>1023</v>
       </c>
       <c r="I35" s="2" t="s">
         <v>174</v>
@@ -25852,13 +26094,13 @@
         <v>382</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>1008</v>
+        <v>1012</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>1009</v>
+        <v>1013</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>931</v>
+        <v>935</v>
       </c>
       <c r="O35" s="4">
         <v>200</v>
@@ -25891,7 +26133,7 @@
         <v>50</v>
       </c>
       <c r="Y35" s="2" t="s">
-        <v>1020</v>
+        <v>1024</v>
       </c>
       <c r="Z35" s="2" t="s">
         <v>52</v>
@@ -25929,13 +26171,13 @@
     </row>
     <row r="36" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>1021</v>
+        <v>1025</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>1021</v>
+        <v>1025</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D36" s="7">
         <v>46072</v>
@@ -25947,10 +26189,10 @@
         <v>39</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>872</v>
+        <v>876</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>873</v>
+        <v>877</v>
       </c>
       <c r="I36" s="6" t="s">
         <v>42</v>
@@ -25959,16 +26201,16 @@
         <v>43</v>
       </c>
       <c r="K36" s="6" t="s">
-        <v>874</v>
+        <v>878</v>
       </c>
       <c r="L36" s="6" t="s">
-        <v>875</v>
+        <v>879</v>
       </c>
       <c r="M36" s="6" t="s">
-        <v>876</v>
+        <v>880</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>877</v>
+        <v>881</v>
       </c>
       <c r="O36" s="8">
         <v>50</v>
@@ -25992,16 +26234,16 @@
         <v>0</v>
       </c>
       <c r="V36" s="6" t="s">
-        <v>878</v>
+        <v>882</v>
       </c>
       <c r="W36" s="6" t="s">
-        <v>879</v>
+        <v>883</v>
       </c>
       <c r="X36" s="6" t="s">
         <v>50</v>
       </c>
       <c r="Y36" s="6" t="s">
-        <v>1022</v>
+        <v>1026</v>
       </c>
       <c r="Z36" s="6" t="s">
         <v>52</v>
@@ -26039,13 +26281,13 @@
     </row>
     <row r="37" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>1023</v>
+        <v>1027</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>1023</v>
+        <v>1027</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D37" s="3">
         <v>46072</v>
@@ -26057,10 +26299,10 @@
         <v>61</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>985</v>
+        <v>989</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>986</v>
+        <v>990</v>
       </c>
       <c r="I37" s="2" t="s">
         <v>148</v>
@@ -26072,13 +26314,13 @@
         <v>361</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="M37" s="2" t="s">
-        <v>1025</v>
+        <v>1029</v>
       </c>
       <c r="N37" s="2" t="s">
-        <v>1026</v>
+        <v>1030</v>
       </c>
       <c r="O37" s="4">
         <v>1600</v>
@@ -26111,7 +26353,7 @@
         <v>50</v>
       </c>
       <c r="Y37" s="2" t="s">
-        <v>1027</v>
+        <v>1031</v>
       </c>
       <c r="Z37" s="2" t="s">
         <v>52</v>
@@ -26149,13 +26391,13 @@
     </row>
     <row r="38" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D38" s="7">
         <v>46072</v>
@@ -26167,10 +26409,10 @@
         <v>39</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>1029</v>
+        <v>1033</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>1030</v>
+        <v>1034</v>
       </c>
       <c r="I38" s="6" t="s">
         <v>42</v>
@@ -26182,13 +26424,13 @@
         <v>382</v>
       </c>
       <c r="L38" s="6" t="s">
-        <v>1008</v>
+        <v>1012</v>
       </c>
       <c r="M38" s="6" t="s">
-        <v>1009</v>
+        <v>1013</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>931</v>
+        <v>935</v>
       </c>
       <c r="O38" s="8">
         <v>500</v>
@@ -26221,7 +26463,7 @@
         <v>50</v>
       </c>
       <c r="Y38" s="6" t="s">
-        <v>1031</v>
+        <v>1035</v>
       </c>
       <c r="Z38" s="6" t="s">
         <v>52</v>
@@ -26259,13 +26501,13 @@
     </row>
     <row r="39" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>1032</v>
+        <v>1036</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>1032</v>
+        <v>1036</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D39" s="3">
         <v>46076</v>
@@ -26277,10 +26519,10 @@
         <v>61</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>985</v>
+        <v>989</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>986</v>
+        <v>990</v>
       </c>
       <c r="I39" s="2" t="s">
         <v>148</v>
@@ -26292,13 +26534,13 @@
         <v>361</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>1025</v>
+        <v>1029</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>1026</v>
+        <v>1030</v>
       </c>
       <c r="O39" s="4">
         <v>1700</v>
@@ -26331,7 +26573,7 @@
         <v>50</v>
       </c>
       <c r="Y39" s="2" t="s">
-        <v>1033</v>
+        <v>1037</v>
       </c>
       <c r="Z39" s="2" t="s">
         <v>52</v>
@@ -26369,13 +26611,13 @@
     </row>
     <row r="40" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
-        <v>1034</v>
+        <v>1038</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>1034</v>
+        <v>1038</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D40" s="7">
         <v>46077</v>
@@ -26399,16 +26641,16 @@
         <v>149</v>
       </c>
       <c r="K40" s="6" t="s">
-        <v>971</v>
+        <v>975</v>
       </c>
       <c r="L40" s="6" t="s">
-        <v>972</v>
+        <v>976</v>
       </c>
       <c r="M40" s="6" t="s">
-        <v>973</v>
+        <v>977</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>974</v>
+        <v>978</v>
       </c>
       <c r="O40" s="8">
         <v>500</v>
@@ -26441,7 +26683,7 @@
         <v>50</v>
       </c>
       <c r="Y40" s="6" t="s">
-        <v>1035</v>
+        <v>1039</v>
       </c>
       <c r="Z40" s="6" t="s">
         <v>52</v>
@@ -26479,13 +26721,13 @@
     </row>
     <row r="41" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>1034</v>
+        <v>1038</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>1034</v>
+        <v>1038</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D41" s="3">
         <v>46077</v>
@@ -26509,16 +26751,16 @@
         <v>149</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>934</v>
+        <v>938</v>
       </c>
       <c r="L41" s="2" t="s">
-        <v>1036</v>
+        <v>1040</v>
       </c>
       <c r="M41" s="2" t="s">
-        <v>1037</v>
+        <v>1041</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>937</v>
+        <v>941</v>
       </c>
       <c r="O41" s="4">
         <v>500</v>
@@ -26551,7 +26793,7 @@
         <v>50</v>
       </c>
       <c r="Y41" s="2" t="s">
-        <v>1035</v>
+        <v>1039</v>
       </c>
       <c r="Z41" s="2" t="s">
         <v>52</v>
@@ -26566,10 +26808,10 @@
         <v>111</v>
       </c>
       <c r="AD41" s="2" t="s">
-        <v>941</v>
+        <v>945</v>
       </c>
       <c r="AE41" s="2" t="s">
-        <v>942</v>
+        <v>946</v>
       </c>
       <c r="AF41" s="2" t="s">
         <v>77</v>
@@ -26589,13 +26831,13 @@
     </row>
     <row r="42" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
-        <v>1038</v>
+        <v>1042</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>1038</v>
+        <v>1042</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D42" s="7">
         <v>46078</v>
@@ -26607,10 +26849,10 @@
         <v>39</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>914</v>
+        <v>918</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>915</v>
+        <v>919</v>
       </c>
       <c r="I42" s="6" t="s">
         <v>174</v>
@@ -26619,16 +26861,16 @@
         <v>175</v>
       </c>
       <c r="K42" s="6" t="s">
-        <v>916</v>
+        <v>920</v>
       </c>
       <c r="L42" s="6" t="s">
-        <v>917</v>
+        <v>921</v>
       </c>
       <c r="M42" s="6" t="s">
-        <v>918</v>
+        <v>922</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>919</v>
+        <v>923</v>
       </c>
       <c r="O42" s="8">
         <v>225</v>
@@ -26661,7 +26903,7 @@
         <v>50</v>
       </c>
       <c r="Y42" s="6" t="s">
-        <v>1039</v>
+        <v>1043</v>
       </c>
       <c r="Z42" s="6" t="s">
         <v>52</v>
@@ -26699,13 +26941,13 @@
     </row>
     <row r="43" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>1040</v>
+        <v>1044</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>1040</v>
+        <v>1044</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D43" s="3">
         <v>46079</v>
@@ -26717,10 +26959,10 @@
         <v>39</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>950</v>
+        <v>954</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>951</v>
+        <v>955</v>
       </c>
       <c r="I43" s="2" t="s">
         <v>137</v>
@@ -26732,13 +26974,13 @@
         <v>361</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="M43" s="2" t="s">
-        <v>1025</v>
+        <v>1029</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>1026</v>
+        <v>1030</v>
       </c>
       <c r="O43" s="4">
         <v>5000</v>
@@ -26762,16 +27004,16 @@
         <v>2354</v>
       </c>
       <c r="V43" s="2" t="s">
-        <v>955</v>
+        <v>959</v>
       </c>
       <c r="W43" s="2" t="s">
-        <v>956</v>
+        <v>960</v>
       </c>
       <c r="X43" s="2" t="s">
         <v>50</v>
       </c>
       <c r="Y43" s="2" t="s">
-        <v>1041</v>
+        <v>1045</v>
       </c>
       <c r="Z43" s="2" t="s">
         <v>52</v>
@@ -26809,13 +27051,13 @@
     </row>
     <row r="44" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
-        <v>1042</v>
+        <v>1046</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>1042</v>
+        <v>1046</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D44" s="7">
         <v>46079</v>
@@ -26842,13 +27084,13 @@
         <v>852</v>
       </c>
       <c r="L44" s="6" t="s">
-        <v>1043</v>
+        <v>1047</v>
       </c>
       <c r="M44" s="6" t="s">
-        <v>1044</v>
+        <v>1048</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>1045</v>
+        <v>1049</v>
       </c>
       <c r="O44" s="8">
         <v>12000</v>
@@ -26881,7 +27123,7 @@
         <v>50</v>
       </c>
       <c r="Y44" s="6" t="s">
-        <v>1046</v>
+        <v>1050</v>
       </c>
       <c r="Z44" s="6" t="s">
         <v>52</v>
@@ -26919,13 +27161,13 @@
     </row>
     <row r="45" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>1047</v>
+        <v>1051</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>1047</v>
+        <v>1051</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D45" s="3">
         <v>46085</v>
@@ -26949,16 +27191,16 @@
         <v>149</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>1048</v>
+        <v>1052</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>1049</v>
+        <v>1053</v>
       </c>
       <c r="M45" s="2" t="s">
-        <v>1050</v>
+        <v>1054</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>1051</v>
+        <v>1055</v>
       </c>
       <c r="O45" s="4">
         <v>5005</v>
@@ -26991,7 +27233,7 @@
         <v>50</v>
       </c>
       <c r="Y45" s="2" t="s">
-        <v>1052</v>
+        <v>1056</v>
       </c>
       <c r="Z45" s="2" t="s">
         <v>52</v>
@@ -27029,13 +27271,13 @@
     </row>
     <row r="46" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
-        <v>1053</v>
+        <v>1057</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>1053</v>
+        <v>1057</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D46" s="7">
         <v>46085</v>
@@ -27059,16 +27301,16 @@
         <v>149</v>
       </c>
       <c r="K46" s="6" t="s">
-        <v>971</v>
+        <v>975</v>
       </c>
       <c r="L46" s="6" t="s">
-        <v>1054</v>
+        <v>1058</v>
       </c>
       <c r="M46" s="6" t="s">
-        <v>1055</v>
+        <v>1059</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>974</v>
+        <v>978</v>
       </c>
       <c r="O46" s="8">
         <v>500</v>
@@ -27101,7 +27343,7 @@
         <v>50</v>
       </c>
       <c r="Y46" s="6" t="s">
-        <v>1056</v>
+        <v>1060</v>
       </c>
       <c r="Z46" s="6" t="s">
         <v>52</v>
@@ -27139,13 +27381,13 @@
     </row>
     <row r="47" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>1053</v>
+        <v>1057</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>1053</v>
+        <v>1057</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D47" s="3">
         <v>46085</v>
@@ -27169,16 +27411,16 @@
         <v>149</v>
       </c>
       <c r="K47" s="2" t="s">
-        <v>934</v>
+        <v>938</v>
       </c>
       <c r="L47" s="2" t="s">
-        <v>1036</v>
+        <v>1040</v>
       </c>
       <c r="M47" s="2" t="s">
-        <v>1037</v>
+        <v>1041</v>
       </c>
       <c r="N47" s="2" t="s">
-        <v>937</v>
+        <v>941</v>
       </c>
       <c r="O47" s="4">
         <v>500</v>
@@ -27211,7 +27453,7 @@
         <v>50</v>
       </c>
       <c r="Y47" s="2" t="s">
-        <v>1056</v>
+        <v>1060</v>
       </c>
       <c r="Z47" s="2" t="s">
         <v>52</v>
@@ -27226,10 +27468,10 @@
         <v>111</v>
       </c>
       <c r="AD47" s="2" t="s">
-        <v>941</v>
+        <v>945</v>
       </c>
       <c r="AE47" s="2" t="s">
-        <v>942</v>
+        <v>946</v>
       </c>
       <c r="AF47" s="2" t="s">
         <v>77</v>
@@ -27249,13 +27491,13 @@
     </row>
     <row r="48" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
-        <v>1057</v>
+        <v>1061</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>1057</v>
+        <v>1061</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D48" s="7">
         <v>46085</v>
@@ -27267,10 +27509,10 @@
         <v>39</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>1058</v>
+        <v>1062</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>1059</v>
+        <v>1063</v>
       </c>
       <c r="I48" s="6" t="s">
         <v>148</v>
@@ -27282,13 +27524,13 @@
         <v>139</v>
       </c>
       <c r="L48" s="6" t="s">
-        <v>1060</v>
+        <v>1064</v>
       </c>
       <c r="M48" s="6" t="s">
-        <v>1061</v>
+        <v>1065</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>1062</v>
+        <v>1066</v>
       </c>
       <c r="O48" s="8">
         <v>3700</v>
@@ -27321,7 +27563,7 @@
         <v>50</v>
       </c>
       <c r="Y48" s="6" t="s">
-        <v>1063</v>
+        <v>1067</v>
       </c>
       <c r="Z48" s="6" t="s">
         <v>52</v>
@@ -27359,13 +27601,13 @@
     </row>
     <row r="49" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>1064</v>
+        <v>1068</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>1064</v>
+        <v>1068</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D49" s="3">
         <v>46085</v>
@@ -27377,10 +27619,10 @@
         <v>39</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>872</v>
+        <v>876</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>873</v>
+        <v>877</v>
       </c>
       <c r="I49" s="2" t="s">
         <v>174</v>
@@ -27389,7 +27631,7 @@
         <v>175</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>1000</v>
+        <v>1004</v>
       </c>
       <c r="L49" s="2" t="s">
         <v>52</v>
@@ -27431,7 +27673,7 @@
         <v>52</v>
       </c>
       <c r="Y49" s="2" t="s">
-        <v>1065</v>
+        <v>1069</v>
       </c>
       <c r="Z49" s="2" t="s">
         <v>52</v>
@@ -27446,10 +27688,10 @@
         <v>280</v>
       </c>
       <c r="AD49" s="2" t="s">
-        <v>1003</v>
+        <v>1007</v>
       </c>
       <c r="AE49" s="2" t="s">
-        <v>1004</v>
+        <v>1008</v>
       </c>
       <c r="AF49" s="2" t="s">
         <v>52</v>
@@ -27469,13 +27711,13 @@
     </row>
     <row r="50" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
-        <v>1066</v>
+        <v>1070</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>1066</v>
+        <v>1070</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D50" s="7">
         <v>46091</v>
@@ -27487,10 +27729,10 @@
         <v>39</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>950</v>
+        <v>954</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>951</v>
+        <v>955</v>
       </c>
       <c r="I50" s="6" t="s">
         <v>137</v>
@@ -27502,13 +27744,13 @@
         <v>361</v>
       </c>
       <c r="L50" s="6" t="s">
-        <v>1067</v>
+        <v>1071</v>
       </c>
       <c r="M50" s="6" t="s">
-        <v>1068</v>
+        <v>1072</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>1026</v>
+        <v>1030</v>
       </c>
       <c r="O50" s="8">
         <v>5000</v>
@@ -27532,16 +27774,16 @@
         <v>2354</v>
       </c>
       <c r="V50" s="6" t="s">
-        <v>955</v>
+        <v>959</v>
       </c>
       <c r="W50" s="6" t="s">
-        <v>956</v>
+        <v>960</v>
       </c>
       <c r="X50" s="6" t="s">
         <v>50</v>
       </c>
       <c r="Y50" s="6" t="s">
-        <v>1069</v>
+        <v>1073</v>
       </c>
       <c r="Z50" s="6" t="s">
         <v>52</v>
@@ -27579,13 +27821,13 @@
     </row>
     <row r="51" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>1070</v>
+        <v>1074</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>1070</v>
+        <v>1074</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D51" s="3">
         <v>46091</v>
@@ -27597,10 +27839,10 @@
         <v>39</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>914</v>
+        <v>918</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>915</v>
+        <v>919</v>
       </c>
       <c r="I51" s="2" t="s">
         <v>174</v>
@@ -27609,16 +27851,16 @@
         <v>175</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>916</v>
+        <v>920</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>917</v>
+        <v>921</v>
       </c>
       <c r="M51" s="2" t="s">
-        <v>918</v>
+        <v>922</v>
       </c>
       <c r="N51" s="2" t="s">
-        <v>919</v>
+        <v>923</v>
       </c>
       <c r="O51" s="4">
         <v>225</v>
@@ -27651,7 +27893,7 @@
         <v>50</v>
       </c>
       <c r="Y51" s="2" t="s">
-        <v>1071</v>
+        <v>1075</v>
       </c>
       <c r="Z51" s="2" t="s">
         <v>52</v>
@@ -27689,13 +27931,13 @@
     </row>
     <row r="52" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
-        <v>1072</v>
+        <v>1076</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>1072</v>
+        <v>1076</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D52" s="7">
         <v>46093</v>
@@ -27707,10 +27949,10 @@
         <v>61</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>882</v>
+        <v>886</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="I52" s="6" t="s">
         <v>148</v>
@@ -27719,16 +27961,16 @@
         <v>149</v>
       </c>
       <c r="K52" s="6" t="s">
-        <v>1048</v>
+        <v>1052</v>
       </c>
       <c r="L52" s="6" t="s">
-        <v>1049</v>
+        <v>1053</v>
       </c>
       <c r="M52" s="6" t="s">
-        <v>1050</v>
+        <v>1054</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>1051</v>
+        <v>1055</v>
       </c>
       <c r="O52" s="8">
         <v>507</v>
@@ -27761,7 +28003,7 @@
         <v>50</v>
       </c>
       <c r="Y52" s="6" t="s">
-        <v>1073</v>
+        <v>1077</v>
       </c>
       <c r="Z52" s="6" t="s">
         <v>52</v>
@@ -27799,13 +28041,13 @@
     </row>
     <row r="53" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>1074</v>
+        <v>1078</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>1074</v>
+        <v>1078</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="D53" s="3">
         <v>46097</v>
@@ -27823,22 +28065,22 @@
         <v>330</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>899</v>
+        <v>903</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>900</v>
+        <v>904</v>
       </c>
       <c r="K53" s="2" t="s">
         <v>382</v>
       </c>
       <c r="L53" s="2" t="s">
-        <v>1008</v>
+        <v>1012</v>
       </c>
       <c r="M53" s="2" t="s">
-        <v>1009</v>
+        <v>1013</v>
       </c>
       <c r="N53" s="2" t="s">
-        <v>931</v>
+        <v>935</v>
       </c>
       <c r="O53" s="4">
         <v>3000</v>
@@ -27871,7 +28113,7 @@
         <v>50</v>
       </c>
       <c r="Y53" s="2" t="s">
-        <v>1075</v>
+        <v>1079</v>
       </c>
       <c r="Z53" s="2" t="s">
         <v>52</v>
@@ -27907,8 +28149,226 @@
         <v>31170.42</v>
       </c>
     </row>
-    <row r="54" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="54" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="6" t="s">
+        <v>1080</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>1080</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>875</v>
+      </c>
+      <c r="D54" s="7">
+        <v>46098</v>
+      </c>
+      <c r="E54" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F54" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G54" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="H54" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="I54" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="J54" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="K54" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="L54" s="6" t="s">
+        <v>928</v>
+      </c>
+      <c r="M54" s="6" t="s">
+        <v>929</v>
+      </c>
+      <c r="N54" s="6" t="s">
+        <v>930</v>
+      </c>
+      <c r="O54" s="8">
+        <v>10000</v>
+      </c>
+      <c r="P54" s="8">
+        <v>12.27</v>
+      </c>
+      <c r="Q54" s="9">
+        <v>122700</v>
+      </c>
+      <c r="R54" s="9">
+        <v>3987.75</v>
+      </c>
+      <c r="S54" s="9">
+        <v>126687.75</v>
+      </c>
+      <c r="T54" s="9">
+        <v>122700</v>
+      </c>
+      <c r="U54" s="9">
+        <v>14724</v>
+      </c>
+      <c r="V54" s="6" t="s">
+        <v>942</v>
+      </c>
+      <c r="W54" s="6" t="s">
+        <v>943</v>
+      </c>
+      <c r="X54" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="Y54" s="6" t="s">
+        <v>1081</v>
+      </c>
+      <c r="Z54" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA54" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB54" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC54" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="AD54" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="AE54" s="6" t="s">
+        <v>503</v>
+      </c>
+      <c r="AF54" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="AG54" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH54" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="AI54" s="9">
+        <v>12</v>
+      </c>
+      <c r="AJ54" s="8">
+        <v>75850.3</v>
+      </c>
+    </row>
+    <row r="55" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="2" t="s">
+        <v>1082</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>1082</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>875</v>
+      </c>
+      <c r="D55" s="3">
+        <v>46098</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>886</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>887</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="J55" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="K55" s="2" t="s">
+        <v>888</v>
+      </c>
+      <c r="L55" s="2" t="s">
+        <v>889</v>
+      </c>
+      <c r="M55" s="2" t="s">
+        <v>890</v>
+      </c>
+      <c r="N55" s="2" t="s">
+        <v>891</v>
+      </c>
+      <c r="O55" s="4">
+        <v>507</v>
+      </c>
+      <c r="P55" s="4">
+        <v>21.96</v>
+      </c>
+      <c r="Q55" s="5">
+        <v>11133.72</v>
+      </c>
+      <c r="R55" s="5">
+        <v>361.85</v>
+      </c>
+      <c r="S55" s="5">
+        <v>11495.57</v>
+      </c>
+      <c r="T55" s="5">
+        <v>11133.72</v>
+      </c>
+      <c r="U55" s="5">
+        <v>445.35</v>
+      </c>
+      <c r="V55" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="W55" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="X55" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="Y55" s="2" t="s">
+        <v>1083</v>
+      </c>
+      <c r="Z55" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA55" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB55" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC55" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="AD55" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="AE55" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="AF55" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AG55" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH55" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="AI55" s="5">
+        <v>4</v>
+      </c>
+      <c r="AJ55" s="4">
+        <v>5539.1575199999997</v>
+      </c>
+    </row>
     <row r="56" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="57" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="58" spans="1:36" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>